<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 1)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -660,8 +660,336 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1180595613</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PDRN 100ヒアルロン酸 ブースター トナー 250ml + PDRNヒアルロン酸100モイスチャライジングクリーム 60ml + PDRN ヒアルロン酸カプセル 100セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>11931</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180595613</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1174748969</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[NEW] [新商品] ドクダミポアディープクレンジングフォーム 150ml (2個)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>4431</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174748969</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1171434085</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸100モイスチャライジングクリーム 60ml (2個) + PDRN ヒアルロン酸カプセル 100セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>12801</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171434085</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1151371296</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>アトバリア365 ハイドロエッセンス 200ml (2個)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>8763</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151371296</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1127146298</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5番 マスクパック (10枚) / 白玉グルタチオンＣふりかけマスク</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>4695</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1127146298</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1154643575</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>UVシールド トーンアップサン SPF50+ PA++++ 50ml(+贈呈25ml), 1個 / 韓国 人気 シミ しみ たるみ エイジングケア トーンアップ 日焼け止め クリーム</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>5744</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154643575</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1205457208</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>大豆エッセンス 50ml(+ツボクサエッセンス 20ml), 1個 / 韓国 人気 保湿 鎮静 ニキビ 角質 皮脂 美容液 無香料 ビーンエッセンス</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ミクスン</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>5834</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205457208</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1204840989</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[1+1]3番 すべすべキメケアセラム EX 60ml(30ml+30ml) / 韓国 人気 角質 皮脂 ツヤ 毛穴ケア 導入美容液 ブースター</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>5203</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204840989</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 2)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -988,8 +988,172 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1164314943</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>chinju</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2本セット　マックセルスキンサイエンス365 シンエイク ゴールド アイセラム 15ml×2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ドクターファモール</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164314943</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1212169783</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>The Alpha Arbutin Discoloration Care Hydrogel Mask 3ea (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2884</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212169783</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1210422401</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ニュートロジーナ レインバス ボディウォッシュ 473ml 3個（ウッディスパイスの香り＋ベルガモットムスクの香り＋フリージアグリーンアップルの香り） (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ニュートロジーナ</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>5985</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210422401</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1210363980</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1+1キャンペーン／薬局入店 PDRN ピーディーアールエヌ リジュディンクリーム／ダメージ肌バリアのと鎮静 (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>リール</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1876</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210363980</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J13"/>
+  <autoFilter ref="A1:J17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 3)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1152,8 +1152,213 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1208337865</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>dire</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>グロウトックス ライスセラム 30ml / 米エキス・スクワラン配合 / キメを整える集中ケア美容液</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DI / RE</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>6300</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208337865</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1194316158</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>mijin-cosme</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>メール便 無料 - アクロパス ニードルパッチ 目元 ほうれい線 レチアールエヌ スリム パッチ 3box - PDRN × レチノール配合 - 部分集中ケア - 正規品</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ACROPASS</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>8700</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194316158</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1173424338</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>mijin-cosme</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>国内発送 - メール便 - H セラム スティック ハニーゴールド (マルチバーム) 10g 【1個】 - マルチバーム（保湿） - 韓国コスメ - 3営業日以内(土日祝除く)に発送 - 正規品</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>チョソンア</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173424338</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1194316148</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>mijin-cosme</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>メディヒール パック 詰め替え用 MEDIHEAL PDRN フェイスマスク 【 リフィル 】 30枚 - 毛穴 弾力ケア シートマスク - 韓国コスメ - シートマスクパック - 正規品</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194316148</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1194316155</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>mijin-cosme</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>メディヒール パック 詰め替え用 MEDIHEAL コラーゲン フェイスマスク 【 リフィル 】 30枚 - 弾力ケア シートマスク - 韓国コスメ - シートマスクパック - 正規品</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194316155</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J17"/>
+  <autoFilter ref="A1:J22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 4)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1357,8 +1357,131 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1209977461</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>mijincosme</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>夏美祭 MJケア シートマスク 【60枚】 SALE 選べるセット(6種X各10枚) 組合せ自由 - プラス1枚付き - 保湿 セット 個包装 韓国パック 大容量 シートパック フェイスパック</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MIJIN COSMETICS</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209977461</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1190054453</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>THEMAROSHOP</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュリペアスージングクリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>3399</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190054453</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1192506745</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>THEMAROSHOP</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ベーキングパウダー コラーゲン 毛穴スクラブ 25包入り</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ファームステイ</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192506745</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J22"/>
+  <autoFilter ref="A1:J25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 5)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1480,8 +1480,254 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1141816327</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>JDKM</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>わさびスージングマスク 30g</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Miss Dragon</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>5709</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141816327</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1141816688</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>JDKM</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>トーンアップ ホワイト マッド マスク 3個入り x 2個</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>バイアウア</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>5214</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141816688</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1025039849</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>JDKM</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>VT スーパーヒアロンフォームクレンザー 300ml</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2739</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1025039849</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1084303236</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DANAWA</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>C2Y ディープモイスチャー フットクリーム1個 60mlx3個【正規品】 韓国ブランド</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1084303236</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1205506863</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>【全商品よりどり】 ボンディングケラチンフォームトリートメント200ml / ボンディングアルファケラチンヘアパック 260g / Nude Musk / Green Zest / ダメージケア</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>4350</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205506863</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1204360681</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>【公式】 ボンディングアルファケラチンヘアパック 260g / Nude Musk / ジェラートヘアパック / マーブルセラピー / ダメージケア / サロンクリニック / 髪の絡まりを改善</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204360681</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J25"/>
+  <autoFilter ref="A1:J31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 3, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1726,8 +1726,418 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1161204302</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>kinakomall</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>[正規品]ドリクロ 20ml/脇汗デオドラント/デオドラント/脇汗/制汗剤/脇汗 韓国</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Driclor</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1718</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161204302</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1178361427</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>furimakei</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ZARA MAN 香水 TOBACCO COLLECTION RICH WARM ADDICTIVE 100ML オードトワレ</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ザラ</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>7263</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178361427</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1178361387</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>furimakei</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ディスカバリーセット（5MLX2） アナザー13 + サンタル33</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LE LABO</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>9588</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178361387</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1175756083</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>20240208</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>セレブ愛用 オートイン カーミング クリーム 100ml しっとり鎮静ジェル 保湿 敏感肌 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Purito</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>2384</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175756083</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1172113145</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>20240208</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ヘリ愛用！ 緑豆 クレンジングオイル 選べる200ml/50ml 黒ずみオフ オリヤン 即日発送</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>2809</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172113145</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1130162927</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>360度ショットPDRNアクティブセラム 50ml +マデカクリーム シーズン7 タイムリバース 50ml</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>4491</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130162927</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1194311832</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>レッド イレイジングクリーム 2.0 (リニューアル) 50ml</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194311832</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1190200956</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>クリムゾン スカイ(ポリッシュ) 8ml #シャンパンスパークル #イブニングパーティー</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FINGER SUIT</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>3280</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190200956</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1188287748</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>[大容量]ダーマソルトクリーム120ml</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ABpharm</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>10990</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="b">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188287748</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1176547134</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ポメロ(ポリッシュ) 8ml #シナモンラテ #ピーチオレンジグリッター</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>FINGER SUIT</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176547134</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J31"/>
+  <autoFilter ref="A1:J41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 6, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2136,8 +2136,746 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1183378989</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>yujin20</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>バイオアクティブコンプリート Bコンプレックス ベジカプセル60粒</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Life Extension</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183378989</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1194501160</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>yujin20</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>, Hydro Cera-Nol Real Deep Beauty Mask, 4 Sheets, 1.19 oz (34 g) Each</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ハイドロ</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>4989</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194501160</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1188026399</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>YujinTwo</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Advanced Clinicals Retinol Anti-Wrinkle Serum 52ml（1.75液量オンス）</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ADVANCED CLINICALS</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>2759</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188026399</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1191354937</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>kptown</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>【60枚】24Kゴールド レチノール アイパッチ 目元ケア エイジングケア しわ ハリ 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Terez &amp;amp; Honor</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191354937</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1191354082</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>kptown</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>【60枚】ビタミンC ナイアシンアミド アイパッチ 目元パック 目の下パック トラネキサム酸 ヒアルロン酸 うるおい 保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Terez &amp;amp; Honor</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>2480</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191354082</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1189557181</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>kptown</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>メラノンX クリーム 30ml×3個セット / 透明感 / くすみケア / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>3950</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189557181</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1125754461</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>[1+1]レッドブレミッシュクリアスージングクリーム 50ml 2個+10ml 2個/正規品</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>3469</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125754461</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1212553298</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>【正規品+GIFT付き】リードルショット コラーゲンクリーム 50ml＋スティックパウチ 3個</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>3021</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="b">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212553298</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1212350487</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>[1+1]MEDI AHAイボ取りクリーム25ml 2個&amp;nbsp; / メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>3666</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="b">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350487</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1212350471</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>[1+1]メディオルガブライトニングクリーム30ml 2個/しみ取りクリーム お肌のトーンアップ</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>3055</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="b">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350471</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1212350473</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MEDI AHAイボ取りクリーム25ml/ メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="b">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350473</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1206008325</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ペプチドショット2X 弾力アンプル 30ml（ハリ感ケア／保湿／弾力サポート美容液）</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>2122</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="b">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008325</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1206008294</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ウォーターフィット リカバー BBクリーム 30ml #SPF40 PA+++ #保湿密着</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>2927</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008294</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1205912921</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>レチンアルブースターショット 30ml+30ml #レチナール2.0% #セラミド #エクトイン #カフェイン #ペプチド</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>4046</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205912921</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1171497230</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>K_JIKGU</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ノスカナイントラブルセラム, 30ml</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>パティオン</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>2954</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171497230</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1171497900</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>K_JIKGU</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ホワイトトリュフファーストアロマティックスプレーセラム, 60ml</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>2581</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171497900</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1171498084</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>K_JIKGU</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>レッドアクネボディソープ, 400g</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171498084</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1162429093</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>yoo_k1120</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>コダリビノパーフェクトラジアンズセラム30mlホワイト ニングホワイト ニングアンプル（フランスセラム）</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>コーダリー</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>7340</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162429093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J41"/>
+  <autoFilter ref="A1:J59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 9, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2874,8 +2874,418 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1191781202</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>MEDIHEAL トナーパッド2.0 リフィル 70枚×2個セット 4タイプ選択可</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1918</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191781202</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1204359324</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>【1+1 / SNS話題】ツヤ肌バブルエッセンストナー 95ml</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>curest</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>2131</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204359324</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1171040599</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ジェントル リフレッシング ボディウォッシュ 1L / 大容量 / 敏感肌用 / 低刺激</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>セタフィル</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171040599</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1163545805</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>frombeauty</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>水分バリアPANGヒアルロン酸パンテノールアンプル 100ml</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>EDIT.B</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1995</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163545805</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1132572987</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>frombeauty</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>サロン10アンプルヘアミスト 200ml</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132572987</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1202451334</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>njhmall</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ルフリージア オードパルファム 10ml</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SISAO</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>4941</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202451334</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1198592013</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>PDRN ピンクペプチドアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>3220</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="b">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198592013</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1208272698</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>レッドイレイジングクリーム 2.0 50ml</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208272698</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1208271013</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>コラーゲンジェリークリーム 110ml</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>3930</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208271013</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1172312020</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>hokkorikorea</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>【SALE】【毛穴ケア】PDRN毛穴弾力パッド 100枚 ハリ感 キメ整う エイジングケア ツヤ肌 角質ケア うるおい 人気 韓国コスメ 大容量 毎日ケア 時短 敏感肌OK 透明感 キメケア 保湿</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>3006</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172312020</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J59"/>
+  <autoFilter ref="A1:J69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 12, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3284,8 +3284,705 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1202055978</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>UVクリーム SPF50+ PA ++++ 敏感肌向けトーンアップ韓国コスメの人気日焼け止め</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202055978</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1174315936</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>1. マデカラボ マスク 10枚×2箱（リンクル リバイタライズ）</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174315936</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1178756887</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>nekohime</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>パワーネイル マグネット</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>FINGER SUIT</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>3793</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178756887</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1161381618</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>nekohime</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>サンマデカクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1654</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161381618</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1204176921</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>nekohime</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>[medicube] ブラックヘッド毛穴ブラシ</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1690</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204176921</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1060687901</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Uriage ユリアージュ バリアダム シカクリーム 40ml [製造国 フランス]</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Uriage</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>3156</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1060687901</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1059767256</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ROUND LAB ラウンドラップ 1025 独島 クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1680</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1059767256</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1207556247</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>CooAnCoo</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>シカカーミングサンセラム 50ml SPF50+ PA++++ / 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TOCOBO</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>3270</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207556247</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1207227328</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>CooAnCoo</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>アクアグロウリングサンスクリーン 45ml グリーンティーフレッシュサンスクリーン 45ml</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>2540</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207227328</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1203705320</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>CooAnCoo</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ビタCテカブレミッシュショット ゲルマスクパック（5枚入）（シカ＆リードル）/ シミ取りショットマスク/パックマスク/パック/フェイスパック</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>CKD_GUARANTEED</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1730</v>
+      </c>
+      <c r="G79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203705320</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1102761265</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>CooAnCoo</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>スキンプロテクションエリシアエッセンス 50ml / 肌バリア保護 / 韓国エステ専用</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Beautederm</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>7610</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102761265</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1138225289</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>dreamus</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>シグネチャーパルファム, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>5517</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138225289</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1206859281</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ポアブライトニングシミケアクリームマスク, 4枚 /ブライトニング/韓国マスクパック/ナイアシンアミド/保湿/水分/肌トーン改善/顔の頬リフ</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206859281</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1203000979</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>大豆エッセンス, 50ml</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ミクスン</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G83" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203000979</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1198208356</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>hikoreashop</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>アヌカチンシャンプー, 300ml</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>moev</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1775</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198208356</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1180574367</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>fromAnswer</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>[10Sマイクロバブルパック 4種] エア** バブルCDS マスク パック 80ml, 4種の中から選択 (ハリ/ブライトニング/鎮静/水分) 150 回分</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Gear By Gash</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>4014</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180574367</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1207330609</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>joohoh2</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>[メンズ オールインワン 限定企画3種セット] アクアパワー オールインワン 200ml セット ＋クレンザー40ml／オールインワン20ml 付き</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>ビオテルム</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>5292</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207330609</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J69"/>
+  <autoFilter ref="A1:J86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 15, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3981,8 +3981,910 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1118867909</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%エクスポリエイティングトナー 100ml韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>2346</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1118867909</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1188512361</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ノニアクネバブルクレンザー, 155ml /韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188512361</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1130886239</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>バイオガ ビオチン ダメージヘア改善 脱毛緩和シャンプー 1000ml /韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>BIORGA</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130886239</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1097276457</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>リアルカレンデュラピールオフパック, 100g 韓国スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>3109</v>
+      </c>
+      <c r="G90" t="n">
+        <v>1</v>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097276457</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1203335944</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>ボディローション ホワイトマスク520ml /韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ブーケガルニ</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203335944</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1196699361</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>蓮花PDRNヒアルロン光彩セラム 30ml 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>ハンスキン</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196699361</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1193167209</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>パンテノール クリーム 100ml 韓国スキンケア 韓国 コスメ #水分#保湿 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>4504</v>
+      </c>
+      <c r="G93" t="n">
+        <v>1</v>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193167209</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1168692108</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>【正規品】松の木 鎮静 シカ クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168692108</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1164469069</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>【正規品】グリーンシカ コラーゲン クリアフォーム 2.0 300ml</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164469069</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1163729695</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>【正規品】ディープポア クレンジング ソーダフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163729695</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1206937740</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>【正規品】ティアミドール ブースターセラム 30ml</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>ユーセリン</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>6990</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206937740</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1205554253</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>【正規品】トラネキサム酸スキンブースタークリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>メディテラピー</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205554253</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1201652635</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>GD11</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>【公式】リペア アンプルマスクパック(6枚入×5箱)パック シカエクソソーム PDRN 乾燥 保湿 毛穴 鎮静 臍帯血 ヒト幹細胞 エイジング シートマスク韓国コスメ スキン</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>GD11</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>14900</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201652635</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1201612192</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>GD11</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>【公式】リペアプラスアンプルプログラム美容液 シカエクソソーム PDRN ハリ 毛穴 乾燥 エイジング 韓国コスメ スキンケア 化粧品</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>GD11</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>10580</v>
+      </c>
+      <c r="G100" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201612192</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1201611272</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>GD11</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>【公式】リペア アンプルプログラム美容液(２セット) シカエクソソーム PDRN ハリ 毛穴 乾燥 エイジング 韓国コスメ スキンケア 化粧品</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>GD11</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>4772</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201611272</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1210121103</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>ttonce-korea</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ プロ サンクリーム 50g 2個 ト ラベル スポーツ日焼け止め,DEWYTREE ACディープ熱感カーミングマスク 1枚プレゼント</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>6383</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210121103</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1202343508</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ttonce-korea</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>フットパウダー 35g 3種類から1つ選択（オリジナル・オレンジ・ペパーミント）トラベル【プレゼント】シューズクリーナー3枚 足臭対策 消臭パウダー</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>GRAN'S REMEDY</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>3979</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202343508</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1201467957</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>thecolor</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ウォーターバンクアクアフェイシャル, 30ml</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>ラネージュ</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G104" t="n">
+        <v>2</v>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201467957</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1195611490</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>thecolor</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>アンチポアブラックヘッドクリアキット, 10枚</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>CNP Laboratory</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195611490</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1182152524</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>thecolor</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>グリーンティーセラミドバリアクリーム, 15ml, 3個</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G106" t="n">
+        <v>2</v>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182152524</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1175996173</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>thecolor</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>グリーンティーシードヒアルロンセラム, 130ml</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>3362</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175996173</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>958808136</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>uf_shop</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>クリアスキン8%AHAエッセンス【100ml】</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>イズエンツリー</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>2489</v>
+      </c>
+      <c r="G108" t="n">
+        <v>2</v>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=958808136</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J86"/>
+  <autoFilter ref="A1:J108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 18, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4883,8 +4883,664 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1160562706</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>アトバリア365クリームミスト 120ml</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G109" t="n">
+        <v>3</v>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160562706</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1199565099</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>デリケートゾーン 黒ずみ クリーム ナイアシンアミド 公式 アンダーアームクリーム 100g</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>BnD</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199565099</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1210391803</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>【新商品】 3番 キメブースター時短バブルパック, 90ml</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210391803</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1209814389</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>メイクアップ セッティング フィックス ミスト 75ml（4種選択1）</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209814389</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1180354766</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>[1+1/限定企画] スキンフード キャロット カロチン カミング ウォーターパッド 60枚 ダブル企画</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>6791</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180354766</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1207273381</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>PDRN ピンク コラーゲン バーム セラム 95ml 炭酸 泡 美容液 水光肌 弾力 ほうれい線 乾燥肌 エイジングケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>5049</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207273381</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1211859799</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>ゼロキャスト デイリー 透明 保湿サンスクリーン 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>3211</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211859799</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1211855765</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ビタC フォーストリックス トーニング セラムマスク 22ml 10枚</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>3173</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211855765</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1209466651</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>ラクトリメディ レディース カミングクリーム 15ml</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>メディオン</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>5161</v>
+      </c>
+      <c r="G117" t="n">
+        <v>1</v>
+      </c>
+      <c r="H117" t="b">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209466651</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1209446667</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>【クーリング/Yーンケア】ポエリエ フェミニン インナーパフューム デイリー マルチ香水</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>フォエリー</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G118" t="n">
+        <v>1</v>
+      </c>
+      <c r="H118" t="b">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209446667</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1083146394</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>inmybag</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>カロテンIPMP ブレミッシュセラムパックパッド 80枚</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="b">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083146394</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1168718026</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>bongbongshop</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>トーン＆スポットアンプル+クリーム(80ml)セット /美容液/睡眠保湿クリーム/韓国/スキンケア/チェリー/2種セット/保湿/シミ/くすみ/鎮静/トーンアップ/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Redence</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>7799</v>
+      </c>
+      <c r="G120" t="n">
+        <v>1</v>
+      </c>
+      <c r="H120" t="b">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168718026</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1191474301</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>REJURAN 公式 リジュラン PDRN (c-PDRN) ポアタイトニングトナーパッド 60枚 トナーパッド パック</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191474301</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1193834173</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>dAlba 公式 ダルバ 下地 グリーン ウォータフル トーンアップサンクリーム 50ml 5種 ピンク パープル カバーベージュ 21号 23号 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193834173</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1193834160</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>BRINGGREEN 公式 ブリングリーン ティーツリーシカセンシティブクレンジングウォーター 500ml BRINGGREEN 洗顔 クレンジング</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G123" t="n">
+        <v>1</v>
+      </c>
+      <c r="H123" t="b">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193834160</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>1191474305</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Rejuran 公式 リジュラン リバランシング トナー 120ml+120ml PDRN ( c-PDRN ) 化粧水 口コミ</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="b">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191474305</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J108"/>
+  <autoFilter ref="A1:J124"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 21, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$143</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J124"/>
+  <dimension ref="A1:J143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5539,8 +5539,787 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>1209235398</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿クリーム 50ml 韓国コスメ 韓国ブランド 公式ショップ 韓国スキンケア スキンケア 化粧品 敏感肌 乾燥肌 水分ケア うるおい 韓国アンプル ギフト PDRN CICA</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>2664</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="b">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209235398</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1210318709</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿アンプル 30ml 2個セット 1+1 美容液 セラム 韓国コスメ 韓国スキンケア 化粧品 スキンケア PDRN パインショットエクソソーム CICA うるおい 水分 アンプル</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>3336</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="b">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210318709</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1209368965</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿パッククレンザー 150ml 洗顔 メイク落とし 乾燥肌 敏感肌 弱酸性 韓国スキンケア 韓国コスメ クレンジング 保湿 泡立ち 2WAY パック 韓国化粧品 韓国 韓国好き</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>2454</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="b">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209368965</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1153736555</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>stellacosme</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>[1+1] メルヘンラップ オリジナル 高周波クリーム 800ml, 2個</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>MARCHEN LAB</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>5530</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="b">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1153736555</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1213378280</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>ザ・ビタA レチナールショット タイトニングブースター 15ml/더 비타 A 레티날 샷 타이트닝 부스터 15ml</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>2386</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="b">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213378280</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1167189215</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>ドクダミヒアルロンスージング アンプル 50ml/ 어성초 히알루론 수딩 앰플 50ml</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>2212</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" t="b">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167189215</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1083286884</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>[ エンジェルスリキッド ] グルタチオンプラス ナイアシンアミド 700vクリーム 50ml/나이아신아마이드 700v 크림</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Angel's Liquid</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>3085</v>
+      </c>
+      <c r="G131" t="n">
+        <v>3</v>
+      </c>
+      <c r="H131" t="b">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083286884</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1210476388</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>innerbeauty</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>トーン&amp;amp;スポットコレクターアンプル, 30ml, 2個</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Redence</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G132" t="n">
+        <v>1</v>
+      </c>
+      <c r="H132" t="b">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210476388</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1202066299</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>innerbeauty</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%トーニングソリューション, 240ml</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G133" t="n">
+        <v>3</v>
+      </c>
+      <c r="H133" t="b">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202066299</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1210829738</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>beautyluv</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>プレミアムもちソープ[グリーン], 120g</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G134" t="n">
+        <v>1</v>
+      </c>
+      <c r="H134" t="b">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210829738</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1213607022</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>beautyluv</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>リアルマットメイクアップセッティングフィックスミスト, 75ml</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>2397</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0</v>
+      </c>
+      <c r="H135" t="b">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213607022</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>1211081043</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>beautyluv</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>PDRNアイパッチ</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>2469</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" t="b">
+        <v>0</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211081043</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>1165634740</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>truvio</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>ヘアシールド（ヘアフィクサー/スプレー噴射型）</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>ユリカ</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>3646</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" t="b">
+        <v>0</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165634740</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>1165169271</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>truvio</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>[ミニパフューム/シナモロール キーリング 贈呈] パフューム ミスト 94ml 10種</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>ボディファンタジー</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>2996</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" t="b">
+        <v>0</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165169271</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>1204664064</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>skinqoo</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>【ベビーサンケア】MONDIES ノンケミカル サンスティック / クーリングサンクッション / マイルドサンクリーム赤ちゃん用日焼け止め 敏感肌 UVケア 韓国ベビーコ</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>モンディエス</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" t="b">
+        <v>0</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204664064</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>1185439830</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>skinqoo</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>【角質つるん】バイオームバリア PHA グロウ リファイニングアンプル 30ml 1個 / 低刺激 / パハピンクアンプル</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>UIQ</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>4149</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="b">
+        <v>0</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185439830</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>1204465120</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>skinqoo</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>【正規品】DODOLABEL アイドルホワイトタンニングスプレー 50ml ミニサイズ 携帯用 トーンアップスプレー 韓国コスメ ボディメイク 首顔色補正 自然肌演出 保湿 密着 持ち運び便利 人気</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>DODO LABLE</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>2993</v>
+      </c>
+      <c r="G141" t="n">
+        <v>2</v>
+      </c>
+      <c r="H141" t="b">
+        <v>0</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204465120</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>1204664117</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>skinqoo</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>【1+1】【ベビーサンケア】ノンケミカル サンスティック / クーリングサンクッション / マイルドサンクリーム 赤ちゃん用日焼け止め 敏感肌 UVケア 韓国ベビー</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>モンディエス</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>5005</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" t="b">
+        <v>0</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204664117</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>1204466080</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>skinqoo</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>【正規品】 セラディクス トリプルレチノールアクネウォッシュピール30ml / レチノール導入美容液 毛穴ケア 角質ケア 敏感肌対応 キメ整肌 保湿ケア 韓国スキンケア 人気美容液</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>5220</v>
+      </c>
+      <c r="G143" t="n">
+        <v>3</v>
+      </c>
+      <c r="H143" t="b">
+        <v>0</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204466080</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J124"/>
+  <autoFilter ref="A1:J143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 24, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J143"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6318,8 +6318,828 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>1205747267</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>アクニDr.ファーストブラックディープクレンジングフォーム 75ml</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>アイソイ</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>2286</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" t="b">
+        <v>0</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205747267</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>1205744981</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>シカカーミングパウダーウォッシュ 50g</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>TOCOBO</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="b">
+        <v>0</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205744981</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>1210161140</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>3番キメブースター時短バブルパック 90ml</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>2496</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" t="b">
+        <v>0</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210161140</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>1213040499</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>alpamyeong</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>メンズ 脱毛症状ケア シャンプー 515ml ティーツリー ユーカリ 頭皮クールケア ボリュームアップ 韓国ヘアケア 男性用</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>呂</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>2992</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" t="b">
+        <v>0</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213040499</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>1094657609</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>chillingvibes</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>【2+1】スーパーフード 390ml / ボディーローション(Peach)</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>2745</v>
+      </c>
+      <c r="G148" t="n">
+        <v>1</v>
+      </c>
+      <c r="H148" t="b">
+        <v>0</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094657609</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>1094595212</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>chillingvibes</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>パンキニパフュームハンドクリームミニ 15ml / PUMKINI, CHAMO,FEY9,VEIN / 香水 ハンド</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>3197</v>
+      </c>
+      <c r="G149" t="n">
+        <v>1</v>
+      </c>
+      <c r="H149" t="b">
+        <v>0</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094595212</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>1094668408</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>ledebai0_jp</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>[デウン製薬] キミアンプル7ml / 韓国 美容液</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>イージーデュー</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>5550</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="b">
+        <v>0</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094668408</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>1096984158</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>K-Blush</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>【限定特典メディヒールマスク付】プレミアム2.0 ネックスティック 20g ペプチド1000ショット 首ケア ベタつかない保湿ボリュームアップハリ 弾力 リフティング 首のしわあごのしわ韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G151" t="n">
+        <v>2</v>
+      </c>
+      <c r="H151" t="b">
+        <v>0</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096984158</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>1089915438</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>K-Blush</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>【公式正品】【角質ケア】グリコール酸7％ エクスフォリエーティング トナー 100ml /240mlAHA配合 拭き取り化粧水なめらか肌・キメケア・夜用スキンケア脇の黒ずみケア毛穴のざらつきケア韓国</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>2699</v>
+      </c>
+      <c r="G152" t="n">
+        <v>2</v>
+      </c>
+      <c r="H152" t="b">
+        <v>0</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089915438</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>1212749218</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>K-Blush</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】乳酸(Lactic Acid)10%+ヒアルロン酸HA 30ml 美容液 角質ケア 保湿 キメ なめらか肌 フェイスセラム スキンケア 韓国美容液 人気</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="b">
+        <v>0</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212749218</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>1186300374</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>kokowakorea</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>オードパルファム50ml（3種類）</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>I GENTLEMAN</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>5270</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="b">
+        <v>0</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186300374</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>1192209159</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>kokowakorea</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>シルエットヘアパルファム68ml企画2種タック1</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>tooq</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>5350</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="b">
+        <v>0</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192209159</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>1182791384</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>kokowakorea</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>マリンオーキッドマルチパフューム</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>GRANHAND</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>5970</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="b">
+        <v>0</v>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182791384</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>1177840431</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>kokowakorea</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>ポリゲンシークニングセラム50ml+スケーラー60g</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>4590</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="b">
+        <v>0</v>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177840431</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>1158938315</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>kokowakorea</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>ボディローションバニラムスク520ML 1+1</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>ブーケガルニ</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>3670</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="b">
+        <v>0</v>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158938315</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>1194074735</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>octaglobal</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸カプセル100 セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="b">
+        <v>0</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194074735</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>1134795243</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>BeautyPalette</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>テラクネ365 クリアディープクレンジングフォーム, 200ml</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>3398</v>
+      </c>
+      <c r="G160" t="n">
+        <v>1</v>
+      </c>
+      <c r="H160" t="b">
+        <v>0</v>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134795243</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>1210242426</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>BeautyPalette</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸カプセル100 セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>3311</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="b">
+        <v>0</v>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210242426</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>1210085885</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>BeautyPalette</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>プロバイオダーム3Dリフティングアイ＆リンクルクリーム, 25ml, 2個</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>5355</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="b">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210085885</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>1210078217</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>BeautyPalette</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>PDRNコラーゲンフェイシャルショットトナー, 300ml</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>molvany</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>6155</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="b">
+        <v>0</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210078217</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J143"/>
+  <autoFilter ref="A1:J163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 27, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$172</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7138,8 +7138,377 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>1199006543</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>playstar</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>バランスフルシカコントロールセラム, 50ml</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="b">
+        <v>0</v>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199006543</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>1176085366</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>playstar</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>アクアスージングトナー, 200ml</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>CNP Laboratory</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>2050</v>
+      </c>
+      <c r="G165" t="n">
+        <v>1</v>
+      </c>
+      <c r="H165" t="b">
+        <v>0</v>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176085366</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>1193601980</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 100ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G166" t="n">
+        <v>2</v>
+      </c>
+      <c r="H166" t="b">
+        <v>0</v>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193601980</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>1206909143</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 240ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="b">
+        <v>0</v>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206909143</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>1202095634</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 240ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>4020</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="b">
+        <v>0</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202095634</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>1209089569</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml1個 韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="b">
+        <v>0</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089569</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>1209089497</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml 2個 set/韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="b">
+        <v>0</v>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089497</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>1203000544</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>SEBINZZANG</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>ミスト100ml×2本PDRN配合導入液ヒアルロン酸 弾力水光肌保湿カプセルスキンケア 化粧水 スプレー 艶肌 乾燥肌 敏感肌 低刺激 毛穴 エイジングケア鎮静</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>5400</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="b">
+        <v>0</v>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203000544</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>1203834476</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>KORESHOP</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>白樺水分サンクッション 15g</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>2109</v>
+      </c>
+      <c r="G172" t="n">
+        <v>3</v>
+      </c>
+      <c r="H172" t="b">
+        <v>0</v>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203834476</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J163"/>
+  <autoFilter ref="A1:J172"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 30, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$193</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J172"/>
+  <dimension ref="A1:J193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7507,8 +7507,869 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>1196852846</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>AC ディープカミング ポア サンスティック 20g x 1個 / SPF 50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>デューイーツリー</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="b">
+        <v>0</v>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196852846</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>1132737248</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>バランシウム セラミド 高保湿シート マスク 26ml x 10枚</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>3960</v>
+      </c>
+      <c r="G174" t="n">
+        <v>2</v>
+      </c>
+      <c r="H174" t="b">
+        <v>0</v>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132737248</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>1130447122</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>3番 結果いっぱいのエッセンス トナー 200ml (50種類の発酵/肌の輝き/弾力)</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" t="b">
+        <v>0</v>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130447122</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>1209269112</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>【1+1】マデカソサイド保湿サンスリーム 痕跡リペア 50+50g / SPF 50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>4320</v>
+      </c>
+      <c r="G176" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" t="b">
+        <v>0</v>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209269112</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>1196819316</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>グルタチオンビタシートマスク デイリーピック 30枚</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>2734</v>
+      </c>
+      <c r="G177" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" t="b">
+        <v>0</v>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196819316</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>1182043662</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>エクソソームシカ ツボクサ鎮静クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G178" t="n">
+        <v>0</v>
+      </c>
+      <c r="H178" t="b">
+        <v>0</v>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182043662</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>1174381529</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Kbeautyichiban</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>【正規品】【韓国人気香水 】センノク 香水 50ml スローセプテンバー ウッディ フローラル オリーブヤング 話題香水 slow september</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>SENNOK</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>10390</v>
+      </c>
+      <c r="G179" t="n">
+        <v>1</v>
+      </c>
+      <c r="H179" t="b">
+        <v>0</v>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174381529</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>1177461953</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Kbeautyichiban</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>[正規品] 【数量限定】 センノク 香水 石けんの香り ソープクリーンソープ 50ml / 韓国人気 香水 清潔感</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>SENNOK</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>10990</v>
+      </c>
+      <c r="G180" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" t="b">
+        <v>0</v>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177461953</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>1170826458</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>kseoulshop</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>[コラーゲン美容液]椿 ディープコラーゲン 弾力アンプル 30ml/美容液/コラーゲン/エイジングケア・ハリ・たるみ・毛穴ケア・毛穴たるみ・キメを整える・リフトアップ・保湿・水分ケア・韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>4765</v>
+      </c>
+      <c r="G181" t="n">
+        <v>1</v>
+      </c>
+      <c r="H181" t="b">
+        <v>0</v>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170826458</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>1182484329</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>kseoulshop</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>[企画セット]桃エキス モイスチャーマスク 5枚入り＋1枚プレゼント企画セット/パック・マスクパック・シートマスクパック・韓国パック・保湿ケアパック・トーンケア・トーンアップ</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>2816</v>
+      </c>
+      <c r="G182" t="n">
+        <v>2</v>
+      </c>
+      <c r="H182" t="b">
+        <v>0</v>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182484329</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>1176474050</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>kseoulshop</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>[ハリケア]シカ コラーゲン マスク 30枚入／シートマスクパック・パック・韓国パック・エイジングケア・ハリ・たるみ・赤みケア・ニキビケア・トラブルケア・弾力・リフトアップパック</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>3733</v>
+      </c>
+      <c r="G183" t="n">
+        <v>1</v>
+      </c>
+      <c r="H183" t="b">
+        <v>0</v>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176474050</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>1156813607</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>jeppastore</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>リッチパフューム ボディローション 200ml ホワイトムスクの香り</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>1511</v>
+      </c>
+      <c r="G184" t="n">
+        <v>0</v>
+      </c>
+      <c r="H184" t="b">
+        <v>0</v>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156813607</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>1160365138</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>jeppastore</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>RGIII レッドジンセン スカルプシャンプー 300ml + ヘアパック 200ml スカルプ ＆ ヘア集中ケアセット 紅参 高栄養ケア 脱毛 対策</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>RGIII</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>3071</v>
+      </c>
+      <c r="G185" t="n">
+        <v>1</v>
+      </c>
+      <c r="H185" t="b">
+        <v>0</v>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160365138</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>1159706877</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>jeppastore</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>prep ヒカフェイン モイストオールインワンローション 150g メンズ 乳液 しっとり保湿</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>アモーレパシフィック</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>1594</v>
+      </c>
+      <c r="G186" t="n">
+        <v>0</v>
+      </c>
+      <c r="H186" t="b">
+        <v>0</v>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159706877</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>1201560856</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>[NEW] PDRN カフェイン 1000 オーバーナイト ラッピング マスク 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>P.CALM</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G187" t="n">
+        <v>0</v>
+      </c>
+      <c r="H187" t="b">
+        <v>0</v>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201560856</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>1208992240</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>[NEW] マイルド ヴィーガン トーンアップ 日焼け止め 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G188" t="n">
+        <v>0</v>
+      </c>
+      <c r="H188" t="b">
+        <v>0</v>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208992240</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>1191141866</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>[NEW] スーパー コラーゲン バブル セラム マスク 90g 1個</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>AROCELL</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>5550</v>
+      </c>
+      <c r="G189" t="n">
+        <v>0</v>
+      </c>
+      <c r="H189" t="b">
+        <v>0</v>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191141866</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>1168717728</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>[新商品] キャロット カロチン モイスト エフェクター 55ml 1個</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G190" t="n">
+        <v>0</v>
+      </c>
+      <c r="H190" t="b">
+        <v>0</v>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168717728</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>1146804177</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>[正品] ゼロ 毛穴 ブラックヘッド ディープ クレンジングオイル 205ml 1個</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G191" t="n">
+        <v>0</v>
+      </c>
+      <c r="H191" t="b">
+        <v>0</v>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146804177</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>1211709109</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>leoshopkorea</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>ミジャンセン サロン10 タンパク質 トリートメント 280ml ハイダメージ 髪質改善 補修 保湿 ヘアケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>2541</v>
+      </c>
+      <c r="G192" t="n">
+        <v>0</v>
+      </c>
+      <c r="H192" t="b">
+        <v>0</v>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211709109</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>1195464780</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>leoshopkorea</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>[1+1]大容量 メラトーニング ワンデーアンプル 30ml +30ml 大容量 / 韓国NO.1シミケアアンプル DW-EGF配合 コスパ 肝斑 そばかす 集中ケア 正規品</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>イージーデュー</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>11891</v>
+      </c>
+      <c r="G193" t="n">
+        <v>0</v>
+      </c>
+      <c r="H193" t="b">
+        <v>0</v>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195464780</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J172"/>
+  <autoFilter ref="A1:J193"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 33, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J193"/>
+  <dimension ref="A1:J200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8368,8 +8368,295 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>1207556093</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>itibana</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>FA S　ザ クリア クレンジングジェル クール180mL 国内正規品</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>FAS</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>6534</v>
+      </c>
+      <c r="G194" t="n">
+        <v>0</v>
+      </c>
+      <c r="H194" t="b">
+        <v>0</v>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207556093</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>1207840743</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>syannsyannQ10</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>SA　BON　フェイスポリッシャーリフレッシング 60mL／フェイスウォッシュ（スクラブ）正規品</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>サボン</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G195" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" t="b">
+        <v>0</v>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207840743</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>1207120098</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>LUNORASELECT</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>マスターズ エアリッチ サンスティック 22g 2個 セット ポケモン エディション 日焼け止め UVカット 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>4836</v>
+      </c>
+      <c r="G196" t="n">
+        <v>1</v>
+      </c>
+      <c r="H196" t="b">
+        <v>0</v>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207120098</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>1208245842</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>rarakr</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>コラーゲン バウンシング スリーピング＆ウォッシュオフ マスク (100ml) 弾力・保湿</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>GIK</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>2709</v>
+      </c>
+      <c r="G197" t="n">
+        <v>0</v>
+      </c>
+      <c r="H197" t="b">
+        <v>0</v>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208245842</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>1208668038</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>rarakr</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>フレッシュ クラウド ボディ＆スカルプ スクラブ (ラベンダー＆ペア) 260g ヴィーガン 頭皮ケア 角質ケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G198" t="n">
+        <v>0</v>
+      </c>
+      <c r="H198" t="b">
+        <v>0</v>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208668038</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>1117552337</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>rivina84</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>韓国スキンケア レチノエート X8 プロ ディープリンクル スキンソフナー 150ml ハリと弾力のある潤い肌のためのエッセンス</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>エンプラニ</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>7900</v>
+      </c>
+      <c r="G199" t="n">
+        <v>0</v>
+      </c>
+      <c r="H199" t="b">
+        <v>0</v>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117552337</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>1166659309</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>rivina84</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>秘貼(ビチョプ) ディスカバリーセット/ アンプル / トナー / エマルジョン / クレンジングフォーム / 韓国コスメ 下地 角質 キメケア エイジングケア</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>THE WHOO</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G200" t="n">
+        <v>0</v>
+      </c>
+      <c r="H200" t="b">
+        <v>0</v>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166659309</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J193"/>
+  <autoFilter ref="A1:J200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 36, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$215</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:J215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8655,8 +8655,623 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>1213387450</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Crystal_K</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>THEVITAレチナールショットタイトニングブースター, 15ml, 2個</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>4600</v>
+      </c>
+      <c r="G201" t="n">
+        <v>0</v>
+      </c>
+      <c r="H201" t="b">
+        <v>0</v>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213387450</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>1165615884</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>ゼロ毛穴パッド2.0 70枚1セット</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>3372</v>
+      </c>
+      <c r="G202" t="n">
+        <v>0</v>
+      </c>
+      <c r="H202" t="b">
+        <v>0</v>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165615884</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>1207138612</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>ビーネイチャー バナナ ホワイト マスクパック 10枚入</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>2422</v>
+      </c>
+      <c r="G203" t="n">
+        <v>0</v>
+      </c>
+      <c r="H203" t="b">
+        <v>0</v>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207138612</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>1207138588</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>プランシナジー シルキー マスクパック 10枚入</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>3087</v>
+      </c>
+      <c r="G204" t="n">
+        <v>0</v>
+      </c>
+      <c r="H204" t="b">
+        <v>0</v>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207138588</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>1165228864</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>ザリアルノニエネルギーアンプル30ml 1個</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>3087</v>
+      </c>
+      <c r="G205" t="n">
+        <v>0</v>
+      </c>
+      <c r="H205" t="b">
+        <v>0</v>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165228864</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>1196514379</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>LILIEN</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>[~7/26日までイベント中] ゼロ毛穴パッド本品1+リフィル1＋10枚+ミニケース 計150枚 企画セット</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>5900</v>
+      </c>
+      <c r="G206" t="n">
+        <v>1</v>
+      </c>
+      <c r="H206" t="b">
+        <v>0</v>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196514379</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>1136771755</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>LILIEN</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>ホワイトトリュフ&amp;nbsp;ファースト&amp;nbsp;スプレーセラム100ml + ウォーターフル トーンアップ SUN CREAM(ピンク）50ml 企画セット</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>6700</v>
+      </c>
+      <c r="G207" t="n">
+        <v>0</v>
+      </c>
+      <c r="H207" t="b">
+        <v>0</v>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136771755</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>1205563457</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>ガラクトミー エンザイム ピーリングジェル, 75ml, 1個</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>1829</v>
+      </c>
+      <c r="G208" t="n">
+        <v>0</v>
+      </c>
+      <c r="H208" t="b">
+        <v>0</v>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205563457</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>1171042034</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>アクティブクリーンアップクレンジングパウダー酵素洗顔剤, 80g</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>4005</v>
+      </c>
+      <c r="G209" t="n">
+        <v>1</v>
+      </c>
+      <c r="H209" t="b">
+        <v>0</v>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171042034</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>1203766483</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ サーフィン サンスティック 20g</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>3201</v>
+      </c>
+      <c r="G210" t="n">
+        <v>0</v>
+      </c>
+      <c r="H210" t="b">
+        <v>0</v>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203766483</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>1096782550</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>アクア ヒアルロニック エッセンス 大容量, 250ml</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>3888</v>
+      </c>
+      <c r="G211" t="n">
+        <v>0</v>
+      </c>
+      <c r="H211" t="b">
+        <v>0</v>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096782550</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>1207091863</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>リードルショット フォーメン オールインワン100 Mプラス 150ml＋30ml 企画セット メンズスキンケア 韓国コスメ 化粧水 乳液 美容液</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>3855</v>
+      </c>
+      <c r="G212" t="n">
+        <v>0</v>
+      </c>
+      <c r="H212" t="b">
+        <v>0</v>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091863</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>1174137858</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>ローズマリー &amp;amp; シーソルト &amp;amp; AHA シャンプー 500ml × 2本セット 韓国シャンプー スカルプケア 頭皮クレンジング ボリュームケア</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>オーガニスト</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G213" t="n">
+        <v>0</v>
+      </c>
+      <c r="H213" t="b">
+        <v>0</v>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174137858</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>1024539184</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>[1+1]ハニーアンドマカデミア ネイチャーシャンプー 500ml+プロテイントリートメント 500mlホワイトムスクの香り</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F214" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G214" t="n">
+        <v>1</v>
+      </c>
+      <c r="H214" t="b">
+        <v>0</v>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1024539184</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>1207091851</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>3番 ノーファンデ陶器肌トーンアップUVクリーム 50ml (SPF50+ PA++++) / トーンケアクリーム 保湿ベース 水分クリーム 化粧下地 ナチュラルトーンアップ</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G215" t="n">
+        <v>0</v>
+      </c>
+      <c r="H215" t="b">
+        <v>0</v>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091851</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J200"/>
+  <autoFilter ref="A1:J215"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 39, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$215</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$224</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J215"/>
+  <dimension ref="A1:J224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9270,8 +9270,377 @@
         </is>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>1049486852</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>NRU</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>タイム レボリューション ナイトリペア アンプル 5X, 1個</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>4326</v>
+      </c>
+      <c r="G216" t="n">
+        <v>0</v>
+      </c>
+      <c r="H216" t="b">
+        <v>0</v>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1049486852</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>1093761271</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>インテンシブロングラスティングサンスクリーンEX 60ml /SPF50+PA++++</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>1575</v>
+      </c>
+      <c r="G217" t="n">
+        <v>0</v>
+      </c>
+      <c r="H217" t="b">
+        <v>0</v>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093761271</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>1177950809</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>ブドウ糖ハイドロエッセンストナー, 500ml</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>パティオン</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>3105</v>
+      </c>
+      <c r="G218" t="n">
+        <v>0</v>
+      </c>
+      <c r="H218" t="b">
+        <v>0</v>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177950809</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>1172804214</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>primeland567</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>海ぶどう レチノール 毛穴弾力クリーム 50g</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Mommy Care</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G219" t="n">
+        <v>1</v>
+      </c>
+      <c r="H219" t="b">
+        <v>0</v>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172804214</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>1209321763</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>【GIFT】[プレミアムPDRN セット] (トナー/アンプル/クリーム) 最大3種フル構成+パック1枚贈呈/MEDICUBE</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F220" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G220" t="n">
+        <v>0</v>
+      </c>
+      <c r="H220" t="b">
+        <v>0</v>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209321763</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>1211863823</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>【選べる】リードルショット 100 / 300 / 700 + AHCアイクリーム本品付き (韓国大人気スキンケアセット)</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F221" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G221" t="n">
+        <v>0</v>
+      </c>
+      <c r="H221" t="b">
+        <v>0</v>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211863823</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>1209714705</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>【GIFT】PDRNヒアルロン酸カプセル100セラム, 30ml[プレミアムPDRN セット]ピンクPDRN 基礎セット (アンプル)</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F222" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G222" t="n">
+        <v>0</v>
+      </c>
+      <c r="H222" t="b">
+        <v>0</v>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209714705</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>1209150921</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>【GIFT】【選べる1+1】 自分好みに選ぶ セラム4種セット / 桃セラム ドクダミ ナイアシン PDRN 水光肌 ハリ 弾力 ケア</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F223" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G223" t="n">
+        <v>0</v>
+      </c>
+      <c r="H223" t="b">
+        <v>0</v>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209150921</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>1191691008</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>HANAK-BEAUTYSHOP</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>[1位サンベース]ウォータフルビタカプセルエイジングケアサンクリーム, 50ml/日焼け止め 日焼けどめ ビタミンC 美白 低刺激 紫外線対策 UVカット 日焼け対策 韓国コスメ 化粧下地 プライマー</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F224" t="n">
+        <v>4532</v>
+      </c>
+      <c r="G224" t="n">
+        <v>0</v>
+      </c>
+      <c r="H224" t="b">
+        <v>0</v>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191691008</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J215"/>
+  <autoFilter ref="A1:J224"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 42, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$237</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J224"/>
+  <dimension ref="A1:J237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9639,8 +9639,541 @@
         </is>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>1197355571</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>marynmayjp</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>【公式】スピキュールコラーゲンPDRNクリーム15g／保湿クリーム／CICA／ヒアルロン酸／導入美容液／毛穴／肌のキメ／なめらか肌／化粧ノリ／うるおいハリケア／エイジングケア</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>2190</v>
+      </c>
+      <c r="G225" t="n">
+        <v>3</v>
+      </c>
+      <c r="H225" t="b">
+        <v>0</v>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197355571</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>1209063735</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>marynmayjp</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>【公式】スピキュールアゼライン酸PDRNクリーム15g／CICA／ニキビケア／肌荒れ／ゆらぎ肌／トラブル肌／肌の赤み／鎮静／くすみケア／角質ケア</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>2190</v>
+      </c>
+      <c r="G226" t="n">
+        <v>0</v>
+      </c>
+      <c r="H226" t="b">
+        <v>0</v>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209063735</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>1168503263</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>modepick</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>ハンドウォッシュ LUCIEN CARR 450ml 正規品 ハンドソープ おしゃれな香り 韓国コスメ 韓国人気アイテム</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>GRANHAND</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>3630</v>
+      </c>
+      <c r="G227" t="n">
+        <v>0</v>
+      </c>
+      <c r="H227" t="b">
+        <v>0</v>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168503263</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>1194081987</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>modepick</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>【SEVENTEEN ミンギュ着用】半袖Tシャツ マルチーズ グラフィック プリント YK23HSTS12-1 韓国ファッション オーバーサイズ ユニセックス</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>WaiKei</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>4260</v>
+      </c>
+      <c r="G228" t="n">
+        <v>1</v>
+      </c>
+      <c r="H228" t="b">
+        <v>0</v>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194081987</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>1199679733</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>HIHYMY</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>【韓国限定】ハンドバーム 35ml ナチュラル 高保湿 しっとりケア 韓国トレンド</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>hinok</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G229" t="n">
+        <v>0</v>
+      </c>
+      <c r="H229" t="b">
+        <v>0</v>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199679733</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>1188839770</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>[保湿 保水 栄養 シートマスク 10枚 5種類から選択] 高保湿 まとめ買い 夜用 デイリー スキンケア</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>1709</v>
+      </c>
+      <c r="G230" t="n">
+        <v>2</v>
+      </c>
+      <c r="H230" t="b">
+        <v>0</v>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188839770</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>1197460025</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>【1+1 クリームミスト 120ml】保湿ミスト 化粧水ミスト うるおいケア 整肌ケア スプレー 韓国スキンケア デイリーケア</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F231" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G231" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" t="b">
+        <v>0</v>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197460025</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>1188077394</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>[秀麗な本超保湿クリーム 50ml] 韓国漢方 高保湿 エイジングケア シワ/改/善 /弾力アップ しっとり濃密テクスチャー</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>秀麗韓</t>
+        </is>
+      </c>
+      <c r="F232" t="n">
+        <v>4427</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" t="b">
+        <v>0</v>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188077394</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>1138450382</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>woorinin</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>[BEST] スキン 1004 マダガスカル センテラ アンプル 55ml</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F233" t="n">
+        <v>2480</v>
+      </c>
+      <c r="G233" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" t="b">
+        <v>0</v>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138450382</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>1150649094</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>tiaramall</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>[1+1]センテラ クイックカーミングパッド 70枚入り2個/パックパッドトナーパッド化粧水トナー鎮静水分保湿</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>3591</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" t="b">
+        <v>0</v>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150649094</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>1108196605</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>tiaramall</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>[230ml]アトバリア365クリーム 80ml+ 30ml 5個</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F235" t="n">
+        <v>6678</v>
+      </c>
+      <c r="G235" t="n">
+        <v>0</v>
+      </c>
+      <c r="H235" t="b">
+        <v>0</v>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1108196605</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>1165988568</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>liblingz</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>【GIFT】朝鮮 美女 ジョソンビューティー 米エキス サンクリーム SPF50+/ 70ml/50ml 韓国&amp;amp;グローバル 人気/ 敏感肌向け！/ プロバイオティクス配合サンクリーム</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F236" t="n">
+        <v>1999</v>
+      </c>
+      <c r="G236" t="n">
+        <v>0</v>
+      </c>
+      <c r="H236" t="b">
+        <v>0</v>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165988568</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>1204964045</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>liblingz</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>【GIFT/リニューアル】 トリプルコラーゲントナー 4.0 / 化粧水 ハリ ツヤ インナードライハリ スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>1989</v>
+      </c>
+      <c r="G237" t="n">
+        <v>0</v>
+      </c>
+      <c r="H237" t="b">
+        <v>0</v>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204964045</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J224"/>
+  <autoFilter ref="A1:J237"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 45, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$246</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J237"/>
+  <dimension ref="A1:J246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10172,8 +10172,377 @@
         </is>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>1185242627</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイター 1500ショット ネックパッチ1.0,1枚 /3枚購入ごとに ペプチドトックス ボア/ 体系的管理/一日一枚の習慣で荒れていたネックラインを滑らかに~</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F238" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G238" t="n">
+        <v>1</v>
+      </c>
+      <c r="H238" t="b">
+        <v>0</v>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185242627</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>1194273240</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイター 1500ショット ネックパッチ1.0_1セット(4枚） /1か月集中管理/ 体系的管理/一日一枚の習慣で荒れていたネックラインを滑らかに~</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F239" t="n">
+        <v>4580</v>
+      </c>
+      <c r="G239" t="n">
+        <v>0</v>
+      </c>
+      <c r="H239" t="b">
+        <v>0</v>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194273240</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>1193753404</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイテ 1000 ショート ネックスティック20g+Collagen Naite Thread Neck Cream1.5ml*2ea</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F240" t="n">
+        <v>4680</v>
+      </c>
+      <c r="G240" t="n">
+        <v>1</v>
+      </c>
+      <c r="H240" t="b">
+        <v>0</v>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193753404</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>1190349163</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>ヘソルアナゲンアクティブトニック100ml/つやのないもつれ髪再び生き生きとした髪へ</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>HAESOL</t>
+        </is>
+      </c>
+      <c r="F241" t="n">
+        <v>3880</v>
+      </c>
+      <c r="G241" t="n">
+        <v>0</v>
+      </c>
+      <c r="H241" t="b">
+        <v>0</v>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190349163</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>1212749170</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>easyworld</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>restore pha facial r 200ml</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>ネオストラータ</t>
+        </is>
+      </c>
+      <c r="F242" t="n">
+        <v>4920</v>
+      </c>
+      <c r="G242" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" t="b">
+        <v>0</v>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212749170</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>1122993259</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>easyworld</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>ジェントル クレンジング ジェル 500ml</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>ムステラ</t>
+        </is>
+      </c>
+      <c r="F243" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G243" t="n">
+        <v>1</v>
+      </c>
+      <c r="H243" t="b">
+        <v>0</v>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1122993259</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>1205868858</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>easyworld</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>パーフェクトuv サンスクリーン スキンケアジェル spf50 90g</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>アネッサ</t>
+        </is>
+      </c>
+      <c r="F244" t="n">
+        <v>3780</v>
+      </c>
+      <c r="G244" t="n">
+        <v>0</v>
+      </c>
+      <c r="H244" t="b">
+        <v>0</v>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205868858</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>1107548956</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>ParkGunShop</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>【皮脂バランスケア】セロジンク セバム コントロール トーニング ミスト 150mL さっぱり化粧水ミスト / テカリ対策 / 敏感肌にも</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>ラロッシュポゼ</t>
+        </is>
+      </c>
+      <c r="F245" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G245" t="n">
+        <v>0</v>
+      </c>
+      <c r="H245" t="b">
+        <v>0</v>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107548956</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>1106986645</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>TeaTime</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>【2個セット】シークレット マルチバーム 7g×2 発酵保湿スティック 韓国コスメ 携帯用 高保湿 ツヤ肌 ハリケア</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F246" t="n">
+        <v>4399</v>
+      </c>
+      <c r="G246" t="n">
+        <v>0</v>
+      </c>
+      <c r="H246" t="b">
+        <v>0</v>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106986645</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J237"/>
+  <autoFilter ref="A1:J246"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 48, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$246</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$261</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J246"/>
+  <dimension ref="A1:J261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10541,8 +10541,623 @@
         </is>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>1023263418</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>SWNO1</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>【即納】【正規品】【最新製造日】 1個目 2個目 パースピレックス オリジナル デオドラント ロールオン 脇汗 ワキガ 制汗剤 20ml</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>パースピレックス</t>
+        </is>
+      </c>
+      <c r="F247" t="n">
+        <v>2230</v>
+      </c>
+      <c r="G247" t="n">
+        <v>0</v>
+      </c>
+      <c r="H247" t="b">
+        <v>0</v>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1023263418</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>1016471395</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>SWNO1</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>【即納】【正規品】【最新製造日】 1個目 パースピレックス ストロング デオドラント ロールオン 脇汗 ワキガ 制汗剤 20ml</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>パースピレックス</t>
+        </is>
+      </c>
+      <c r="F248" t="n">
+        <v>2230</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="b">
+        <v>0</v>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1016471395</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>1200694196</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>SWNO1</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>【即納】【正規品】【最新製造日】 1個目 2個目 パースピレックス デオドラント ロールオン 脇汗 ワキガ 制汗剤 20ml</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>パースピレックス</t>
+        </is>
+      </c>
+      <c r="F249" t="n">
+        <v>3660</v>
+      </c>
+      <c r="G249" t="n">
+        <v>1</v>
+      </c>
+      <c r="H249" t="b">
+        <v>0</v>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200694196</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>1176820670</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>mbhonline</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>ラフドット インティメイトウォッシュ アクアラベンダー 詰め替え用 デリケートゾーン用ソープ 100mL</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>laugh.</t>
+        </is>
+      </c>
+      <c r="F250" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G250" t="n">
+        <v>2</v>
+      </c>
+      <c r="H250" t="b">
+        <v>0</v>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176820670</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>1213379918</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>エルセブ トータルリペア 5 インスタントミラクルヘアパック400ml 2個</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F251" t="n">
+        <v>4444</v>
+      </c>
+      <c r="G251" t="n">
+        <v>0</v>
+      </c>
+      <c r="H251" t="b">
+        <v>0</v>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213379918</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>1212659970</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>サロン10プロテインシャンプーダメージヘア用990ml1個</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F252" t="n">
+        <v>3018</v>
+      </c>
+      <c r="G252" t="n">
+        <v>0</v>
+      </c>
+      <c r="H252" t="b">
+        <v>0</v>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212659970</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>1212659429</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>サロン10 プロテイントリートメント ダメージヘア用250ml 3個</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F253" t="n">
+        <v>3956</v>
+      </c>
+      <c r="G253" t="n">
+        <v>0</v>
+      </c>
+      <c r="H253" t="b">
+        <v>0</v>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212659429</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>1212659125</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>サロン10プロテインヘアトリートメント極ダメージヘア用250ml1個</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F254" t="n">
+        <v>1806</v>
+      </c>
+      <c r="G254" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" t="b">
+        <v>0</v>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212659125</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>1162075812</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>goingover</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>JEANNE ARTHES(ジャンヌ・アルテス) ジャンヌ・アルテス スルタン オードパルファム 1</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>ジャンヌアルテス</t>
+        </is>
+      </c>
+      <c r="F255" t="n">
+        <v>4144</v>
+      </c>
+      <c r="G255" t="n">
+        <v>3</v>
+      </c>
+      <c r="H255" t="b">
+        <v>0</v>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162075812</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>1163081544</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>goingover</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>ラ・カスタ アロマエステ ヘアローション スムース リフィル(詰め替え用) *髪用ローション*</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>ラ・カスタ</t>
+        </is>
+      </c>
+      <c r="F256" t="n">
+        <v>2312</v>
+      </c>
+      <c r="G256" t="n">
+        <v>1</v>
+      </c>
+      <c r="H256" t="b">
+        <v>0</v>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163081544</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>1188763613</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>geishaCat</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>ジルリーン 涙袋ペンシル (031 クリームベージュ) ライトカラー 涙袋 コンシーラー アイライン</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>jill leen.</t>
+        </is>
+      </c>
+      <c r="F257" t="n">
+        <v>2254</v>
+      </c>
+      <c r="G257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H257" t="b">
+        <v>0</v>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188763613</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>1188906909</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>geishaCat</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>ナナコスター LEA メイクバーム 45g スタイリング剤 ワックス シアバター 保湿 濡れ髪 オレンジベルガモットの香り サロン品質 ヘア バーム メンズ レディース</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>ナナコスター</t>
+        </is>
+      </c>
+      <c r="F258" t="n">
+        <v>3612</v>
+      </c>
+      <c r="G258" t="n">
+        <v>0</v>
+      </c>
+      <c r="H258" t="b">
+        <v>0</v>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188906909</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>1207551225</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>happypunch</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>アリィー クロノビューティ フラットスムースフィルターＵＶ 厚塗り感ないフラット美肌へ 凹凸補整フィルターＵＶ SPF50＋／PA＋＋＋＋／UV耐水性スーパーウォータープルーフフリクションプルーフ普段</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>アリィー</t>
+        </is>
+      </c>
+      <c r="F259" t="n">
+        <v>2223</v>
+      </c>
+      <c r="G259" t="n">
+        <v>1</v>
+      </c>
+      <c r="H259" t="b">
+        <v>0</v>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207551225</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>1209149814</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>happypunch</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>NILE 泥パック 毛穴パック ピーリング 黒ずみ 角質取り</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Nile</t>
+        </is>
+      </c>
+      <c r="F260" t="n">
+        <v>1984</v>
+      </c>
+      <c r="G260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" t="b">
+        <v>0</v>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209149814</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>1209149809</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>happypunch</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>NILE ピーリングジェル 角質取り 顔 メンズレディース (CALIFORNIAグレープフルーツの香り)</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Nile</t>
+        </is>
+      </c>
+      <c r="F261" t="n">
+        <v>2684</v>
+      </c>
+      <c r="G261" t="n">
+        <v>0</v>
+      </c>
+      <c r="H261" t="b">
+        <v>0</v>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209149809</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J246"/>
+  <autoFilter ref="A1:J261"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 51, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$268</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J261"/>
+  <dimension ref="A1:J268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11156,8 +11156,295 @@
         </is>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>1200862105</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>kirei-station</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>【2個セット】チャコット フィニッシングキープミスト クール 50ml×2 メイクの仕上げや下地に使える2WAYミスト 清涼感とうるおいを与えメイクをキープ ふわふわ微細ミストの1層式 日本製</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>チャコット</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>3479</v>
+      </c>
+      <c r="G262" t="n">
+        <v>3</v>
+      </c>
+      <c r="H262" t="b">
+        <v>0</v>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200862105</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>1190965338</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>aperire_official</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>ビープローズン ポア パックトゥフォーム 洗顔料 120g クーリング 毛穴 パックフォーム</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>アペリレ</t>
+        </is>
+      </c>
+      <c r="F263" t="n">
+        <v>1755</v>
+      </c>
+      <c r="G263" t="n">
+        <v>0</v>
+      </c>
+      <c r="H263" t="b">
+        <v>0</v>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190965338</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>1146790722</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>aperire_official</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>[Glass Skin] ブルーミングデイズ グローバーム 01 pure</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>アペリレ</t>
+        </is>
+      </c>
+      <c r="F264" t="n">
+        <v>3120</v>
+      </c>
+      <c r="G264" t="n">
+        <v>1</v>
+      </c>
+      <c r="H264" t="b">
+        <v>0</v>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146790722</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>1200827772</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>itfu-cosmetic</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>【キメ・毛穴・ハリ3つのケア／2個SET】スキンリバランシング スンユルアンプル50ml　PDRN ペプチド スキンブースター ハトムギ成分 毛穴ケア コラーゲン ナイアシンアミド 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>イッピュ</t>
+        </is>
+      </c>
+      <c r="F265" t="n">
+        <v>4150</v>
+      </c>
+      <c r="G265" t="n">
+        <v>3</v>
+      </c>
+      <c r="H265" t="b">
+        <v>0</v>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200827772</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>1212133884</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>b-labskincare</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>【公式】【クレンジング1位・W洗顔不要】スクアレンリセットポアディープクレンジングオイル, 200ml (メイク落とし /毛穴汚れ/スクワラン/LHA/高保/ブラックヘッド/敏感肌/低刺激)</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>B:Lab</t>
+        </is>
+      </c>
+      <c r="F266" t="n">
+        <v>1520</v>
+      </c>
+      <c r="G266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H266" t="b">
+        <v>0</v>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212133884</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>1115638534</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>旅行用ヘアボディ5種+コットンポーチ1セット 韓国シャンプー 純正品 旅行キット トラベルキット トリートメント ボディウォッシュ ボディローション クレンジングフォーム 旅行 携帯用シャンプー</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>NARD</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G267" t="n">
+        <v>0</v>
+      </c>
+      <c r="H267" t="b">
+        <v>0</v>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115638534</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>1149453077</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>dal24</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>プロフェッショナル頭皮シャンプーブラシ1本 韓国 頭皮 ブラシ シャンプー 櫛 マッサージ 角質 フケ におい ヘアー</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>rolencos</t>
+        </is>
+      </c>
+      <c r="F268" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" t="b">
+        <v>0</v>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149453077</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J261"/>
+  <autoFilter ref="A1:J268"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 54, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$268</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$275</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J268"/>
+  <dimension ref="A1:J275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11443,8 +11443,295 @@
         </is>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>1198755469</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>kiwiglow</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>ビーガンジェジュ 蓮マイルド角質ケアトナーパッド</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>KIWIGLOW</t>
+        </is>
+      </c>
+      <c r="F269" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G269" t="n">
+        <v>1</v>
+      </c>
+      <c r="H269" t="b">
+        <v>0</v>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198755469</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>1196826611</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml / 保湿乳液 敏感肌対応 うるおいケア スキンケアローション 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F270" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G270" t="n">
+        <v>3</v>
+      </c>
+      <c r="H270" t="b">
+        <v>0</v>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196826611</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>1164705875</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>ウォータープルーフプロ日焼け止め 50g+サンスティック 20g / アウトドア スポーツ対応UVクリーム 汗・水に強いスティックタイプ 手を汚さない</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F271" t="n">
+        <v>5499</v>
+      </c>
+      <c r="G271" t="n">
+        <v>1</v>
+      </c>
+      <c r="H271" t="b">
+        <v>0</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164705875</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>1178111873</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>K-beautyclub</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>クリーンノート パウダリーコットン シャンプー 1L + トリートメント 1L セット頭皮ケア・皮脂除去・弱酸性・爽やかな香りのスカルプシャンプー</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>3799</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="b">
+        <v>0</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178111873</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>1190126098</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>kiseki-select</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>スピケア V3エキサイティングファンデーション 15g 本体 SPICARE 韓国コスメ LOT番号付</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>SPICARE</t>
+        </is>
+      </c>
+      <c r="F273" t="n">
+        <v>4529</v>
+      </c>
+      <c r="G273" t="n">
+        <v>0</v>
+      </c>
+      <c r="H273" t="b">
+        <v>0</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190126098</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>1205431137</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>kiseki-select</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>ミルボン ジェミールフラン メルティバターバーム 40g 2個セット 洗い流さない トリートメント アウトバス ハンドクリーム 美容室 サロン専売品 ミルボン milbon ヘアケア おすす</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G274" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" t="b">
+        <v>0</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205431137</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>1192993118</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>kiseki-select</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>REVI ルヴィ セルフゴマージュ SUPER 120g 基礎化粧品 ピーリング ゴマージュ マッサージ フェイシャルケア ホームケア ホームエステ REVI 銀座ロッソ 透明感 ハリ</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>REVI</t>
+        </is>
+      </c>
+      <c r="F275" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G275" t="n">
+        <v>0</v>
+      </c>
+      <c r="H275" t="b">
+        <v>0</v>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192993118</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J268"/>
+  <autoFilter ref="A1:J275"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 57, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$275</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$297</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J275"/>
+  <dimension ref="A1:J297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11730,8 +11730,910 @@
         </is>
       </c>
     </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>1187961763</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>[2026] NEW 最低特典カーミング バランスジェル-保湿 / 鎮静 100ml(1+1)</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F276" t="n">
+        <v>9920</v>
+      </c>
+      <c r="G276" t="n">
+        <v>3</v>
+      </c>
+      <c r="H276" t="b">
+        <v>0</v>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187961763</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>1174936338</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>プリジュビネーション ファーミングバクチオールセラム[童顔弾力セラム] 50ml</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F277" t="n">
+        <v>6902</v>
+      </c>
+      <c r="G277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H277" t="b">
+        <v>0</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174936338</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>1208171928</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>[2026BEST] ザマトロジー 2種 セット-光彩 / 弾力(ブースター130ml+セラム45ml)</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F278" t="n">
+        <v>12799</v>
+      </c>
+      <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="b">
+        <v>0</v>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208171928</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>1199006617</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Jurian</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>アゼライン酸16BBカーミングセラム, 30ml</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F279" t="n">
+        <v>2578</v>
+      </c>
+      <c r="G279" t="n">
+        <v>1</v>
+      </c>
+      <c r="H279" t="b">
+        <v>0</v>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199006617</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>1199701690</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Jurian</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>カーミング バランスジェル 100ml / 水分バランス 調節</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F280" t="n">
+        <v>4735</v>
+      </c>
+      <c r="G280" t="n">
+        <v>0</v>
+      </c>
+      <c r="H280" t="b">
+        <v>0</v>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199701690</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>1193433365</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>【公式】 コナピディル フィクシカ CONAPIDIL Fixcica 13g</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F281" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G281" t="n">
+        <v>3</v>
+      </c>
+      <c r="H281" t="b">
+        <v>0</v>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433365</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>1193433355</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>【公式】 コナピディル グリーンボクシン CONAPIDIL Greenboxin 150ml</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F282" t="n">
+        <v>9200</v>
+      </c>
+      <c r="G282" t="n">
+        <v>2</v>
+      </c>
+      <c r="H282" t="b">
+        <v>0</v>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433355</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>1193433366</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>【公式】 コナピディル フィニッシュローション CONAPIDIL Finish Lotion 20g</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F283" t="n">
+        <v>9800</v>
+      </c>
+      <c r="G283" t="n">
+        <v>1</v>
+      </c>
+      <c r="H283" t="b">
+        <v>0</v>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433366</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>1193433359</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>【公式】 アクセンダ ルティナー aXENDA Routiner 15ml</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F284" t="n">
+        <v>9100</v>
+      </c>
+      <c r="G284" t="n">
+        <v>2</v>
+      </c>
+      <c r="H284" t="b">
+        <v>0</v>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433359</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>1210385244</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>【日本メーカ―公式】ファーマ21 モイストリペアヘアマスク 乾燥ケア しっとり保湿 髪質ケア パサつき・広がり対策 サロン品質 ヘアトリートメント ヘアパック 230g</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F285" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G285" t="n">
+        <v>0</v>
+      </c>
+      <c r="H285" t="b">
+        <v>0</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210385244</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>1210384486</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>【日本メーカー公式】ファーマ21 ラグジュリアスリペアヘアマスク 年齢髪ケア 髪質改善 ダメージ補修 美容液成分配合 しっとりまとまる髪 サロン品質 ヘアトリートメント ヘアパック 230g</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F286" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G286" t="n">
+        <v>0</v>
+      </c>
+      <c r="H286" t="b">
+        <v>0</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210384486</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>1210384445</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>【日本メーカー公式】ファーマ21 シルキーグロスリペアヘアマスク 湿気対策 髪質改善 くせ毛・うねり・広がり・パサつき・絡まりケア シルクのようなツヤ髪へ サロン品質 ヘアトリートメント ヘアパック</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F287" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G287" t="n">
+        <v>0</v>
+      </c>
+      <c r="H287" t="b">
+        <v>0</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210384445</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>1199000651</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>【日本メーカー公式】ファーマ21 すっきりヘアコアシャンプー フケかゆみ 芯から補修 パサつき抑え もこもこ泡 摩擦レス 軽やか指通り 爽快感 低刺激 無添加 445mL</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F288" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0</v>
+      </c>
+      <c r="H288" t="b">
+        <v>0</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199000651</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>1175249089</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>ザ セラミド スキンバリア モイスチャライザークリーム 80ml 2個</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>6230</v>
+      </c>
+      <c r="G289" t="n">
+        <v>0</v>
+      </c>
+      <c r="H289" t="b">
+        <v>0</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175249089</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>1152704413</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>オーガニック ホホバオイル ゴールド 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>FRANCOISE&amp;amp;Fragrance</t>
+        </is>
+      </c>
+      <c r="F290" t="n">
+        <v>2506</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="b">
+        <v>0</v>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152704413</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>1154992110</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>レッド ブレミッシュ スージング アップ サンクリーム SPF50+ PA++++ 50ml 2個</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F291" t="n">
+        <v>4149</v>
+      </c>
+      <c r="G291" t="n">
+        <v>0</v>
+      </c>
+      <c r="H291" t="b">
+        <v>0</v>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154992110</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>1154991907</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>KIRAKORE</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラ エアフィット サンクリーム プラス 50ml 2個</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>3984</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0</v>
+      </c>
+      <c r="H292" t="b">
+        <v>0</v>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154991907</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>1213443102</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>[正規品]アーバンエコ ハラケケ トナー 150ml, 1個</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F293" t="n">
+        <v>3028</v>
+      </c>
+      <c r="G293" t="n">
+        <v>0</v>
+      </c>
+      <c r="H293" t="b">
+        <v>0</v>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213443102</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>1200735680</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>[正規品]ALL NEW シグニア リファイニング ウォーターエッセンス 180ml, 1個</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>ヘラ</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>10543</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0</v>
+      </c>
+      <c r="H294" t="b">
+        <v>0</v>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200735680</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>1196714483</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>[正規品] レチノール レティジェクション セラム 30ml, 1個</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>7345</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0</v>
+      </c>
+      <c r="H295" t="b">
+        <v>0</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196714483</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>1165247523</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>[正規品] オールデイ メイクアップフィクサー 75ml 1個</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>3013</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="b">
+        <v>0</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165247523</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>1213167963</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>[正規品]インテンスケア ゴールド 24K スネイルフォームクレンザー 150ml, 1個</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>2434</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0</v>
+      </c>
+      <c r="H297" t="b">
+        <v>0</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213167963</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J275"/>
+  <autoFilter ref="A1:J297"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 60, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$297</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$310</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J297"/>
+  <dimension ref="A1:J310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12632,8 +12632,541 @@
         </is>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>1205550323</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>リジュラン ダーマ ヒーラー ポア タイトニング トナー パッド 220mL</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>3960</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0</v>
+      </c>
+      <c r="H298" t="b">
+        <v>0</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205550323</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>1177829431</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>マイファーストセラム 50ml</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>De:maf</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>2430</v>
+      </c>
+      <c r="G299" t="n">
+        <v>0</v>
+      </c>
+      <c r="H299" t="b">
+        <v>0</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177829431</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>1158425809</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>グリーンディープポアクレンジングバーム 100g</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G300" t="n">
+        <v>1</v>
+      </c>
+      <c r="H300" t="b">
+        <v>0</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158425809</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>1164170834</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>sweet-box</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>[SKIN1004] (jL) Madagascar Centella Poremizing Light Gel Cream 75ml / マダガスカル センテラ ポアミゼーション ライトジェルクリー</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>1899</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0</v>
+      </c>
+      <c r="H301" t="b">
+        <v>0</v>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164170834</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>1199692215</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>ラサーナ 海藻 ヘア セラム ミスト（200ml）</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F302" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0</v>
+      </c>
+      <c r="H302" t="b">
+        <v>0</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692215</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>1199692156</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>ラサーナ 海藻 海泥 シャンプー＆トリートメント セット（空ボトル付き）</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>7300</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0</v>
+      </c>
+      <c r="H303" t="b">
+        <v>0</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692156</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>1199692199</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>ラサーナ 海藻 ヘア セラム ミルク 120g</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0</v>
+      </c>
+      <c r="H304" t="b">
+        <v>0</v>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692199</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>1199692158</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>ラサーナ プレミオール ホワイトティーの香り 2点セット シャンプー＆トリートメントセット（空ボトル付き）</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>7940</v>
+      </c>
+      <c r="G305" t="n">
+        <v>1</v>
+      </c>
+      <c r="H305" t="b">
+        <v>0</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692158</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>1195196973</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>HIHYMY26</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>1秒 ダメージケア マーブル ヘアパック 300g LPP プロテイン トリートメント</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>BIORECIPE</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>5224</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="b">
+        <v>0</v>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195196973</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>1212713877</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Lulupi</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>【フィー】 シェイキングシナジーミスト 50ml 全3種</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>2654</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0</v>
+      </c>
+      <c r="H307" t="b">
+        <v>0</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212713877</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>1181847777</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>【ポムポムプリンコラボ】ライティングトーンアップサンクッション/ヴィーガンリリーフサンクリーム/サンエッセンス/オーセンティックリップグロイバーム/セット企画 / オリーブヤング限定</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>アッテ</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G308" t="n">
+        <v>2</v>
+      </c>
+      <c r="H308" t="b">
+        <v>0</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181847777</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1189371186</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>【NEW!】 シェイキングミスト</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>2856</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="b">
+        <v>0</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189371186</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>1213323194</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>【ピングーコラボ】全種まとめ ポストアルファクーリングパッド 70枚+70枚 / クーリングペプチドアンプル 30ml / ファーストクーリングマスク 5+3枚 / シカクーリングマスク 5+3枚</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>2310</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="b">
+        <v>0</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213323194</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J297"/>
+  <autoFilter ref="A1:J310"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 63, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$310</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$322</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J310"/>
+  <dimension ref="A1:J322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13165,8 +13165,500 @@
         </is>
       </c>
     </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>1068190736</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>arimcosmetic</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>パフュームシードライン6種 ボディウォッシュ クリーム ローション ミルク クレンザー ミスト オイル香りと保湿を一度に 5つの無添加 超微粒 バラエキス ギフト用</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G311" t="n">
+        <v>3</v>
+      </c>
+      <c r="H311" t="b">
+        <v>0</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1068190736</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>1120351146</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>arimcosmetic</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>【30枚】すりおろしのマスクシート 新鮮な自然植物たっぷり 高密着 無添加 保湿 栄養 水分 鎮静 アロエ キュウリ 韓国コスメマスクパックです</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>2660</v>
+      </c>
+      <c r="G312" t="n">
+        <v>1</v>
+      </c>
+      <c r="H312" t="b">
+        <v>0</v>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120351146</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>1088835091</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>arimcosmetic</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>旅行用/ 携帯用 化粧品コレクション 韓国コスメ 1ml x 120枚 5ml x 30個 アンプル エマルジョン クリーム CC アイクリーム クレンジングフォーム セラム</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>イザノックス</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="b">
+        <v>0</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1088835091</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>1191255099</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>laglow</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>5番 白玉グルタチオンC トーンアップベース SPF50+ PA++++ 30ml 美容液下地 UV下地 化粧下地 トーンアップ 透明感 ツヤ肌 日焼け止め 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>2655</v>
+      </c>
+      <c r="G314" t="n">
+        <v>3</v>
+      </c>
+      <c r="H314" t="b">
+        <v>0</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191255099</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>1177685719</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>laglow</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>センテラ ティーツリカ リリーフ アンプル 100ml / SOS鎮静ケア / ゆらぎ肌対策 / 水分アンプル / ノンコメドジェニック / オイリー肌向け</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>2350</v>
+      </c>
+      <c r="G315" t="n">
+        <v>2</v>
+      </c>
+      <c r="H315" t="b">
+        <v>0</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177685719</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>1199411031</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>[2+2] 白樺 水分 日焼け止めスプレー, 100ml 4ea(SPF 50 + PA ++++)</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>6007</v>
+      </c>
+      <c r="G316" t="n">
+        <v>0</v>
+      </c>
+      <c r="H316" t="b">
+        <v>0</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199411031</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>1164978194</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>peachshop</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>【ビビアン】 ニチ ルームスプレー ウォルナット クリーク グリーン 100ml 1個, 繊維香水 繊維脱臭剤 ドレスパフューム Walnut Creek Green</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G317" t="n">
+        <v>1</v>
+      </c>
+      <c r="H317" t="b">
+        <v>0</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164978194</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>1095419459</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>peachshop</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>コントロールA ティーツリーメントスージング スポット 15m /Ctrl+A/ピンクパウダー/ニキビ/ニキビケア/ 薬/teatree/吹き出物/肌荒れ/集中ケア/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>3099</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0</v>
+      </c>
+      <c r="H318" t="b">
+        <v>0</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1095419459</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>1212001587</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>wish</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>レプリカ オン ア デート EDT BT 7ml【ミニ香水 ミニボトル】【香水 メンズ レディース】</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>1925</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0</v>
+      </c>
+      <c r="H319" t="b">
+        <v>0</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212001587</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>1212001233</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>wish</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>アクア エッセンツィアーレ ブルー EDT SP 100ml【香水 ギフト メンズ】</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>CHANEL</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>7645</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0</v>
+      </c>
+      <c r="H320" t="b">
+        <v>0</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212001233</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>1195231911</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>wish</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>サムライ ライト EDT SP 100ml SAMOURAI LIGHT【香水 メンズ】ALAIN DELON アラン・ドロン</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>サムライ</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>4763</v>
+      </c>
+      <c r="G321" t="n">
+        <v>0</v>
+      </c>
+      <c r="H321" t="b">
+        <v>0</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195231911</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>1208366563</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>srcosme</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>【ミニサイズ】クリスチャン ディ オール ソヴァージュ パルファン　10ml メンズ　Sauvage　PARFUM 10mL</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Dior</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G322" t="n">
+        <v>1</v>
+      </c>
+      <c r="H322" t="b">
+        <v>0</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208366563</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J310"/>
+  <autoFilter ref="A1:J322"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 66, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$322</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$330</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J322"/>
+  <dimension ref="A1:J330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13657,8 +13657,336 @@
         </is>
       </c>
     </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>1194573796</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュクリアスージングクリーム, 70ml, 2個</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0</v>
+      </c>
+      <c r="H323" t="b">
+        <v>0</v>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194573796</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>1193991472</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>yujunystore</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>ティーツリーカ リリーフ アンプル,1個,100ml</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>3634</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0</v>
+      </c>
+      <c r="H324" t="b">
+        <v>0</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193991472</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>1203740798</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>631403</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>【香水のまとめ NEW登場】騎士ユニコーン/イチゴキューピッド/レディース/ストロベリーキューピットフレグランス/パフューム/アトマイザー/高い賦香率/魅力的な香り/新年プレゼント/中国</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>FLOWER KNOWS</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>4299</v>
+      </c>
+      <c r="G325" t="n">
+        <v>2</v>
+      </c>
+      <c r="H325" t="b">
+        <v>0</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203740798</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>1208001525</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>autumnrock</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>イハダ 化粧水 しっとり 薬用ローション 肌荒れ 混合肌 ニキビ 乾燥 敏感肌 低刺激 うるおい 本体 ニキビ 弱酸性 無香料 無着色 無添加 180mL</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>イハダ</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>1960</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0</v>
+      </c>
+      <c r="H326" t="b">
+        <v>0</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208001525</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>1153497615</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>AHA 30% + BHA 2% ピーリングソリューション 30ml</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>2597</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0</v>
+      </c>
+      <c r="H327" t="b">
+        <v>0</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1153497615</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>1152849853</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>[26SS/New]デオキシリボス 頭皮強化アンプル 20ml #エクソソーム #ビオチン #EGF</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>4652</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0</v>
+      </c>
+      <c r="H328" t="b">
+        <v>0</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152849853</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>1171460964</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>パフュームドポ ボディウォッシュ 600ml 2種から1つ選択</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>VEILMENT</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>2532</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0</v>
+      </c>
+      <c r="H329" t="b">
+        <v>0</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171460964</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>1166654877</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>[26SS/New]アイパッチ 60枚 2種（コラーゲン／キャビア PDRN）から1つ選択</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>2851</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0</v>
+      </c>
+      <c r="H330" t="b">
+        <v>0</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166654877</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J322"/>
+  <autoFilter ref="A1:J330"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 69, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$330</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$343</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J330"/>
+  <dimension ref="A1:J343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13985,8 +13985,541 @@
         </is>
       </c>
     </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>1167872503</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>beautyplace</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>スノーウォーターフォースカルプ＆ボディ シトラスクール 化粧水 スカルプケア 頭皮ケア冷感 ボディミスト 猛暑対策</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>DAILY AROMA JAPAN</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G331" t="n">
+        <v>0</v>
+      </c>
+      <c r="H331" t="b">
+        <v>0</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167872503</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>1188510609</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>AVECPUBLIC</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>スーパージェクションクリーム, 20ml</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>7560</v>
+      </c>
+      <c r="G332" t="n">
+        <v>3</v>
+      </c>
+      <c r="H332" t="b">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188510609</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>1126626890</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>超低分子 ヒアルロン酸 トナー 300ml</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>イズエンツリー</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>3286</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="b">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1126626890</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>1127123405</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>PH センシティブ クリーム 60ml</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>5309</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="b">
+        <v>0</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1127123405</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>1199417296</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>プランプハニー セラム 美容液 30g</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>ByUR</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>4845</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
+      <c r="H335" t="b">
+        <v>0</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199417296</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>1142360945</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>毛髪コア強化高栄養タンパク質クリームヘアトリートメント200ml</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>ラグライア</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>2785</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
+      <c r="H336" t="b">
+        <v>0</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142360945</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>1205346742</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>KKK-Shop</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>[メガ割] TAMBURIN*S タンバリン*ズ ヘアオイル 50ml サマーテイルズ イブニンググロウ カモ ダメージ補修 ツヤ 潤い 香り 髪質改善 スタイリング フレグランス 韓国ヘアケア 正規</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>5481</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0</v>
+      </c>
+      <c r="H337" t="b">
+        <v>0</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205346742</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>1212617358</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>ROUTE_K_SEOUL</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>グロウターン エクソソーム スカルプブラシアンプル 100ml 頭皮美容液 韓国ヘアケア</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0</v>
+      </c>
+      <c r="H338" t="b">
+        <v>0</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212617358</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>1135385776</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>p0-town</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>[シカ ディープクレンジング] クリーンイット ゼロ カーミング クレンジング バーム 100ml</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>2030</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0</v>
+      </c>
+      <c r="H339" t="b">
+        <v>0</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135385776</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>1203288450</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>medifa</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>.ダヴ ふわとろクリーミースクラブ ミッドナイトラベンダー 298g Dove ダブ ボディスクラブ【P】</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>ダヴ</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>1768</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
+      <c r="H340" t="b">
+        <v>0</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203288450</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>1201842300</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>medifa</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>.プロスタイル アイス美容スパークリングスプレー 95g ドライシャンプー【R】</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>プロスタイル</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0</v>
+      </c>
+      <c r="H341" t="b">
+        <v>0</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201842300</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>1083089713</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>ピュアフィットシカ 弱酸性クレンジングパッド 100枚入 * 1個</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+      <c r="H342" t="b">
+        <v>0</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083089713</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>1082221247</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>ムード ペブル ネイル 29種</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>ロムアンド</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
+      <c r="H343" t="b">
+        <v>0</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1082221247</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J330"/>
+  <autoFilter ref="A1:J343"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 72, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$343</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$349</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J343"/>
+  <dimension ref="A1:J349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14518,8 +14518,254 @@
         </is>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>1190175660</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>マダガスカルセントラアンプル 55ml, 1個</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>2795</v>
+      </c>
+      <c r="G344" t="n">
+        <v>1</v>
+      </c>
+      <c r="H344" t="b">
+        <v>0</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175660</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>1190175438</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>ノーセバム サンクッション EX SPF50+ PA++++, 1個</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0</v>
+      </c>
+      <c r="H345" t="b">
+        <v>0</v>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175438</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>1210577063</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>wingkone</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>【正規品】【NEW】【脱色/染め】 眉毛脱色 イージーブロウトーンチェンジャー 5回分 / イージーブロウムードチェンジャー 5回分 / アイブロウ / 韓国コスメ / 眉毛</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G346" t="n">
+        <v>3</v>
+      </c>
+      <c r="H346" t="b">
+        <v>0</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210577063</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>1181822405</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>kirakirahosi</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>ACON エクオンディープ クレンジングフォーム 100mL</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0</v>
+      </c>
+      <c r="H347" t="b">
+        <v>0</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181822405</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1181822404</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>kirakirahosi</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>コンセントレートアンプル 30ml クリニックライン</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>5300</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0</v>
+      </c>
+      <c r="H348" t="b">
+        <v>0</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181822404</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>1192796253</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>heyhey</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>リジュビエス　アンプル　６ml x 2本入り リジュビ-エス　リジュビーS</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>4650</v>
+      </c>
+      <c r="G349" t="n">
+        <v>3</v>
+      </c>
+      <c r="H349" t="b">
+        <v>0</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192796253</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J343"/>
+  <autoFilter ref="A1:J349"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 75, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$349</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$370</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J349"/>
+  <dimension ref="A1:J370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14764,8 +14764,869 @@
         </is>
       </c>
     </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>1161193499</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>BURUN</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>【韓国公式化粧品】EGFスケーリングモイスチャーフットクリーム 130g 角質ケア 韓国コスメ 高保湿</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>2150</v>
+      </c>
+      <c r="G350" t="n">
+        <v>0</v>
+      </c>
+      <c r="H350" t="b">
+        <v>0</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161193499</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>1163018199</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>BURUN</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>【1+1】角質ケア導入美容液 つるつるブースターエッセンス 100ml×2本</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>CNP Laboratory</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G351" t="n">
+        <v>0</v>
+      </c>
+      <c r="H351" t="b">
+        <v>0</v>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163018199</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>1201938749</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>beautique</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>ベアバニーコレクティングサンパウダー 5g 毛穴カバー 4種</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>EDIT.B</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>1780</v>
+      </c>
+      <c r="G352" t="n">
+        <v>0</v>
+      </c>
+      <c r="H352" t="b">
+        <v>0</v>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201938749</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>1189270361</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>【Wid】 フォリゲン トニック 120ml 2個セット・頭皮ケア・ヘアトニック・抜け毛予防・頭皮栄養・スカルプケア</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>5287</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0</v>
+      </c>
+      <c r="H353" t="b">
+        <v>0</v>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189270361</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>1188452071</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>【Wid】 アスコルビルテトラィソパルミテート ソリューション 20% イン ビタミンF / 30ml / 1個 / ビタミンC美容液 / オイル美容液 / 透明感 / ハリケア</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F354" t="n">
+        <v>5841</v>
+      </c>
+      <c r="G354" t="n">
+        <v>0</v>
+      </c>
+      <c r="H354" t="b">
+        <v>0</v>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452071</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>1188452072</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>【Wid】 グリコール酸 7% エクスフォリエイティング トナー / 240ml / 2個セット / ふき取り化粧水 / 角質ケア / 肌キメ整え / ツヤ肌</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>6385</v>
+      </c>
+      <c r="G355" t="n">
+        <v>0</v>
+      </c>
+      <c r="H355" t="b">
+        <v>0</v>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452072</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>1179809144</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>[角質ケア] マンデル酸 10％ + HA 30ml 毛穴ケア つるつる美肌 セラム</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G356" t="n">
+        <v>0</v>
+      </c>
+      <c r="H356" t="b">
+        <v>0</v>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179809144</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>1169201226</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>[1+1]ジェントルブラック フレッシュ クレンジングオイル 150ml+150ml</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>4584</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0</v>
+      </c>
+      <c r="H357" t="b">
+        <v>0</v>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169201226</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>1110101930</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>フォリゲンシャンプー 500ml</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F358" t="n">
+        <v>2847</v>
+      </c>
+      <c r="G358" t="n">
+        <v>0</v>
+      </c>
+      <c r="H358" t="b">
+        <v>0</v>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110101930</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>1202057165</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>[1+1] インフューズド コラーゲン コンセントレート フルイド 50ml 2件</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>4428</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0</v>
+      </c>
+      <c r="H359" t="b">
+        <v>0</v>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202057165</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>1202051148</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>インフュージングコラーゲンパウダー, 1.5g</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>3258</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0</v>
+      </c>
+      <c r="H360" t="b">
+        <v>0</v>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202051148</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>1202043668</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>thenido</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>[1+1] インフュージングコラーゲンミスト 50ml 2件</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>BEAUDIANI</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>4473</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
+      <c r="H361" t="b">
+        <v>0</v>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202043668</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>1159643310</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>ハッピー フォーメン EDC 50ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>クリニーク</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0</v>
+      </c>
+      <c r="H362" t="b">
+        <v>0</v>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159643310</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>1158430479</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>アベンヌウォーター 300ml 3本セット （化粧水）</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>アベンヌ</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>3620</v>
+      </c>
+      <c r="G363" t="n">
+        <v>3</v>
+      </c>
+      <c r="H363" t="b">
+        <v>0</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158430479</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>1162421706</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>クラシック ウォームコットン EDP 30ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>クリーン</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0</v>
+      </c>
+      <c r="H364" t="b">
+        <v>0</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162421706</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>1192146158</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>アナスイ EDT 30ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>アナスイ</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>3020</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0</v>
+      </c>
+      <c r="H365" t="b">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192146158</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>1189247744</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>アルティム8 スブリム ビューティクレンジングオイルn 150ml （メイク落とし） 【国内正規品】</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>シュウウエムラ</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>5610</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0</v>
+      </c>
+      <c r="H366" t="b">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189247744</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>1198883487</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>cocodrug</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>【国内正規品】 アールエムケー　Wトリートメントオイル　(美容オイル) 50ml</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>アールエムケー</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>3740</v>
+      </c>
+      <c r="G367" t="n">
+        <v>3</v>
+      </c>
+      <c r="H367" t="b">
+        <v>0</v>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198883487</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>1197910915</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>cocodrug</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>エリクシール　シュペリエル　デーケアレボリューション　トーンアップ　BE +ca　ピュアベージュ 日中用美容液 SPF50+PA++++　35g</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>資生堂</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
+      <c r="H368" t="b">
+        <v>0</v>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197910915</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>1194584634</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>cocodrug</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>エリクシール ブライトニング　ローション ca みずみずしいタイプ（つめかえ用）化粧水【医薬部外品】150ml</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>資生堂</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0</v>
+      </c>
+      <c r="H369" t="b">
+        <v>0</v>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194584634</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>1194584287</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>cocodrug</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>エリクシール ブライトニング　ローション ca みずみずしいタイプ 化粧水【医薬部外品】170ml</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>資生堂</t>
+        </is>
+      </c>
+      <c r="F370" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G370" t="n">
+        <v>0</v>
+      </c>
+      <c r="H370" t="b">
+        <v>0</v>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194584287</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J349"/>
+  <autoFilter ref="A1:J370"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 78, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$370</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$377</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J370"/>
+  <dimension ref="A1:J377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15625,8 +15625,295 @@
         </is>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>1138374893</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>香栄化学 エルカラ20 400ml レフィル 詰替用</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>香栄化学</t>
+        </is>
+      </c>
+      <c r="F371" t="n">
+        <v>3657</v>
+      </c>
+      <c r="G371" t="n">
+        <v>0</v>
+      </c>
+      <c r="H371" t="b">
+        <v>0</v>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138374893</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>1117338699</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>ブルガリ アクア プールオム EDT オードトワレ SP 30ml 香水 BVLGARI</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>ブルガリ</t>
+        </is>
+      </c>
+      <c r="F372" t="n">
+        <v>9631</v>
+      </c>
+      <c r="G372" t="n">
+        <v>1</v>
+      </c>
+      <c r="H372" t="b">
+        <v>0</v>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117338699</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>1117341863</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>メゾン マルジェラ レプリカ バブル バス EDT オードトワレ SP 10ml ミニ香水 MAISON MARGIELA</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F373" t="n">
+        <v>3821</v>
+      </c>
+      <c r="G373" t="n">
+        <v>0</v>
+      </c>
+      <c r="H373" t="b">
+        <v>0</v>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117341863</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>1183179464</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>ハー ロンドン ドリーム EDP SP 30ml</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Burberry</t>
+        </is>
+      </c>
+      <c r="F374" t="n">
+        <v>11198</v>
+      </c>
+      <c r="G374" t="n">
+        <v>0</v>
+      </c>
+      <c r="H374" t="b">
+        <v>0</v>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183179464</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>1065580984</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>グロウ バイジェイロー EDT SP 100ml</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>ジェニファーロペス</t>
+        </is>
+      </c>
+      <c r="F375" t="n">
+        <v>4373</v>
+      </c>
+      <c r="G375" t="n">
+        <v>0</v>
+      </c>
+      <c r="H375" t="b">
+        <v>0</v>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1065580984</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>1066844135</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>オードモワゼル フローラル EDT SP 100ml</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>GIVENCHY</t>
+        </is>
+      </c>
+      <c r="F376" t="n">
+        <v>12073</v>
+      </c>
+      <c r="G376" t="n">
+        <v>0</v>
+      </c>
+      <c r="H376" t="b">
+        <v>0</v>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1066844135</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>1183179421</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>ポロ レッド （チューブサンプル） EDT SP 1.2ml</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Ralph Lauren</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0</v>
+      </c>
+      <c r="H377" t="b">
+        <v>0</v>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183179421</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J370"/>
+  <autoFilter ref="A1:J377"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 81, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$377</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$394</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J377"/>
+  <dimension ref="A1:J394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15912,8 +15912,705 @@
         </is>
       </c>
     </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>1209235049</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>differNdeeper</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>【公式】メラチノール クラウドクリーム 50g /レチノール/メラニンケア/シミケア</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>DIFFER&amp;amp;DEEPER</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G378" t="n">
+        <v>2</v>
+      </c>
+      <c r="H378" t="b">
+        <v>0</v>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209235049</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>1210321053</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>differNdeeper</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>【公式】メラチノール クラウドクリーム 50g＋メラティノールアンプル(2ml*7ea) /レチノール/メラニンケア/シミケア</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>DIFFER&amp;amp;DEEPER</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0</v>
+      </c>
+      <c r="H379" t="b">
+        <v>0</v>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210321053</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>1209234684</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>differNdeeper</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>【公式】ピエルトラ ファーミングバンドリフター 50ml/リフティング/肌のキメ改善/コエンザイム/顔・首のたるみケア /弾力 /シワ・たるみ改善 / 真のVラインケア</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>DIFFER&amp;amp;DEEPER</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G380" t="n">
+        <v>1</v>
+      </c>
+      <c r="H380" t="b">
+        <v>0</v>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209234684</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>1206892952</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>veridel</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>[1+1] ウォーターグロウバリア TXショット 5000 美容液 30ml 2個</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>veridel</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>3888</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+      <c r="H381" t="b">
+        <v>0</v>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206892952</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>1190206306</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>SEOULTOMODACHI</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>コウジ酸ビタナイアシントナー, 250ml</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G382" t="n">
+        <v>1</v>
+      </c>
+      <c r="H382" t="b">
+        <v>0</v>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190206306</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>1201899328</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>SEOULTOMODACHI</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>ウォーターグロウバリア TXショット 5000 美容液 30ml</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>veridel</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G383" t="n">
+        <v>0</v>
+      </c>
+      <c r="H383" t="b">
+        <v>0</v>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201899328</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>1192657055</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>SEOULTOMODACHI</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>コウジ酸ビタゼリーセラムミスト, 100ml</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G384" t="n">
+        <v>0</v>
+      </c>
+      <c r="H384" t="b">
+        <v>0</v>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192657055</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>1200677289</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>JJCompany</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>グリコール酸7% トーニングソリューション 100ml 角質ケア 拭き取り化粧水 毛穴ケア 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>2302</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0</v>
+      </c>
+      <c r="H385" t="b">
+        <v>0</v>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200677289</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>1129908462</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>leelix</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>PHセンシティブ クリーム 60ml x 2個セット (チューブタイプ 高保湿 敏感肌)</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>9322</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0</v>
+      </c>
+      <c r="H386" t="b">
+        <v>0</v>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1129908462</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>1132004375</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>leelix</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>フルフィット プロポリス ライト アンプル 40ml +40ml</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>3996</v>
+      </c>
+      <c r="G387" t="n">
+        <v>1</v>
+      </c>
+      <c r="H387" t="b">
+        <v>0</v>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132004375</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>1203960088</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>345リリーフクリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F388" t="n">
+        <v>2453</v>
+      </c>
+      <c r="G388" t="n">
+        <v>0</v>
+      </c>
+      <c r="H388" t="b">
+        <v>0</v>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203960088</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>1192047927</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%トーニングソリューション 240ml トーニング ソリューション</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F389" t="n">
+        <v>2216</v>
+      </c>
+      <c r="G389" t="n">
+        <v>2</v>
+      </c>
+      <c r="H389" t="b">
+        <v>0</v>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192047927</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>1133764204</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>shintenchi</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>バイオコラーゲンリアルディープマスク, 4枚</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F390" t="n">
+        <v>2120</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0</v>
+      </c>
+      <c r="H390" t="b">
+        <v>0</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133764204</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>1207544119</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>shintenchi</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>エキスパートマデカクリームリニューPDRN, 50ml</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>2330</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0</v>
+      </c>
+      <c r="H391" t="b">
+        <v>0</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207544119</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>1118545938</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>ksco</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>センテラライトクレンジングオイル, 200ml</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0</v>
+      </c>
+      <c r="H392" t="b">
+        <v>0</v>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1118545938</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>1199379098</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>ksco</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>ゼリーセラムミスト, 50ml</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G393" t="n">
+        <v>0</v>
+      </c>
+      <c r="H393" t="b">
+        <v>0</v>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199379098</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>1163668247</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>ksco</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>シューマジゴールド糸ラッピングマスク, 90g</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>メディテラピー</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>5580</v>
+      </c>
+      <c r="G394" t="n">
+        <v>0</v>
+      </c>
+      <c r="H394" t="b">
+        <v>0</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163668247</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J377"/>
+  <autoFilter ref="A1:J394"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 84, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$394</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$403</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J394"/>
+  <dimension ref="A1:J403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16609,8 +16609,377 @@
         </is>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>1203203087</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>mrelephant</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>スキンケアパッド 4種 (各タイプ別)/シラカバ]潤い水分/セリ カミング鎮静/ユジャC トーンアップ(ブライトニング)/ザクロ ハリ弾力パーミング/</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>コアコス</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0</v>
+      </c>
+      <c r="H395" t="b">
+        <v>0</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203203087</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>1195547873</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>mrelephant</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>SOS メガ Mケア ソリューションアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>MOJELIM</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0</v>
+      </c>
+      <c r="H396" t="b">
+        <v>0</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195547873</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>1096353729</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>SM_Mall</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>コスパ 【公式/韓国正品】デリケートゾーンソープ／フォーム170ml 2種択一／かゆみ匂いケア／弱酸性／デリケートゾーンケア／フェミニンウォッシュ／爽やか／韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>アロマティカ</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0</v>
+      </c>
+      <c r="H397" t="b">
+        <v>0</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096353729</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>1159224305</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>シカフルアンプル30ml 1個</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>1894</v>
+      </c>
+      <c r="G398" t="n">
+        <v>1</v>
+      </c>
+      <c r="H398" t="b">
+        <v>0</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159224305</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>1149395148</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド 20% セラム80ml1個</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>2473</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0</v>
+      </c>
+      <c r="H399" t="b">
+        <v>0</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149395148</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>1200324318</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>ヒアルロン酸2% + B5 セラム 30ml 1個</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>2671</v>
+      </c>
+      <c r="G400" t="n">
+        <v>0</v>
+      </c>
+      <c r="H400" t="b">
+        <v>0</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200324318</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>1197354746</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>345 リリーフクリームミスト1個 100ml</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G401" t="n">
+        <v>0</v>
+      </c>
+      <c r="H401" t="b">
+        <v>0</v>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197354746</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>1206682479</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>cafebespoke</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>グリーンプロポリス 頭皮クレンジング シャンプー+トリートメント [1000ml+1000ml] セット</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G402" t="n">
+        <v>3</v>
+      </c>
+      <c r="H402" t="b">
+        <v>0</v>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206682479</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>1172777299</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>fmalwm</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>パフューム ヘアミスト サンセットフォグ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>ハクスリー</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>5833</v>
+      </c>
+      <c r="G403" t="n">
+        <v>0</v>
+      </c>
+      <c r="H403" t="b">
+        <v>0</v>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172777299</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J394"/>
+  <autoFilter ref="A1:J403"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 87, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$403</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$424</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J403"/>
+  <dimension ref="A1:J424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16978,8 +16978,869 @@
         </is>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>1148735293</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>k-worldshop</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>スタイリング アニメーター ウェット カールクリーム ボリュームヘア 男性 女性 150ml 1個</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>SAVWA PROFESSIONAL</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>4712</v>
+      </c>
+      <c r="G404" t="n">
+        <v>0</v>
+      </c>
+      <c r="H404" t="b">
+        <v>0</v>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148735293</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>1152577703</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>k-worldshop</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>レチノール 1% スクワラン30ml</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>2437</v>
+      </c>
+      <c r="G405" t="n">
+        <v>0</v>
+      </c>
+      <c r="H405" t="b">
+        <v>0</v>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152577703</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>1152513552</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>k-worldshop</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>スプリング ピンク トーンアップ サンクリーム SPF50+PA ++++ 50ml 1個 サンスクリーン 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>MODELO</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>3577</v>
+      </c>
+      <c r="G406" t="n">
+        <v>1</v>
+      </c>
+      <c r="H406" t="b">
+        <v>0</v>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152513552</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>1151287022</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>k-worldshop</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>シッピーワン ヘアプレミアム トリートメント 250ml 髪の栄養 頭皮 髪質</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>CP-1</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>2214</v>
+      </c>
+      <c r="G407" t="n">
+        <v>1</v>
+      </c>
+      <c r="H407" t="b">
+        <v>0</v>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151287022</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>1151033114</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>k-worldshop</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラ ヒアルー シカ 光彩 トナー 210ml</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0</v>
+      </c>
+      <c r="H408" t="b">
+        <v>0</v>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151033114</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>1199126524</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>ec-unicorn</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>トリファクス　シャンプー 500ml 詰め替え</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>SUNCALL</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0</v>
+      </c>
+      <c r="H409" t="b">
+        <v>0</v>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199126524</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>1167205791</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>ec-unicorn</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>【詰替セット】 ミントベル マリンブルー シャンプー 1900ml スパコンディショナー 700ml クールシャンプー ミントシャンプー 詰め替え 詰替え用 頭皮ケア サロン専売 美容室 夏</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>SUNCALL</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>10860</v>
+      </c>
+      <c r="G410" t="n">
+        <v>0</v>
+      </c>
+      <c r="H410" t="b">
+        <v>0</v>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167205791</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>1130492851</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>ec-unicorn</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>CA バンリッシュ クロマプロテクト BAINRICHE CHROMA RESPECT 1000ml シャンプー ポンプ付 ヘアシャンプー カラーケアシャンプー カラーケア 艶髪 業務用</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>ケラスターゼ</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>10450</v>
+      </c>
+      <c r="G411" t="n">
+        <v>0</v>
+      </c>
+      <c r="H411" t="b">
+        <v>0</v>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130492851</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>1202057079</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>dayz</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>ナ プラ ネント ボンドプレップミスト 200mL</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>ナプラ</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>2198</v>
+      </c>
+      <c r="G412" t="n">
+        <v>1</v>
+      </c>
+      <c r="H412" t="b">
+        <v>0</v>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202057079</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>1028383165</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>dayz</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>ミルボン オルディーブ カラー ベーシックトーン　フェミニティピンク 【　8-fPK　】　80g　6点セット</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>3810</v>
+      </c>
+      <c r="G413" t="n">
+        <v>0</v>
+      </c>
+      <c r="H413" t="b">
+        <v>0</v>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1028383165</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>482099707</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>dayz</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>ウ アオ べジミックス シリコン除去 シャンプー 1000mL 詰め替え用</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>ウアオ</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>2838</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0</v>
+      </c>
+      <c r="H414" t="b">
+        <v>0</v>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=482099707</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>1202057072</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>dayz</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>ナ プラ ネント ボンドプレップミスト 500mL 詰め替え用</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>ナプラ</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>2962</v>
+      </c>
+      <c r="G415" t="n">
+        <v>0</v>
+      </c>
+      <c r="H415" t="b">
+        <v>0</v>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202057072</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>1194168468</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>tokitomecosme</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>【国内正規品】オバジC 酵素洗顔パウダーDP 0.4g×30個 Obagi 毛穴ケア 洗顔料 個包装 ビタミンC 酵素 洗顔 角栓 黒ずみ ザラつき ロート製薬</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>オバジ</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>2862</v>
+      </c>
+      <c r="G416" t="n">
+        <v>0</v>
+      </c>
+      <c r="H416" t="b">
+        <v>0</v>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194168468</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>1209121752</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>【2本セット・2026年新発売・国内正規品】イドラクラリティ 薬用 ブライトニング エッセンス ウォーター 医薬部外品 200ml 美容液 化粧水 ローション エッセンス 潤い 保湿</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>コスメデコルテ</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>13902</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0</v>
+      </c>
+      <c r="H417" t="b">
+        <v>0</v>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209121752</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>1200341995</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>【国内正規品】コスメデコルテ AQ 毛穴美容液オイル 40mL クレンジング オイルクレンジング うるおい 美容液 クレンジング美容液 なめらかな肌 フェイスオイル スキンケア 美容液オイル</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>コスメデコルテ</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>10859</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0</v>
+      </c>
+      <c r="H418" t="b">
+        <v>0</v>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200341995</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>1160784536</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>MONNALI MIHATSU モナリ ミハツ カバートリートメント 200g ブラックシリーズ 黒いトリートメント ヘアケア エイジングケア スカルプケア メンズ レディース</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>MONNALI</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>3902</v>
+      </c>
+      <c r="G419" t="n">
+        <v>0</v>
+      </c>
+      <c r="H419" t="b">
+        <v>0</v>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160784536</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>1160784512</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>【2点セット】MONNALI MIHATSU モナリ ミハツ クレンジングシャンプー 350ml+トリートメント 200g+ ブラックシリーズ 黒いシャンプー ヘアケア エイジ</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>MONNALI</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>9295</v>
+      </c>
+      <c r="G420" t="n">
+        <v>0</v>
+      </c>
+      <c r="H420" t="b">
+        <v>0</v>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160784512</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>1145827664</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>c-urbanqoo10</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>オリリー サロンプロフェッショナル ハンドケア 100g 国内正規品</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>オリリー</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>2502</v>
+      </c>
+      <c r="G421" t="n">
+        <v>1</v>
+      </c>
+      <c r="H421" t="b">
+        <v>0</v>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145827664</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>1147314397</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>c-urbanqoo10</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>シーボン ブライトベール UV プロテクター 40g 国内正規品</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>C'BON</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>6003</v>
+      </c>
+      <c r="G422" t="n">
+        <v>0</v>
+      </c>
+      <c r="H422" t="b">
+        <v>0</v>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147314397</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>1208715918</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>c-urbanqoo10</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>セインムー ボーテロンド シェルル バスト ハリ デコルテ ボディケア美容液 100ml</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>seins mous</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>65253</v>
+      </c>
+      <c r="G423" t="n">
+        <v>0</v>
+      </c>
+      <c r="H423" t="b">
+        <v>0</v>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208715918</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>1205361632</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>c-urbanqoo10</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>ラダメール オリゴフォースセラムハイドレーティン 美容液 韓国コスメ 50ml</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>LADAMER</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>8748</v>
+      </c>
+      <c r="G424" t="n">
+        <v>1</v>
+      </c>
+      <c r="H424" t="b">
+        <v>0</v>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205361632</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J403"/>
+  <autoFilter ref="A1:J424"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 90, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$424</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$433</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J424"/>
+  <dimension ref="A1:J433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17839,8 +17839,377 @@
         </is>
       </c>
     </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>1163571137</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>K-BEAUTYBOX</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>グッセラスーパーセラミドクリーム 60ml 2個 高保湿クリームナイトケア</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>ホリカホリカ</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>4584</v>
+      </c>
+      <c r="G425" t="n">
+        <v>0</v>
+      </c>
+      <c r="H425" t="b">
+        <v>0</v>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163571137</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>1196415617</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>【WiD2】 AHA・BHA配合 28デイズヒアルクリーム (30ml) ザラつきOFF！なめらか透明肌へ 1個</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G426" t="n">
+        <v>1</v>
+      </c>
+      <c r="H426" t="b">
+        <v>0</v>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196415617</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>1196366572</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>【WiD2】 ガラクトナイアシンエッセンスマスク 10枚入り 肌をクリアに・高保湿・エイジングケア</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>2851</v>
+      </c>
+      <c r="G427" t="n">
+        <v>0</v>
+      </c>
+      <c r="H427" t="b">
+        <v>0</v>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196366572</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>1193786879</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>chaudmaison</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>AESTURA 公式 エストラ エイシカ365クイックマスクパッド 60枚 トナーパッド パック</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G428" t="n">
+        <v>0</v>
+      </c>
+      <c r="H428" t="b">
+        <v>0</v>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193786879</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>1193635878</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>chaudmaison</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>AMPLE:N 公式 アンプルエヌ ペプチドショット アンプル 2X 100ml ペプチドショット 2X アンプルn 美容液</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G429" t="n">
+        <v>2</v>
+      </c>
+      <c r="H429" t="b">
+        <v>0</v>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193635878</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>1193841835</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Oliveofficial</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Celimax 公式 セリマックス レチナール タイトニング ブースター 15ml+15ml THE ビタA レチノールショット タイトニングブースター</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>7990</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0</v>
+      </c>
+      <c r="H430" t="b">
+        <v>0</v>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193841835</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>1193633283</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>REALBEAUTYSHOP</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>BRING GREEN 公式 ブリングリーン ティーツリーシカディープ洗顔フォーム 120ml+120ml BRINGGREEN 洗顔 クレンジング</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G431" t="n">
+        <v>1</v>
+      </c>
+      <c r="H431" t="b">
+        <v>0</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193633283</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>1193632664</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>REALBEAUTYSHOP</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>BRING GREEN 公式 ブリングリーン ティーツリーＣ トナー 500ml BRINGGREEN 化粧水</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G432" t="n">
+        <v>0</v>
+      </c>
+      <c r="H432" t="b">
+        <v>0</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193632664</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>1193632481</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>REALBEAUTYSHOP</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>BRING GREEN 公式 ブリングリーン ティーツリーシカセンシティブクレンジングウォーター 500ml BRINGGREEN 洗顔 クレンジング</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G433" t="n">
+        <v>1</v>
+      </c>
+      <c r="H433" t="b">
+        <v>0</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193632481</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J424"/>
+  <autoFilter ref="A1:J433"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 93, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$433</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$443</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J433"/>
+  <dimension ref="A1:J443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18208,8 +18208,418 @@
         </is>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>1193439473</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>watiforskin</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>【選べる12タイプ】マイクロスピキュール＆ボルプロショットクリーム 50ml/グリコール酸・ナイアシンアミド・レチノール・バクチオル・トラネキサム酸・ヒアルロン酸・PDRN配合</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Wati For Skin</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G434" t="n">
+        <v>1</v>
+      </c>
+      <c r="H434" t="b">
+        <v>0</v>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193439473</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>1193438313</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>watiforskin</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>【選べる導入美容液】マイクロショット100 美容液 30ml 12種/微細針 肌トラブル管理ソリューション / 韓国化粧品/リドルショットコンセプト</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Wati For Skin</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G435" t="n">
+        <v>3</v>
+      </c>
+      <c r="H435" t="b">
+        <v>0</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193438313</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>1149907926</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>sssemibeauty</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>ブラックシュガーパーフェクトファーストセラム 150ml</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>2299</v>
+      </c>
+      <c r="G436" t="n">
+        <v>0</v>
+      </c>
+      <c r="H436" t="b">
+        <v>0</v>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149907926</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>1172085888</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>sssemibeauty</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>フルフィットプロポリスライトアンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>2337</v>
+      </c>
+      <c r="G437" t="n">
+        <v>0</v>
+      </c>
+      <c r="H437" t="b">
+        <v>0</v>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172085888</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>1117324982</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>西洋プラムピンクグルタチオンデイリースペシャルマスク 30枚入 1個</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>5075</v>
+      </c>
+      <c r="G438" t="n">
+        <v>0</v>
+      </c>
+      <c r="H438" t="b">
+        <v>0</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117324982</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>1207285368</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>アルガンエッセンシャルディープケアヘアパック大容量470ml 1個</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>2660</v>
+      </c>
+      <c r="G439" t="n">
+        <v>0</v>
+      </c>
+      <c r="H439" t="b">
+        <v>0</v>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207285368</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>1201631207</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>ルートジェン脱毛症状専門ケア頭皮エッセンス80ml 2個</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>呂</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>3755</v>
+      </c>
+      <c r="G440" t="n">
+        <v>0</v>
+      </c>
+      <c r="H440" t="b">
+        <v>0</v>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201631207</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>1164356074</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>goldstarstore</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>アドベンスドスネイル92オールインワンチューブ型クリーム100g 1個</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>3440</v>
+      </c>
+      <c r="G441" t="n">
+        <v>0</v>
+      </c>
+      <c r="H441" t="b">
+        <v>0</v>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164356074</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>1191102778</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>mamamall</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>インテカスージングクリーム, 31ml</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>メイクプレム</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G442" t="n">
+        <v>2</v>
+      </c>
+      <c r="H442" t="b">
+        <v>0</v>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191102778</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>1138105738</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>mamamall</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>ハイポアラジェニックLHA CIS ジェルクレンザー　200ml</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>molvany</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>4150</v>
+      </c>
+      <c r="G443" t="n">
+        <v>2</v>
+      </c>
+      <c r="H443" t="b">
+        <v>0</v>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138105738</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J433"/>
+  <autoFilter ref="A1:J443"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 96, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$443</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$460</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J443"/>
+  <dimension ref="A1:J460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18618,8 +18618,705 @@
         </is>
       </c>
     </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>1203205247</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>vanguardvista</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>[正規品] 人気 おすすめ 韓国 クリーム Rx 30ml+7ml セット スキンケア クリーム ギフト</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>ドミナス</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>5820</v>
+      </c>
+      <c r="G444" t="n">
+        <v>0</v>
+      </c>
+      <c r="H444" t="b">
+        <v>0</v>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203205247</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>1176812478</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>meisonmatcha</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>[2個]トータルリペア5 ミラクル ヘアパック 170ml</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>1626</v>
+      </c>
+      <c r="G445" t="n">
+        <v>0</v>
+      </c>
+      <c r="H445" t="b">
+        <v>0</v>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176812478</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>1172106877</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>ジークップ ケアセラ エコアスノウ 硫黄石鹸 (4個入)</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>ケアセラ</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>3710</v>
+      </c>
+      <c r="G446" t="n">
+        <v>0</v>
+      </c>
+      <c r="H446" t="b">
+        <v>0</v>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172106877</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>1169173710</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>ニューヨーク インティリー オードパルファムEDP 10ml</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>7780</v>
+      </c>
+      <c r="G447" t="n">
+        <v>0</v>
+      </c>
+      <c r="H447" t="b">
+        <v>0</v>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169173710</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>1169173462</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>ローストウッド オードパルファムEDP 10ml</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F448" t="n">
+        <v>7780</v>
+      </c>
+      <c r="G448" t="n">
+        <v>0</v>
+      </c>
+      <c r="H448" t="b">
+        <v>0</v>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169173462</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>1181384570</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>KOREAMALL1</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>[ギャラリア] MADET LEN レッドムスク オードパルファム RED MUSC</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>MAD et LEN</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>63970</v>
+      </c>
+      <c r="G449" t="n">
+        <v>0</v>
+      </c>
+      <c r="H449" t="b">
+        <v>0</v>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181384570</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>1191434560</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>chibashop</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>ハイプライム コラーゲン フィルムマスクパック 5枚</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>DERMARSSANCE</t>
+        </is>
+      </c>
+      <c r="F450" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G450" t="n">
+        <v>0</v>
+      </c>
+      <c r="H450" t="b">
+        <v>0</v>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191434560</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1115552034</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>[1+1] [SNS, AMAZON 大人気] 米サンクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>3558</v>
+      </c>
+      <c r="G451" t="n">
+        <v>0</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115552034</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>1193643194</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>【正規品】【Qoo10人気】レチノールリペアセラム30ml ヴィーガンリポソームレチノール3%セラム</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>スキンアンドラブ</t>
+        </is>
+      </c>
+      <c r="F452" t="n">
+        <v>4736</v>
+      </c>
+      <c r="G452" t="n">
+        <v>0</v>
+      </c>
+      <c r="H452" t="b">
+        <v>0</v>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193643194</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>1193643034</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>【正規品】コラーゲンナイトラッピングマスク 75ml + ブラシ</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>メディキューブバイオ</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G453" t="n">
+        <v>0</v>
+      </c>
+      <c r="H453" t="b">
+        <v>0</v>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193643034</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>1193642954</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>【正規品】[ライスシリーズ] 7 ライス セラミド グローセラム /ライス 70 インテンス モイスチャー ミルク /ライス ブライトニング酵素洗顔パウダー /ライス70 グロウミルキートナー</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F454" t="n">
+        <v>4516</v>
+      </c>
+      <c r="G454" t="n">
+        <v>0</v>
+      </c>
+      <c r="H454" t="b">
+        <v>0</v>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193642954</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>1193642948</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>KCOS1</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>GIVENCY 【正規品】 プリズム リーブル ミニパウダー No0/No1/No2/No3/No4 ジバンシイ プリズム リーブル PRISME LIBRE ルース パウダー</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>7570</v>
+      </c>
+      <c r="G455" t="n">
+        <v>0</v>
+      </c>
+      <c r="H455" t="b">
+        <v>0</v>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193642948</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>1202152284</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Probioderm Collagen Remodeling Booster Shot Program 35ml</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F456" t="n">
+        <v>3360</v>
+      </c>
+      <c r="G456" t="n">
+        <v>0</v>
+      </c>
+      <c r="H456" t="b">
+        <v>0</v>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202152284</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>1202519032</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>[Glory exclusive]AZ Care Cleansing Oil, 200mL</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G457" t="n">
+        <v>0</v>
+      </c>
+      <c r="H457" t="b">
+        <v>0</v>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202519032</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>1202165457</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>[RYO] Root Gen Hair Loss Care Scalp Essence, 80mL</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>No Brand</t>
+        </is>
+      </c>
+      <c r="F458" t="n">
+        <v>2040</v>
+      </c>
+      <c r="G458" t="n">
+        <v>0</v>
+      </c>
+      <c r="H458" t="b">
+        <v>0</v>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202165457</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>1047570493</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>SJOCEAN</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>[1+1] リアル ヒアルロニック 100 クリーム 80ml+80ml / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>WELLAGE</t>
+        </is>
+      </c>
+      <c r="F459" t="n">
+        <v>5040</v>
+      </c>
+      <c r="G459" t="n">
+        <v>0</v>
+      </c>
+      <c r="H459" t="b">
+        <v>0</v>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1047570493</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>1181192539</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>thetebah</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>[TONYMOLY トニーモリー] ワンダーセラミドモチトナー / Wonder Ceramide Mochi Toner - 500ml / エイジングケア / 低刺激 / もちもち#エイジン</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F460" t="n">
+        <v>2417</v>
+      </c>
+      <c r="G460" t="n">
+        <v>0</v>
+      </c>
+      <c r="H460" t="b">
+        <v>0</v>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181192539</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J443"/>
+  <autoFilter ref="A1:J460"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 99, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$460</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$475</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J460"/>
+  <dimension ref="A1:J475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19315,8 +19315,623 @@
         </is>
       </c>
     </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>1040290899</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>felisamall</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>[GRANHAND]【1+1】 ハンドクリーム60g　3種 SUSIE SALMON</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>GRANHAND</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>8150</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0</v>
+      </c>
+      <c r="H461" t="b">
+        <v>0</v>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1040290899</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>1208658337</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>[Tamburins] SUMMER TAILS ディスカバリーセット</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0</v>
+      </c>
+      <c r="H462" t="b">
+        <v>0</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208658337</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>1203988364</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>[大容量] オービタミネボディミルク 400ml</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>ビオテルム</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>6250</v>
+      </c>
+      <c r="G463" t="n">
+        <v>0</v>
+      </c>
+      <c r="H463" t="b">
+        <v>0</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203988364</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>1193624609</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>TXT愛用 BOMBSHELLUTH バムシェル 10ml Oil Perfumeオイル香水</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>DANIELS TRUTH</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>6550</v>
+      </c>
+      <c r="G464" t="n">
+        <v>3</v>
+      </c>
+      <c r="H464" t="b">
+        <v>0</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193624609</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>1189436342</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>VT リードルショット ユニバース キット 2ml × 5本 x 9種（全45本）正規品 韓国化粧品 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F465" t="n">
+        <v>3250</v>
+      </c>
+      <c r="G465" t="n">
+        <v>3</v>
+      </c>
+      <c r="H465" t="b">
+        <v>0</v>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189436342</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>1208892070</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>W-NY</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>moumou(ムームー)オードパルファン(香水)リネン(透き通るような爽やかな香り)10ml</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>mou mou</t>
+        </is>
+      </c>
+      <c r="F466" t="n">
+        <v>2620</v>
+      </c>
+      <c r="G466" t="n">
+        <v>0</v>
+      </c>
+      <c r="H466" t="b">
+        <v>0</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208892070</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>1213426114</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>bodiance</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>シルキーベルベット ブライトブースティング ボディウォッシュ 750ml / 色素沈着ケア / ツヤ肌 / 弱酸性 /トーンケア</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Bodiance</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G467" t="n">
+        <v>0</v>
+      </c>
+      <c r="H467" t="b">
+        <v>0</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213426114</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>1205520797</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>ポアコントロール131 クレンジングオイル200ml／毛穴ケア／皮脂バランス</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F468" t="n">
+        <v>3153</v>
+      </c>
+      <c r="G468" t="n">
+        <v>0</v>
+      </c>
+      <c r="H468" t="b">
+        <v>0</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205520797</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>1204558349</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>リポソームバブルブースター 95ml 2種（コラーゲン／キャビア PDRN）から1つ選択</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>3498</v>
+      </c>
+      <c r="G469" t="n">
+        <v>0</v>
+      </c>
+      <c r="H469" t="b">
+        <v>0</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204558349</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>1190357115</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>アゼライン酸CICAスキンクリアトナー 250ml</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F470" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G470" t="n">
+        <v>0</v>
+      </c>
+      <c r="H470" t="b">
+        <v>0</v>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190357115</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>1157789377</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>ドクダミLHAモイスチャーピーリングジェル 120ml</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G471" t="n">
+        <v>0</v>
+      </c>
+      <c r="H471" t="b">
+        <v>0</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157789377</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>1211655439</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>cosmeparfaite</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>コンフォート ストレッチィ ウォッシュII 55g 宅配便</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>カネボウ</t>
+        </is>
+      </c>
+      <c r="F472" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G472" t="n">
+        <v>0</v>
+      </c>
+      <c r="H472" t="b">
+        <v>0</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211655439</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>1211655440</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>cosmeparfaite</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>インスタント オフ オイル リミテッド サイズ 310ml 宅配便</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>カネボウ</t>
+        </is>
+      </c>
+      <c r="F473" t="n">
+        <v>6180</v>
+      </c>
+      <c r="G473" t="n">
+        <v>0</v>
+      </c>
+      <c r="H473" t="b">
+        <v>0</v>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211655440</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>1205052684</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>MOMOCHI_SHOP</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>【毛穴洗顔】 ゼロ毛穴 クレンジングフォーム 120g サリチル酸 BHA洗顔 カプセル洗顔 韓国洗顔 毛穴ケア 皮脂ケア フォーム洗顔 韓国スキンケア 角質ケア 毛穴汚れ 韓国コスメ デイリー洗顔</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F474" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G474" t="n">
+        <v>0</v>
+      </c>
+      <c r="H474" t="b">
+        <v>0</v>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205052684</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>1212968157</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>MOMOCHI_SHOP</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>【目元ハリケア】 アイファルト アイバック クリーム 10ml 目元たるみ アイクリーム 保湿 レチノール EGF ナイアシンアミド セラミド 目元ケア 乾燥小じわ 韓国コスメ くまケア</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F475" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G475" t="n">
+        <v>0</v>
+      </c>
+      <c r="H475" t="b">
+        <v>0</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212968157</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J460"/>
+  <autoFilter ref="A1:J475"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 102, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$475</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$481</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J475"/>
+  <dimension ref="A1:J481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19930,8 +19930,254 @@
         </is>
       </c>
     </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>1112935346</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>【選べる2個セット】デビルズ パフュームファンタジーシャンプー &amp;amp; コンディショナー, 1L+1L</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F476" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G476" t="n">
+        <v>1</v>
+      </c>
+      <c r="H476" t="b">
+        <v>0</v>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1112935346</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>1084157476</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>【NEW COLOR】イージーブロウトーンチェンジャー (5回分) /ブリーチ / 眉毛脱色 /眉カラーケア</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>サムバイミー</t>
+        </is>
+      </c>
+      <c r="F477" t="n">
+        <v>4110</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0</v>
+      </c>
+      <c r="H477" t="b">
+        <v>0</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1084157476</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>1191967561</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>lucylucy</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>【knock,】メルトイン ボディトナー 300ml 4種の香り / ボディミスト ボディローション ボディケア</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>ノック</t>
+        </is>
+      </c>
+      <c r="F478" t="n">
+        <v>5150</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0</v>
+      </c>
+      <c r="H478" t="b">
+        <v>0</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191967561</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>1107510664</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>KSB</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>[新作]ムード レイヤー スティック クレヨン 5color 00 milky syrup 01 caramel drizzle 02 rose milk tea 03 mauve latte</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>alternative stereo</t>
+        </is>
+      </c>
+      <c r="F479" t="n">
+        <v>2405</v>
+      </c>
+      <c r="G479" t="n">
+        <v>1</v>
+      </c>
+      <c r="H479" t="b">
+        <v>0</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107510664</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>1205514714</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Nandak</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>[ダーママスク10枚プレゼント] マデカクリームハイドラカーミング50ml3個韓国人気化粧品</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F480" t="n">
+        <v>5850</v>
+      </c>
+      <c r="G480" t="n">
+        <v>1</v>
+      </c>
+      <c r="H480" t="b">
+        <v>0</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205514714</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>1213367912</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>spklbzr</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>ルベル イオ クリーム メルトリペア ヘアトリートメント 200g 赤 684</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>イオ</t>
+        </is>
+      </c>
+      <c r="F481" t="n">
+        <v>1755</v>
+      </c>
+      <c r="G481" t="n">
+        <v>0</v>
+      </c>
+      <c r="H481" t="b">
+        <v>0</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213367912</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J475"/>
+  <autoFilter ref="A1:J481"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 105, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$481</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$491</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J481"/>
+  <dimension ref="A1:J491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20176,8 +20176,418 @@
         </is>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>1213540776</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>little_healing</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>RIMMEL(リンメル) ザ マルチタスカー コンシーラー 030 ライト標準 10ml</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>リンメルロンドン</t>
+        </is>
+      </c>
+      <c r="F482" t="n">
+        <v>1860</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0</v>
+      </c>
+      <c r="H482" t="b">
+        <v>0</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213540776</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>1204153918</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>little_healing</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>CAC ベースローション</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>CAC</t>
+        </is>
+      </c>
+      <c r="F483" t="n">
+        <v>3221</v>
+      </c>
+      <c r="G483" t="n">
+        <v>0</v>
+      </c>
+      <c r="H483" t="b">
+        <v>0</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204153918</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>1210874306</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>City45</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Mマーク M-mark アミノ酸角質層まで水 詰替用</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Ｍマーク</t>
+        </is>
+      </c>
+      <c r="F484" t="n">
+        <v>2146</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0</v>
+      </c>
+      <c r="H484" t="b">
+        <v>0</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210874306</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>1210872337</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>City45</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>デラクシオ イプル サボタージュ マルチオイルスプレー 100ml</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>千代田化学</t>
+        </is>
+      </c>
+      <c r="F485" t="n">
+        <v>2224</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0</v>
+      </c>
+      <c r="H485" t="b">
+        <v>0</v>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210872337</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>1210871481</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>City45</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>肌をうるおす保湿スキンケア 肌をうるおす保湿角質層まで水モイストリッチ 詰替用</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>肌をうるおす保湿スキンケア</t>
+        </is>
+      </c>
+      <c r="F486" t="n">
+        <v>2052</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0</v>
+      </c>
+      <c r="H486" t="b">
+        <v>0</v>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210871481</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>1158335117</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>ma-t-ma-to</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>ケアセラ(CareCera) APフェイス&amp;amp;ボディクリーム 70g (セラミドプラス×7種の天然型セラミド配合)</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>ケアセラ</t>
+        </is>
+      </c>
+      <c r="F487" t="n">
+        <v>1837</v>
+      </c>
+      <c r="G487" t="n">
+        <v>2</v>
+      </c>
+      <c r="H487" t="b">
+        <v>0</v>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158335117</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>1207003649</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>raughbright</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>洗顔パスタ ホワイトダイヤ 単品 90g</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>ロゼット</t>
+        </is>
+      </c>
+      <c r="F488" t="n">
+        <v>1814</v>
+      </c>
+      <c r="G488" t="n">
+        <v>1</v>
+      </c>
+      <c r="H488" t="b">
+        <v>0</v>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207003649</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>1199581764</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>lovemck1127</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>鎮静保湿セット 人気 ドクダミ77トナー＋セラミド美容液 ニキビ 毛穴 敏感肌 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F489" t="n">
+        <v>5510</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0</v>
+      </c>
+      <c r="H489" t="b">
+        <v>0</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199581764</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>1166880899</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>lovemck1127</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>エアリー密着シートマスク ティーツリー, 1個入り, 20個</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F490" t="n">
+        <v>1740</v>
+      </c>
+      <c r="G490" t="n">
+        <v>1</v>
+      </c>
+      <c r="H490" t="b">
+        <v>0</v>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166880899</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>977992270</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>farfallarossa</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>パナソニック リフトケア 美顔器 バイタリフト かっさ 温感 デュアルダイナミックEMS搭載 防水</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>パナソニック</t>
+        </is>
+      </c>
+      <c r="F491" t="n">
+        <v>33208</v>
+      </c>
+      <c r="G491" t="n">
+        <v>1</v>
+      </c>
+      <c r="H491" t="b">
+        <v>0</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=977992270</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J481"/>
+  <autoFilter ref="A1:J491"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 108, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$491</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J491"/>
+  <dimension ref="A1:J501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20586,8 +20586,418 @@
         </is>
       </c>
     </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>1167189098</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>GEPSTORE</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>韓国 ブラックスネイル コラーゲン ツーミスト セラム 100ml 3+3</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F492" t="n">
+        <v>11880</v>
+      </c>
+      <c r="G492" t="n">
+        <v>0</v>
+      </c>
+      <c r="H492" t="b">
+        <v>0</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167189098</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>1163541573</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>GEPSTORE</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>アノーブ グロウ ボディローション 290ml×2 ヌーバニラ 韓国ビューティー ボディケア</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F493" t="n">
+        <v>6780</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0</v>
+      </c>
+      <c r="H493" t="b">
+        <v>0</v>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163541573</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>1106037437</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>GEPSTORE</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>ルシード エル ハイダメージ リペア ヘアオイル 90ml 髪質復元</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>ルシージェー</t>
+        </is>
+      </c>
+      <c r="F494" t="n">
+        <v>1835</v>
+      </c>
+      <c r="G494" t="n">
+        <v>0</v>
+      </c>
+      <c r="H494" t="b">
+        <v>0</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106037437</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>1213547055</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>トリプルシールド ハイドロロック サンセラム SPF50+ PA++++ 50ml</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Forencos</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G495" t="n">
+        <v>0</v>
+      </c>
+      <c r="H495" t="b">
+        <v>0</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213547055</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>1212836013</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>スキン パーフェクティング BHA リキッド エクスフォリエント 118ml + 30ml / 角質ケア 毛穴ケア ピーリング 低刺激 スキンケア</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>ポーラチョイス</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0</v>
+      </c>
+      <c r="H496" t="b">
+        <v>0</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212836013</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>1211205774</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>マルチペプチドトナー 50ml x 5個 / 肌保湿 / 保湿充填</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>ルネセル</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0</v>
+      </c>
+      <c r="H497" t="b">
+        <v>0</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211205774</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>1183054314</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>jkmtr-jp</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Round Lab（ラウンドラボ）1025 ドクド クリーム 80ml ― 5種セラミドで内側まで満たす鎮静×保湿クリーム</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0</v>
+      </c>
+      <c r="H498" t="b">
+        <v>0</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183054314</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>1156238215</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>jkmtr-jp</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>[正規品/ 公式] ブッシュマン ウォータープルーフ プロ 日焼け止め 50g SPF50+ PA++++ 1個</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0</v>
+      </c>
+      <c r="H499" t="b">
+        <v>0</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156238215</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>1137010633</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>daewonar</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>サロン10 プロフェッショナル シカ セラミド オイル セラム 60ml+25ml×1 しっとり髪 Kビューティー ヘアケア</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F500" t="n">
+        <v>3350</v>
+      </c>
+      <c r="G500" t="n">
+        <v>1</v>
+      </c>
+      <c r="H500" t="b">
+        <v>0</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137010633</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>1118245002</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>daewonar</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>エアリーフィ ット サンスティック 14g Airy fit Sun Stick SPF 50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F501" t="n">
+        <v>2985</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0</v>
+      </c>
+      <c r="H501" t="b">
+        <v>0</v>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1118245002</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J491"/>
+  <autoFilter ref="A1:J501"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 1, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$327</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$342</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J327"/>
+  <dimension ref="A1:J342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13862,8 +13862,623 @@
         </is>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>1194192866</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>charmbeauty</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>アンダーヘアカッター30　(ミオ)　UH-30 安心の日本製 ムダ毛 ケア デリケートゾーン</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>グリーンベル</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>1138</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0</v>
+      </c>
+      <c r="H328" t="b">
+        <v>0</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194192866</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>1089142571</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>plantz</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>日本製 こども ダイヤルヘアカッター 赤ちゃん ベビー 乳幼児 スキハサミ ヘアカット クシ付き BA-112 安全 セルフ ベビー用品 散髪 前髪 子供 子ども</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>グリーンベル</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>1180</v>
+      </c>
+      <c r="G329" t="n">
+        <v>4</v>
+      </c>
+      <c r="H329" t="b">
+        <v>0</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089142571</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>1207222259</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>NUSE</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>【7/1 NEW】 リジュトーニングサンクッション 全5色</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>nuse</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G330" t="n">
+        <v>7</v>
+      </c>
+      <c r="H330" t="b">
+        <v>0</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207222259</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>1204196688</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>esthenojikan</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>アウトレット（旧パッケージ品）Tant RUX SOAP タントリュクス ソープ 200ml デリケートゾーン 洗浄料 フェムケア フェムテック / 即日発送 T001</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>タントリュクス</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>3025</v>
+      </c>
+      <c r="G331" t="n">
+        <v>0</v>
+      </c>
+      <c r="H331" t="b">
+        <v>0</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204196688</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>1153550013</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>refilled</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>【公式】 リフィルド サイトカインヘッドスパ＆リペアトリートメント 200ml/ダメージケア/ノンシリコン/潤い/ヘアトリートメント</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Refilled</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G332" t="n">
+        <v>5</v>
+      </c>
+      <c r="H332" t="b">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1153550013</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>1197369444</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>refilled</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>【公式】 リフィルド 頭皮カッサ/小顔/マッサージ/むくみケア</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Refilled</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="b">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197369444</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>1161577709</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>refilled</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>【公式】 リフィルド ヘアリカバリーサイトカインエフェクター/サイトカイン10倍/高濃度/持ち歩き/手軽育毛ケア</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Refilled</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>2590</v>
+      </c>
+      <c r="G334" t="n">
+        <v>15</v>
+      </c>
+      <c r="H334" t="b">
+        <v>0</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161577709</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>1100332949</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>balifesta</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>サンスクリーン Daily Refreshing Serum SPF50+ PA++++ 170ml 海外直送品</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
+      <c r="H335" t="b">
+        <v>0</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1100332949</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>1208319671</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>balifesta</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Mugwort　Acne Clay Stick　40g</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>SKINTIFIC</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
+      <c r="H336" t="b">
+        <v>0</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208319671</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>1208182736</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>balifesta</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>PDRN シリーズ　Radiance Bright Serum Spray　100ml</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>SKINTIFIC</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>5590</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0</v>
+      </c>
+      <c r="H337" t="b">
+        <v>0</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208182736</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>1172883577</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>CHEERYCHERRY</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>水分シートマスク_製品10個</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>1620</v>
+      </c>
+      <c r="G338" t="n">
+        <v>1</v>
+      </c>
+      <c r="H338" t="b">
+        <v>0</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172883577</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>1172728510</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>CHEERYCHERRY</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>保湿シートマスク_製品10個</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>1620</v>
+      </c>
+      <c r="G339" t="n">
+        <v>6</v>
+      </c>
+      <c r="H339" t="b">
+        <v>0</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172728510</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>1212303365</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>UUPPDQ10</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>ハイドロコロイド ロール 多用途 自由裁断 5cmx3.6m 5cmx1.5m 汚染を防止 摩擦を軽減 防水 通気性のある快適さ 滑り止め 肌を守る 靴ずれ防止 肌に優しい</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>ELAIMEI</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>1530</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
+      <c r="H340" t="b">
+        <v>0</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212303365</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>1103482828</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>SEVENPM</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>ターンアップ除毛クリーム 0.15マイクロブラシ</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>セブンピーエム</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>1995</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0</v>
+      </c>
+      <c r="H341" t="b">
+        <v>0</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1103482828</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>1179365922</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Cellology</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>色素沈着 メリタンアンプル2.0 30ml シミ シミケア 黒ずみ アンプル 美容液</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>セルオロジー</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>2930</v>
+      </c>
+      <c r="G342" t="n">
+        <v>5</v>
+      </c>
+      <c r="H342" t="b">
+        <v>0</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179365922</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J327"/>
+  <autoFilter ref="A1:J342"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 2, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$342</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$350</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J342"/>
+  <dimension ref="A1:J350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14477,8 +14477,336 @@
         </is>
       </c>
     </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>1206757124</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>soofee_jp</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>【公式】 ボタニカル リリーフ 化粧水＋乳液</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>スぺ</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
+      <c r="H343" t="b">
+        <v>0</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206757124</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>1116576489</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>bs-cosme</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>洗顔 アミノ洗顔料・100mL ヒト型 セラミド 配合 保湿 アスタキサンチン アミノ酸 ニキビ</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>BS-COSME</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>1030</v>
+      </c>
+      <c r="G344" t="n">
+        <v>7</v>
+      </c>
+      <c r="H344" t="b">
+        <v>0</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116576489</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>1116576447</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>bs-cosme</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>美容水 GG グリシルグリシン 5％ 溶液・30mL / 導入美容液 高配合 さっぱり 化粧水 グリセリンフリー</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>BS-COSME</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>790</v>
+      </c>
+      <c r="G345" t="n">
+        <v>15</v>
+      </c>
+      <c r="H345" t="b">
+        <v>0</v>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116576447</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>1116576508</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>bs-cosme</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>ビタミンE誘導体2点セットビタミンE溶液・30mL+エッセンスBK・30mL</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>BS-COSME</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G346" t="n">
+        <v>0</v>
+      </c>
+      <c r="H346" t="b">
+        <v>0</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116576508</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>1154723100</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>infodplus</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>エグゼスピ316日焼け止めクリーム</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>INFODPLUS</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G347" t="n">
+        <v>11</v>
+      </c>
+      <c r="H347" t="b">
+        <v>0</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154723100</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1176950870</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>withyoumarket</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Cleansing Device 2 デバイス2 デバイス 振動 クレンザー 肌マッサージ器 電動 クレンザー 顔マッサージ器具 皮脂除去器</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>EGG</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>18900</v>
+      </c>
+      <c r="G348" t="n">
+        <v>4</v>
+      </c>
+      <c r="H348" t="b">
+        <v>0</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176950870</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>1191309783</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>withyoumarket</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>[Event] mask pack (一枚パック計4枚) 水のいらない モデリングパック 水分補給/ 毛穴縮小/ しわ改善/ 肌の弾力/ 保湿ケア</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>VISUAL ADE</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>990</v>
+      </c>
+      <c r="G349" t="n">
+        <v>1</v>
+      </c>
+      <c r="H349" t="b">
+        <v>0</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191309783</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>1172537458</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>farmic</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>アップルタチオン トーニング トナーパッド ダブルセット 60枚(160ml) /グルタチオン配合/毛穴ケア/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>farmic</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G350" t="n">
+        <v>1</v>
+      </c>
+      <c r="H350" t="b">
+        <v>0</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172537458</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J342"/>
+  <autoFilter ref="A1:J350"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 7, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$394</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$395</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J394"/>
+  <dimension ref="A1:J395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16609,8 +16609,49 @@
         </is>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>1204653366</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>KLumion</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>【3本セット】 熱ダメージから髪を守る ヒーティングガード ノーウォッシュ トリートメント 147ml 3個 洗い流さないトリートメント ヘアケア 栄養 タンパク質 まとめ買い</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>3416</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0</v>
+      </c>
+      <c r="H395" t="b">
+        <v>0</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204653366</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J394"/>
+  <autoFilter ref="A1:J395"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 8)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$406</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$409</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J406"/>
+  <dimension ref="A1:J409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17101,8 +17101,131 @@
         </is>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>1205625456</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>onishi-cosme</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>ホワイテスＶＣウォッシュ (150g) 洗顔 カルノシン ビタミンCエステル プラセンタエキス セラミド グリチルリチン 【大西ドクターズコスメ】</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Dr.Onishi Cosmeceutical</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G407" t="n">
+        <v>0</v>
+      </c>
+      <c r="H407" t="b">
+        <v>0</v>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205625456</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>1205624717</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>onishi-cosme</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>スキンプロテクトクレンズ (150ml) クレンジングジェル EGF コラーゲン ビタミンE アロエベラエキス 界面活性剤不使用 【大西ドクターズコスメ】</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Dr.Onishi Cosmeceutical</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0</v>
+      </c>
+      <c r="H408" t="b">
+        <v>0</v>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205624717</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>1205607511</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>onishi-cosme</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>VCローション (55ml) 化粧水 APPS ビタミンC誘導体 【大西ドクターズコスメ】</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Dr.Onishi Cosmeceutical</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0</v>
+      </c>
+      <c r="H409" t="b">
+        <v>0</v>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205607511</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J406"/>
+  <autoFilter ref="A1:J409"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 25, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$443</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$445</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J443"/>
+  <dimension ref="A1:J445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18493,8 +18493,90 @@
         </is>
       </c>
     </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>1194283472</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>bequemstore</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>ケアセラ(CareCera) APフェイス&amp;amp;ボディ 乳液 200ml (セラミドプラス×8種の天然型セラミド配合)</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>ケアセラ</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>864</v>
+      </c>
+      <c r="G444" t="n">
+        <v>0</v>
+      </c>
+      <c r="H444" t="b">
+        <v>0</v>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194283472</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>1194288393</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>bequemstore</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>セザンヌ マスカラリムーバー 5.0g 頑固なマスカラもするんと落とす 幅広コーム</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>セザンヌ</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>597</v>
+      </c>
+      <c r="G445" t="n">
+        <v>6</v>
+      </c>
+      <c r="H445" t="b">
+        <v>0</v>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194288393</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J443"/>
+  <autoFilter ref="A1:J445"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 26, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$445</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$446</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J445"/>
+  <dimension ref="A1:J446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18575,8 +18575,49 @@
         </is>
       </c>
     </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>1179610392</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>aishodo</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>舞妓フェイスウオッシュ</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>AISHODO</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>950</v>
+      </c>
+      <c r="G446" t="n">
+        <v>0</v>
+      </c>
+      <c r="H446" t="b">
+        <v>0</v>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179610392</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J445"/>
+  <autoFilter ref="A1:J446"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 28, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$446</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$447</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J446"/>
+  <dimension ref="A1:J447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18616,8 +18616,49 @@
         </is>
       </c>
     </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>1182343949</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>bijinnuka</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>エッセンスクレンジングジェル （135g）　ヒアルロン酸　ジヒドロキシプロピルアルギニンHCI　米発酵液</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>RICE UP SKIN</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G447" t="n">
+        <v>1</v>
+      </c>
+      <c r="H447" t="b">
+        <v>0</v>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182343949</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J446"/>
+  <autoFilter ref="A1:J447"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 37)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$447</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$451</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J447"/>
+  <dimension ref="A1:J451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18657,8 +18657,172 @@
         </is>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>1053474210</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>SilkyWax</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>SilkyWax ブラジリアンワックス ペーパー 100枚 ワックス 脱毛 ストリップス ストリップスペーパー セルフ 自宅</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Silky Wax</t>
+        </is>
+      </c>
+      <c r="F448" t="n">
+        <v>678</v>
+      </c>
+      <c r="G448" t="n">
+        <v>5</v>
+      </c>
+      <c r="H448" t="b">
+        <v>0</v>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1053474210</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>1160008640</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>SilkyWax</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>ブラジリアンワックス 450g スターターセット ペーパー スパチュラ シュガーワックス ワックス脱毛 脱毛器 全身 脱毛 VIO脱毛 純国産無添加</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Silky Wax</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G449" t="n">
+        <v>3</v>
+      </c>
+      <c r="H449" t="b">
+        <v>0</v>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160008640</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>1160008478</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>SilkyWax</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>【純国産/大容量450g】 シュガーワックス 単品 ブラジリアンワックス VIO 全身 脱毛 無添加 水で洗い流せる デリケートゾーン</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Silky Wax</t>
+        </is>
+      </c>
+      <c r="F450" t="n">
+        <v>2480</v>
+      </c>
+      <c r="G450" t="n">
+        <v>2</v>
+      </c>
+      <c r="H450" t="b">
+        <v>0</v>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160008478</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1113303393</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>SilkyWax</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>ブラジリアンワックス　鼻毛ワックス脱毛キット 3回分 ストッパー付 メンズ 男性 女性 鼻毛処理 レディース 鼻毛取り 自宅 セルフ 鼻毛脱毛キット</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Silky Wax</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>580</v>
+      </c>
+      <c r="G451" t="n">
+        <v>6</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1113303393</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J447"/>
+  <autoFilter ref="A1:J451"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 4, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$452</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$454</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J452"/>
+  <dimension ref="A1:J454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18862,8 +18862,90 @@
         </is>
       </c>
     </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>1210843857</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>drmarci</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Dr. Marci 米発酵セルタチオン 色素沈着・美白 メラノンクリーム, 1個</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>dr.marci</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>3760</v>
+      </c>
+      <c r="G453" t="n">
+        <v>0</v>
+      </c>
+      <c r="H453" t="b">
+        <v>0</v>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210843857</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>1210837461</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>drmarci</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Dr. Marci 毛穴引き締め54% 皮脂コントロール クリーム, 1個</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>dr.marci</t>
+        </is>
+      </c>
+      <c r="F454" t="n">
+        <v>3760</v>
+      </c>
+      <c r="G454" t="n">
+        <v>0</v>
+      </c>
+      <c r="H454" t="b">
+        <v>0</v>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210837461</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J452"/>
+  <autoFilter ref="A1:J454"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 8, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$454</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$455</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J454"/>
+  <dimension ref="A1:J455"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18944,8 +18944,49 @@
         </is>
       </c>
     </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>1191430718</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>laboreve</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>ラボレブ ピーチマイクロバイオーム 78 PDRNトナー</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Laboreve</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G455" t="n">
+        <v>1</v>
+      </c>
+      <c r="H455" t="b">
+        <v>0</v>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191430718</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J454"/>
+  <autoFilter ref="A1:J455"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 14)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$455</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$458</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J455"/>
+  <dimension ref="A1:J458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18985,8 +18985,131 @@
         </is>
       </c>
     </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>1214263390</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>ocura</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>【公式正規品】 バイオリフト HBA-X ブースタージェル 200mL (5本セット)</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>OCURA</t>
+        </is>
+      </c>
+      <c r="F456" t="n">
+        <v>16415</v>
+      </c>
+      <c r="G456" t="n">
+        <v>0</v>
+      </c>
+      <c r="H456" t="b">
+        <v>0</v>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214263390</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>1214262100</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>ocura</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>【公式正規品】 バイオリフト HBA-X ブースタージェル 200mL (2本セット)</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>OCURA</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>7840</v>
+      </c>
+      <c r="G457" t="n">
+        <v>0</v>
+      </c>
+      <c r="H457" t="b">
+        <v>0</v>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214262100</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>1209394020</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>ocura</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>【公式正規品】 バイオリフト HBA-X ブースタージェル 200mL</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>OCURA</t>
+        </is>
+      </c>
+      <c r="F458" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G458" t="n">
+        <v>2</v>
+      </c>
+      <c r="H458" t="b">
+        <v>0</v>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209394020</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J455"/>
+  <autoFilter ref="A1:J458"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 10)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$460</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$463</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J460"/>
+  <dimension ref="A1:J463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19190,8 +19190,131 @@
         </is>
       </c>
     </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>1146079054</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>kenbi</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>プレミアムナチュレクレンジング PNクレンジング 250g</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>ミューフル</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>12100</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0</v>
+      </c>
+      <c r="H461" t="b">
+        <v>0</v>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146079054</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>1146192873</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>kenbi</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>プレミアムナチュレローション PNローション 300mL</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>ミューフル</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0</v>
+      </c>
+      <c r="H462" t="b">
+        <v>0</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146192873</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>669602673</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>kenbi</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>アクア ラ ビュー 500ml</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>ギブアンドギブ</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>5500</v>
+      </c>
+      <c r="G463" t="n">
+        <v>4</v>
+      </c>
+      <c r="H463" t="b">
+        <v>0</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=669602673</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J460"/>
+  <autoFilter ref="A1:J463"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 11)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$463</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$464</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J463"/>
+  <dimension ref="A1:J464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19313,8 +19313,49 @@
         </is>
       </c>
     </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>1150799106</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>nporder</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>MDSKIN LABO シートマスク パック アゼライン酸 ビタミンC誘導体 グリチルリチン酸ジカリウム セラミド フェイスマスク フェイスパック オールインワン</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>MDSKIN LABO</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>800</v>
+      </c>
+      <c r="G464" t="n">
+        <v>3</v>
+      </c>
+      <c r="H464" t="b">
+        <v>0</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150799106</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J463"/>
+  <autoFilter ref="A1:J464"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 19, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$465</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$469</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J465"/>
+  <dimension ref="A1:J469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19395,8 +19395,172 @@
         </is>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>1211548014</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>sohairofficial</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>[NS 500 SB+SF] ソヘア ナリシングシャンプー ダメージケア 500g (1+1)</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>sohair</t>
+        </is>
+      </c>
+      <c r="F466" t="n">
+        <v>4150</v>
+      </c>
+      <c r="G466" t="n">
+        <v>0</v>
+      </c>
+      <c r="H466" t="b">
+        <v>0</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211548014</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>1214907497</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>sohairofficial</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>[RF100] モロッコアルガンオイル リファインド ダブルケア エッセンス</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>sohair</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G467" t="n">
+        <v>6</v>
+      </c>
+      <c r="H467" t="b">
+        <v>0</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214907497</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>1211802618</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>sohairofficial</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>[NS 500 SF] ソヘア ナリシングシャンプー ダメージケア スウィートフルーティ 500g</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>sohair</t>
+        </is>
+      </c>
+      <c r="F468" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G468" t="n">
+        <v>0</v>
+      </c>
+      <c r="H468" t="b">
+        <v>0</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211802618</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>1211060520</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>sohairofficial</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>[NS 1000 OG] ソヘア ナリシングシャンプー ダメージケア オリジナルハニーフラワー 1000g</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>sohair</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G469" t="n">
+        <v>0</v>
+      </c>
+      <c r="H469" t="b">
+        <v>0</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211060520</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J465"/>
+  <autoFilter ref="A1:J469"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 29, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$470</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$473</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J470"/>
+  <dimension ref="A1:J473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19600,8 +19600,131 @@
         </is>
       </c>
     </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>1090183841</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>gcb</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>B.C.A.D.HOMME トータルエマルジョン 120ml オールインワン 化粧水</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>ビーシーエーディー</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G471" t="n">
+        <v>0</v>
+      </c>
+      <c r="H471" t="b">
+        <v>0</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1090183841</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>1090331730</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>gcb</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>【お得な3本＋1本プレゼント】ナチュラルビューティセレクション スキャルプエッセンススプレー 180g 頭皮＆ボディ用美容液（リラックスグリーンティ）</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Natural Beauty Selection</t>
+        </is>
+      </c>
+      <c r="F472" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G472" t="n">
+        <v>3</v>
+      </c>
+      <c r="H472" t="b">
+        <v>0</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1090331730</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>1090182799</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>gcb</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>ハードゼリー 300g</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>ロレッタ</t>
+        </is>
+      </c>
+      <c r="F473" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G473" t="n">
+        <v>0</v>
+      </c>
+      <c r="H473" t="b">
+        <v>0</v>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1090182799</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J470"/>
+  <autoFilter ref="A1:J473"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 5, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$473</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$476</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J473"/>
+  <dimension ref="A1:J476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19723,8 +19723,131 @@
         </is>
       </c>
     </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>1190724950</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>3種から1種選択 パフュームヘアオイル 80ml ヒノキ オスマントゥス ラピタ 10mlミニ付 エンジェルミュゲ 艶髪 保湿 ダメージケア 補修 スタイリング べたつかない 人気 ギフト 贈り物</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>La'dor</t>
+        </is>
+      </c>
+      <c r="F474" t="n">
+        <v>4992</v>
+      </c>
+      <c r="G474" t="n">
+        <v>0</v>
+      </c>
+      <c r="H474" t="b">
+        <v>0</v>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190724950</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>1212757907</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>[26年リニューアル新型/クリーム2種セット] ビタトーニングカプセルクリームナイアシンアミド5%単一型+チューブ型 #無膜ビタカプセル トーンアップ 美白 毛穴ケア 保湿 ツヤ肌 ビタミンC 韓国</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F475" t="n">
+        <v>9415</v>
+      </c>
+      <c r="G475" t="n">
+        <v>0</v>
+      </c>
+      <c r="H475" t="b">
+        <v>0</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212757907</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>1209582946</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>ウォーターフル エッセンス サンミスト 50ml 韓国コスメ 日焼け止め 紫外線対策 保湿 ツヤ肌 顔 体用 スプレータイプ メイクの上から 持ち運び便利 UVケア</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F476" t="n">
+        <v>5848</v>
+      </c>
+      <c r="G476" t="n">
+        <v>0</v>
+      </c>
+      <c r="H476" t="b">
+        <v>0</v>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209582946</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J473"/>
+  <autoFilter ref="A1:J476"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 10, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$490</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$492</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J490"/>
+  <dimension ref="A1:J492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20420,8 +20420,90 @@
         </is>
       </c>
     </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>1137567849</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>45do</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>アクアスクワラン モイスチャライジングクリーム 60ml</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>エスネイチャー</t>
+        </is>
+      </c>
+      <c r="F491" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0</v>
+      </c>
+      <c r="H491" t="b">
+        <v>0</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137567849</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>1139845347</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>45do</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>魔女工場 パンテトイン エッセンストナー 200ml / 2in1 化粧水 / 高保湿 / 鎮静ケア</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F492" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G492" t="n">
+        <v>0</v>
+      </c>
+      <c r="H492" t="b">
+        <v>0</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139845347</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J490"/>
+  <autoFilter ref="A1:J492"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 27)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$500</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J500"/>
+  <dimension ref="A1:J501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20830,8 +20830,49 @@
         </is>
       </c>
     </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>1073637375</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>コントロールA ティーツリーメント クレンジングフォーム 120ml 1EA</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F501" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0</v>
+      </c>
+      <c r="H501" t="b">
+        <v>0</v>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1073637375</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J500"/>
+  <autoFilter ref="A1:J501"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 14, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$517</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$520</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J517"/>
+  <dimension ref="A1:J520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21527,8 +21527,131 @@
         </is>
       </c>
     </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>1060232385</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>HAMAHAMA</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>シカ エッセンス サン保湿 敏感肌 乾燥肌 混合肌 スキンケア 韓国コスメ 日焼け止め サンケア SPF50+/PA++++</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F518" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G518" t="n">
+        <v>0</v>
+      </c>
+      <c r="H518" t="b">
+        <v>0</v>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1060232385</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>1193592249</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>HAMAHAMA</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>アップルサイダー ホイップクリームパッククレンザー 200ml</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>アリウル</t>
+        </is>
+      </c>
+      <c r="F519" t="n">
+        <v>3060</v>
+      </c>
+      <c r="G519" t="n">
+        <v>0</v>
+      </c>
+      <c r="H519" t="b">
+        <v>0</v>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193592249</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>1115880952</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>HAMAHAMA</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>ノースカナイントラブルセラム 30ml</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>パティオン</t>
+        </is>
+      </c>
+      <c r="F520" t="n">
+        <v>4260</v>
+      </c>
+      <c r="G520" t="n">
+        <v>0</v>
+      </c>
+      <c r="H520" t="b">
+        <v>0</v>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115880952</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J517"/>
+  <autoFilter ref="A1:J520"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 16, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$522</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$524</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J522"/>
+  <dimension ref="A1:J524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21732,8 +21732,90 @@
         </is>
       </c>
     </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>1099897481</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>STARKOREA</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>クールでクリアな頭皮リフレッシュシャンプーアクアミント 500ml</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F523" t="n">
+        <v>2475</v>
+      </c>
+      <c r="G523" t="n">
+        <v>1</v>
+      </c>
+      <c r="H523" t="b">
+        <v>0</v>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1099897481</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>1150407145</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>greenapple</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>アトバリア 365 ローション ATOBARRIER 365 150ml</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F524" t="n">
+        <v>4950</v>
+      </c>
+      <c r="G524" t="n">
+        <v>0</v>
+      </c>
+      <c r="H524" t="b">
+        <v>0</v>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150407145</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J522"/>
+  <autoFilter ref="A1:J524"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 20, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$533</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$536</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J533"/>
+  <dimension ref="A1:J536"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22183,8 +22183,131 @@
         </is>
       </c>
     </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>1196162300</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>cosmeplaza01</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>【即納】【2026年リニューア新パッケージ・国内正規品・まとめ買い・追跡可能メール便発送】パーフェクトUV スキンケアミルク 日やけ止め NA 本体 60mL×2個セット【4909978147105</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>アネッサ</t>
+        </is>
+      </c>
+      <c r="F534" t="n">
+        <v>4888</v>
+      </c>
+      <c r="G534" t="n">
+        <v>0</v>
+      </c>
+      <c r="H534" t="b">
+        <v>0</v>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196162300</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>1188699095</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>relationmarketing</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>BOJ Relief Sun Aqua-fresh : Rice +B5 Beauty of Joseon 米アクアフレッシュサンクリーム 50ml SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>2794</v>
+      </c>
+      <c r="G535" t="n">
+        <v>0</v>
+      </c>
+      <c r="H535" t="b">
+        <v>0</v>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188699095</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>1188697212</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>relationmarketing</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>熊野油脂 ｃｙｃｌｅａｒ ビタミンCボディミルク 400ML</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>熊野油脂</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>512</v>
+      </c>
+      <c r="G536" t="n">
+        <v>0</v>
+      </c>
+      <c r="H536" t="b">
+        <v>0</v>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188697212</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J533"/>
+  <autoFilter ref="A1:J536"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 22, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$536</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$537</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J536"/>
+  <dimension ref="A1:J537"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22306,8 +22306,49 @@
         </is>
       </c>
     </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>1171281161</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>piko</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>ドクターケイ(Dr.K) 薬用Cクリアクレンジングジェル(医薬部外品)【メイク落とし】ビタミンC誘導体 毛穴 W洗顔不要 まつエクOK クレンジング</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>ドクターケイ</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G537" t="n">
+        <v>0</v>
+      </c>
+      <c r="H537" t="b">
+        <v>0</v>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171281161</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J536"/>
+  <autoFilter ref="A1:J537"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 23, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$537</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$538</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J537"/>
+  <dimension ref="A1:J538"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22347,8 +22347,49 @@
         </is>
       </c>
     </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>1211813734</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Salute666</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>NO.6 ボンドスムーサー ノンウォッシュ エッセンス ミルク 100ml 美容/シャンプー/ ヘアトリートメント</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>オラプレックス</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G538" t="n">
+        <v>0</v>
+      </c>
+      <c r="H538" t="b">
+        <v>0</v>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211813734</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J537"/>
+  <autoFilter ref="A1:J538"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 31, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$547</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$549</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J547"/>
+  <dimension ref="A1:J549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22757,8 +22757,90 @@
         </is>
       </c>
     </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>1192596376</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>[メガ割] manyo factory 魔女工場 ガラクナイアシン エッセンス クリーム 50ml ガラクトミセス 保湿 弾力 ハリ ツヤ 潤い 浸透 スキンケア 基礎化粧品 韓国コスメ 人気 公式</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>4891</v>
+      </c>
+      <c r="G548" t="n">
+        <v>0</v>
+      </c>
+      <c r="H548" t="b">
+        <v>0</v>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192596376</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>1211822634</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>CinderellaBeaute</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>BOBBI BROWN(ボビイ ブラウン) ビタエンリッチド クリーム＆フェイスベース プラス 15mL</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>ボビイブラウン</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>4780</v>
+      </c>
+      <c r="G549" t="n">
+        <v>0</v>
+      </c>
+      <c r="H549" t="b">
+        <v>0</v>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211822634</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J547"/>
+  <autoFilter ref="A1:J549"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 32, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$549</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J549"/>
+  <dimension ref="A1:J550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22839,8 +22839,49 @@
         </is>
       </c>
     </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>1021878726</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>jkmtr-jp</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>[韓国公式/代理店] BEST リノイア ウォーター トリートメント 200ml 1個</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>RE:NOIA</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>1770</v>
+      </c>
+      <c r="G550" t="n">
+        <v>6</v>
+      </c>
+      <c r="H550" t="b">
+        <v>0</v>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1021878726</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J549"/>
+  <autoFilter ref="A1:J550"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 34, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$551</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$553</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J551"/>
+  <dimension ref="A1:J553"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22921,8 +22921,90 @@
         </is>
       </c>
     </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>1208291130</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>OROBA</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>ワキ ひじ VIO Yゾーン ケアクリーム 100ml 保湿 部分ケア デリケートゾーン 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>BnD</t>
+        </is>
+      </c>
+      <c r="F552" t="n">
+        <v>4135</v>
+      </c>
+      <c r="G552" t="n">
+        <v>0</v>
+      </c>
+      <c r="H552" t="b">
+        <v>0</v>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208291130</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>1203203087</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>mrelephant</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>スキンケアパッド 4種 (各タイプ別)/シラカバ]潤い水分/セリ カミング鎮静/ユジャC トーンアップ(ブライトニング)/ザクロ ハリ弾力パーミング/</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>コアコス</t>
+        </is>
+      </c>
+      <c r="F553" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G553" t="n">
+        <v>0</v>
+      </c>
+      <c r="H553" t="b">
+        <v>0</v>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203203087</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J551"/>
+  <autoFilter ref="A1:J553"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 38, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$553</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$554</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J553"/>
+  <dimension ref="A1:J554"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23003,8 +23003,49 @@
         </is>
       </c>
     </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>1159386892</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>ng0912</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Sevich ヘアふわふわパウダー瞬時にヘアコンシーラーカバレッジ瞬時に黒根カバーアップナチュラルインスタントヘアラインシャドウ</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>SEVICH</t>
+        </is>
+      </c>
+      <c r="F554" t="n">
+        <v>1472</v>
+      </c>
+      <c r="G554" t="n">
+        <v>1</v>
+      </c>
+      <c r="H554" t="b">
+        <v>0</v>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159386892</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J553"/>
+  <autoFilter ref="A1:J554"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 40, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$554</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$558</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J554"/>
+  <dimension ref="A1:J558"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23044,8 +23044,172 @@
         </is>
       </c>
     </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>1076629884</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>cellbycellnextera</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>【公式】 パック シートマスク フェイスパック シートパック 顔パック シークレットヌードマスク Secret Nude Mask セルバイセル CELLBYCELL 高保湿 ハリ 無添加 敏感肌</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>CELL by CELL</t>
+        </is>
+      </c>
+      <c r="F555" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G555" t="n">
+        <v>8</v>
+      </c>
+      <c r="H555" t="b">
+        <v>0</v>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1076629884</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>1076625501</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>cellbycellnextera</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>【公式】 日焼け止めクリーム SPF50+ PA+++ 低刺激 紫外線カット パウダリーサンブロッククリーム Powdery Sun BlockCream セルバイセル CELLBYCELL UV</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>CELL by CELL</t>
+        </is>
+      </c>
+      <c r="F556" t="n">
+        <v>6270</v>
+      </c>
+      <c r="G556" t="n">
+        <v>5</v>
+      </c>
+      <c r="H556" t="b">
+        <v>0</v>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1076625501</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>1076566467</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>cellbycellnextera</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>【公式】 クリーム 高保湿クリーム スキンケア ハイドラシーモイスチャークリーム HydraC Moisture Cream セルバイセル CELLBYCELL 低刺激 弱酸性 顔 全身 ベタつかない</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>CELL by CELL</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>6930</v>
+      </c>
+      <c r="G557" t="n">
+        <v>4</v>
+      </c>
+      <c r="H557" t="b">
+        <v>0</v>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1076566467</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>1177820470</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>cellbycellnextera</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>【韓国顧客感動指数1位獲得】 ピーリング 美容液 セルバイセル ビタミン ピーリング セラム スキンケア 美容 角質ケア 毛穴ケア クレンジング 鎮静 保湿 透明感 ザラつき ごわつき</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>CELL by CELL</t>
+        </is>
+      </c>
+      <c r="F558" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G558" t="n">
+        <v>1</v>
+      </c>
+      <c r="H558" t="b">
+        <v>0</v>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177820470</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J554"/>
+  <autoFilter ref="A1:J558"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 43, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$558</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$559</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J558"/>
+  <dimension ref="A1:J559"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23208,8 +23208,49 @@
         </is>
       </c>
     </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>1181831740</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>likeplan</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>インナーメイトウォッシュデイリー150ml/ スペシャル100ml企画セット（+おかわりプレゼント）</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>OVMENT</t>
+        </is>
+      </c>
+      <c r="F559" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G559" t="n">
+        <v>1</v>
+      </c>
+      <c r="H559" t="b">
+        <v>0</v>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181831740</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J558"/>
+  <autoFilter ref="A1:J559"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 44, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$559</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$560</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J559"/>
+  <dimension ref="A1:J560"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23249,8 +23249,49 @@
         </is>
       </c>
     </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>1191750153</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>korimori</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>中外製薬 フレンズ アイドロップ 14ml 4種（スン・クール・クールハイ・アイス）</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Jw Pharmaceutical</t>
+        </is>
+      </c>
+      <c r="F560" t="n">
+        <v>1580</v>
+      </c>
+      <c r="G560" t="n">
+        <v>0</v>
+      </c>
+      <c r="H560" t="b">
+        <v>0</v>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191750153</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J559"/>
+  <autoFilter ref="A1:J560"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 47, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$564</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$568</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J564"/>
+  <dimension ref="A1:J568"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23454,8 +23454,172 @@
         </is>
       </c>
     </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>1209060848</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>botanic-garden</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>ロレアル セリエ エクスパート ビタミノカラー シャンプー 300ml</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>2094</v>
+      </c>
+      <c r="G565" t="n">
+        <v>0</v>
+      </c>
+      <c r="H565" t="b">
+        <v>0</v>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209060848</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>1188309818</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>botanic-garden</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>【送料無料】【2個セット】ミシャ MISSHA グロウ UV トーンアップ プライマー 30mL</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F566" t="n">
+        <v>3768</v>
+      </c>
+      <c r="G566" t="n">
+        <v>1</v>
+      </c>
+      <c r="H566" t="b">
+        <v>0</v>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188309818</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>1154071754</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>botanic-garden</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>ハホニコ キラメトゥインクル　シャンプー【サロン専売品】 1000ml</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>ハホニコ</t>
+        </is>
+      </c>
+      <c r="F567" t="n">
+        <v>2855</v>
+      </c>
+      <c r="G567" t="n">
+        <v>3</v>
+      </c>
+      <c r="H567" t="b">
+        <v>0</v>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154071754</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>1154072467</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>botanic-garden</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>セフティ hunt ハント スタイリングジェル 300g</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>セフティ</t>
+        </is>
+      </c>
+      <c r="F568" t="n">
+        <v>1057</v>
+      </c>
+      <c r="G568" t="n">
+        <v>0</v>
+      </c>
+      <c r="H568" t="b">
+        <v>0</v>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154072467</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J564"/>
+  <autoFilter ref="A1:J568"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 49, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$570</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$573</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J570"/>
+  <dimension ref="A1:J573"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23700,8 +23700,131 @@
         </is>
       </c>
     </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>1127135721</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>sensepicklshop</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>R.E.D. ブレミッシュ クリア クリーム 70ml [ NO BOX]</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>HAVE_R</t>
+        </is>
+      </c>
+      <c r="F571" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G571" t="n">
+        <v>2</v>
+      </c>
+      <c r="H571" t="b">
+        <v>0</v>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1127135721</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>1201224916</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>sensepicklshop</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>ブルー PDRN ダブルアンプル 45ml / PDRNによる年齢痕跡の改善・老廃物除去・シワ改善・ホワイトニング効果</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>HOLITUAL</t>
+        </is>
+      </c>
+      <c r="F572" t="n">
+        <v>10900</v>
+      </c>
+      <c r="G572" t="n">
+        <v>0</v>
+      </c>
+      <c r="H572" t="b">
+        <v>0</v>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201224916</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>1121941472</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>sensepicklshop</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>ホーリチュアル バランシング エッセンス150ML+スムージングローション110ML+サンプル</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>アモーレパシフィック</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>11999</v>
+      </c>
+      <c r="G573" t="n">
+        <v>4</v>
+      </c>
+      <c r="H573" t="b">
+        <v>0</v>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1121941472</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J570"/>
+  <autoFilter ref="A1:J573"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 50, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$573</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$578</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J573"/>
+  <dimension ref="A1:J578"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23823,8 +23823,213 @@
         </is>
       </c>
     </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>1046101797</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>WhiteFlower</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>ヒアテノールハイドラクリーム, 50mL</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F574" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G574" t="n">
+        <v>9</v>
+      </c>
+      <c r="H574" t="b">
+        <v>0</v>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1046101797</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>1046102052</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>WhiteFlower</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>ヒアテノールハイドラフォームクレンザー, 150mL</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G575" t="n">
+        <v>2</v>
+      </c>
+      <c r="H575" t="b">
+        <v>0</v>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1046102052</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>1209271213</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>LUVLUCE</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>ホーリーバジル バブル ディープ マスク 90g, 1個 炭酸泡 毛穴ケア 角質 泥パック スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>P.CALM</t>
+        </is>
+      </c>
+      <c r="F576" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G576" t="n">
+        <v>0</v>
+      </c>
+      <c r="H576" t="b">
+        <v>0</v>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209271213</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>1215003999</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>LUVLUCE</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>【NEW】透明感ケア ダーマアンサー ダーマアンサー TXA-PDRNブライトニングブースターアンプル30ml 美容液 セラム 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>CNP Laboratory</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>4362</v>
+      </c>
+      <c r="G577" t="n">
+        <v>0</v>
+      </c>
+      <c r="H577" t="b">
+        <v>0</v>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215003999</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>1208337662</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>LUVLUCE</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>ヴィーガン リリーフ トーンアップ サンエッセンス ライトピンク 50ml 1個 透き通る肌 日焼け止め UVケア</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>アッテ</t>
+        </is>
+      </c>
+      <c r="F578" t="n">
+        <v>3218</v>
+      </c>
+      <c r="G578" t="n">
+        <v>0</v>
+      </c>
+      <c r="H578" t="b">
+        <v>0</v>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208337662</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J573"/>
+  <autoFilter ref="A1:J578"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 52, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$578</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$583</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J578"/>
+  <dimension ref="A1:J583"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24028,8 +24028,213 @@
         </is>
       </c>
     </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>1210368860</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>【正規品】メディヒ チャン・ドヨン マデカソサイド 痕跡リペア デルマ保湿クリーム 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>ハンユル</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G579" t="n">
+        <v>0</v>
+      </c>
+      <c r="H579" t="b">
+        <v>0</v>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210368860</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>1145740768</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>【正規品】 UVシールド サン スティック 20g SPF50+/PA++++</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F580" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G580" t="n">
+        <v>0</v>
+      </c>
+      <c r="H580" t="b">
+        <v>0</v>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145740768</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>1147757123</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>【正規品】【NEW】ヒーロークッション 2.0 12g 密着水分 [SPF50+/PA]++++]本品+リフィル</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>4890</v>
+      </c>
+      <c r="G581" t="n">
+        <v>1</v>
+      </c>
+      <c r="H581" t="b">
+        <v>0</v>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147757123</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>1209979406</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>【正規品】ハンーユル 幼いヨモギ 皮脂吸着 ヨモギ餅パックフォーム 120ml, 1個</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>ハンユル</t>
+        </is>
+      </c>
+      <c r="F582" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G582" t="n">
+        <v>1</v>
+      </c>
+      <c r="H582" t="b">
+        <v>0</v>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209979406</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>1203714433</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>【正規品】 バイオ インビジブル コラーゲン ペプチド サンセラム 50ml（SPF 50+）</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F583" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G583" t="n">
+        <v>0</v>
+      </c>
+      <c r="H583" t="b">
+        <v>0</v>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203714433</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J578"/>
+  <autoFilter ref="A1:J583"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 55, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$583</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$584</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J583"/>
+  <dimension ref="A1:J584"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24233,8 +24233,49 @@
         </is>
       </c>
     </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>1164573759</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>ivice</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>【各2本セット＋ファンデーションブラシ付】クリスタル シルキー シャンプー・トリートメント・ヘアオイル</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>ジェニーハウス</t>
+        </is>
+      </c>
+      <c r="F584" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G584" t="n">
+        <v>2</v>
+      </c>
+      <c r="H584" t="b">
+        <v>0</v>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164573759</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J583"/>
+  <autoFilter ref="A1:J584"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 59, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$586</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$590</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J586"/>
+  <dimension ref="A1:J590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24356,8 +24356,172 @@
         </is>
       </c>
     </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>1206264240</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>odecomart</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>宅配便 FeMish PERFUME 10ml (ベルベットカシス/ホワイトティー/フルーティシャンパン/ローズジュエリー) フェミッシュパフューム VIOフレグランス</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>セルノート</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G587" t="n">
+        <v>1</v>
+      </c>
+      <c r="H587" t="b">
+        <v>0</v>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206264240</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>1194323430</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>【選べる】オージュア　シャンプー1000ml各種 詰め替え　クエンチ　クエンチモイスト　イミュライズ　タイムサージ インメトリィ　リペアリティ　フィルメロウ　エクイアル　ディオーラム　モイストカーム</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>オージュア</t>
+        </is>
+      </c>
+      <c r="F588" t="n">
+        <v>9200</v>
+      </c>
+      <c r="G588" t="n">
+        <v>1</v>
+      </c>
+      <c r="H588" t="b">
+        <v>0</v>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194323430</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>1194323429</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>【選べる】オージュア　トリートメント1000g各種 詰め替え　クエンチ　クエンチモイスト　イミュライズ　タイムサージ インメトリィ　リペアリティ　フィルメロウ　エクイアル　ディオーラム　モイストカーム</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>オージュア</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>11500</v>
+      </c>
+      <c r="G589" t="n">
+        <v>0</v>
+      </c>
+      <c r="H589" t="b">
+        <v>0</v>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194323429</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>1195074904</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>【正規品】フィヨーレ　クオルシア　カラーシャンプー　紫　purple　1000ml　【サロン専売品】【ブリーチケア】【カラーケア】【ムラシャン】【最安値更新中】【正規品】【色落ちケア】</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>フィヨーレ</t>
+        </is>
+      </c>
+      <c r="F590" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G590" t="n">
+        <v>3</v>
+      </c>
+      <c r="H590" t="b">
+        <v>0</v>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195074904</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J586"/>
+  <autoFilter ref="A1:J590"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 61, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$594</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$597</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J594"/>
+  <dimension ref="A1:J597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24684,8 +24684,131 @@
         </is>
       </c>
     </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>1203467584</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>daily_kim</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>ビタミンCグリーンティーエンザイムセラム30+30ml+ジェシーポーチ企画トイストーリー5エディション</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>4600</v>
+      </c>
+      <c r="G595" t="n">
+        <v>1</v>
+      </c>
+      <c r="H595" t="b">
+        <v>0</v>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203467584</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>1203398878</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>daily_kim</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>マスターズアクアリッチサンクリーム50ml 1+1企画(+ピカチュウピンミラー)</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F596" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G596" t="n">
+        <v>0</v>
+      </c>
+      <c r="H596" t="b">
+        <v>0</v>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203398878</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>1189683758</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>daily_kim</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>バランスフル シカ トナーパッド 60枚+詰め替え 60枚, 1セット</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G597" t="n">
+        <v>0</v>
+      </c>
+      <c r="H597" t="b">
+        <v>0</v>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189683758</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J594"/>
+  <autoFilter ref="A1:J597"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 62, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$597</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$599</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J597"/>
+  <dimension ref="A1:J599"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24807,8 +24807,90 @@
         </is>
       </c>
     </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>1140265933</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>BEBALANCE</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>【公式】ビーバランス ヨモギマスクパック 敏感肌＋鎮静ケア 正規品 10枚入 韓国コスメ ビバランス</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>BE BALANCE</t>
+        </is>
+      </c>
+      <c r="F598" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G598" t="n">
+        <v>3</v>
+      </c>
+      <c r="H598" t="b">
+        <v>0</v>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1140265933</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>1181715148</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>BEBALANCE</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>【公式】ビーバランス リフリマスクパック 敏感肌＋鎮静ケア 正規品 10枚入 韓国コスメ ビバランス</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>BE BALANCE</t>
+        </is>
+      </c>
+      <c r="F599" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G599" t="n">
+        <v>0</v>
+      </c>
+      <c r="H599" t="b">
+        <v>0</v>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181715148</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J597"/>
+  <autoFilter ref="A1:J599"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 64, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$602</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$606</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J602"/>
+  <dimension ref="A1:J606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25012,8 +25012,172 @@
         </is>
       </c>
     </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>1210269451</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>MOJII</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>【公式／並行輸入品（正規流通）】傷あとケア用 シリコーンジェル 7g 1本 ウルトラジェル</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>ダーマティックス</t>
+        </is>
+      </c>
+      <c r="F603" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G603" t="n">
+        <v>1</v>
+      </c>
+      <c r="H603" t="b">
+        <v>0</v>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210269451</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>1194798841</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>MOJII</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>毛穴角質ケア用スキンピリング 1回分</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>BQCELL</t>
+        </is>
+      </c>
+      <c r="F604" t="n">
+        <v>7460</v>
+      </c>
+      <c r="G604" t="n">
+        <v>0</v>
+      </c>
+      <c r="H604" t="b">
+        <v>0</v>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194798841</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>1207862816</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>MOJII</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>【大容量50枚】選べる10種 シートマスク カプセルマスクパック デイリーマスク 保湿 毛穴ケア CICA レチノール 韓国パック</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>GRACE DAY</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>3230</v>
+      </c>
+      <c r="G605" t="n">
+        <v>0</v>
+      </c>
+      <c r="H605" t="b">
+        <v>0</v>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207862816</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>1207862688</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>MOJII</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>【大容量100枚】カプセルマスクパック 10種から選べる 50枚入×2個セット 合計100枚 デイリーマスク 保湿 ハリ 毛穴ケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>GRACE DAY</t>
+        </is>
+      </c>
+      <c r="F606" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G606" t="n">
+        <v>0</v>
+      </c>
+      <c r="H606" t="b">
+        <v>0</v>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207862688</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J602"/>
+  <autoFilter ref="A1:J606"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 73, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$606</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$607</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J606"/>
+  <dimension ref="A1:J607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25176,8 +25176,49 @@
         </is>
       </c>
     </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>1134439190</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>wiggle-wiggle</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>[選択1] wiggle wiggle ヘアカーラー4種 サイズに合わせて選べる #前髪カーラー #前髪クリップ #ヘアロール</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>WIGGLE WIGGLE</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>1450</v>
+      </c>
+      <c r="G607" t="n">
+        <v>5</v>
+      </c>
+      <c r="H607" t="b">
+        <v>0</v>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134439190</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J606"/>
+  <autoFilter ref="A1:J607"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 79, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$609</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$612</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J609"/>
+  <dimension ref="A1:J612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25299,8 +25299,131 @@
         </is>
       </c>
     </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>1178110572</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>bellmaris</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>ビタプラス トナー 200ml 2本 セット 大容量 ビタミンC 化粧水 保湿 韓国</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F610" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G610" t="n">
+        <v>6</v>
+      </c>
+      <c r="H610" t="b">
+        <v>0</v>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178110572</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>1168721462</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>bellmaris</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>ダメージ ヘアケア ハムビット シャンプー 480ml 2本 ツヤ髪 栄養 保湿 頭皮ケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>呂</t>
+        </is>
+      </c>
+      <c r="F611" t="n">
+        <v>3830</v>
+      </c>
+      <c r="G611" t="n">
+        <v>0</v>
+      </c>
+      <c r="H611" t="b">
+        <v>0</v>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168721462</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>1125655018</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>bellmaris</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>清雅 脂性頭皮 ディープクレンジング クーリング シャンプー 480ml 2本 脂 頭皮ケア 爽快シャンプー 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>呂</t>
+        </is>
+      </c>
+      <c r="F612" t="n">
+        <v>3790</v>
+      </c>
+      <c r="G612" t="n">
+        <v>7</v>
+      </c>
+      <c r="H612" t="b">
+        <v>0</v>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125655018</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J609"/>
+  <autoFilter ref="A1:J612"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 80, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$612</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J612"/>
+  <dimension ref="A1:J616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25422,8 +25422,172 @@
         </is>
       </c>
     </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>1185486289</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>KKvibe</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>【選べる2種の香り】パフュームハンドクリーム ベルベットのようなサラふわ仕上げ エイプリルコットン / ピーチブロッサム</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>W.DRESSROOM</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>750</v>
+      </c>
+      <c r="G613" t="n">
+        <v>2</v>
+      </c>
+      <c r="H613" t="b">
+        <v>0</v>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185486289</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>1179394455</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>KKvibe</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>[香りのいい] パフューム ハンドクリーム 50ml / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>W.DRESSROOM</t>
+        </is>
+      </c>
+      <c r="F614" t="n">
+        <v>750</v>
+      </c>
+      <c r="G614" t="n">
+        <v>4</v>
+      </c>
+      <c r="H614" t="b">
+        <v>0</v>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179394455</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>1204182649</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>KKvibe</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>【導入美容液】ザ・6ペプチド スキンブースターセラム / セット (150ml + 30ml)</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>2199</v>
+      </c>
+      <c r="G615" t="n">
+        <v>1</v>
+      </c>
+      <c r="H615" t="b">
+        <v>0</v>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204182649</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>1170126154</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>KKvibe</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>韓国ピュアライスサンクリーム50ml I I Korea Olive Young Cosmetics</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G616" t="n">
+        <v>4</v>
+      </c>
+      <c r="H616" t="b">
+        <v>0</v>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170126154</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J612"/>
+  <autoFilter ref="A1:J616"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 88, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$620</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$622</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J620"/>
+  <dimension ref="A1:J622"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25750,8 +25750,90 @@
         </is>
       </c>
     </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>1173915032</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>moni_korea</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>レッド ブレミッシュ クイック PHA マスク 30枚 低刺激 肌鎮静 敏感肌 1分で水分チャージ＆鎮静</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F621" t="n">
+        <v>3069</v>
+      </c>
+      <c r="G621" t="n">
+        <v>0</v>
+      </c>
+      <c r="H621" t="b">
+        <v>0</v>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173915032</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>1179881816</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>moni_korea</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>ビタペアC ダークスポット クリーム 50ml x 2,</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F622" t="n">
+        <v>3203</v>
+      </c>
+      <c r="G622" t="n">
+        <v>1</v>
+      </c>
+      <c r="H622" t="b">
+        <v>0</v>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179881816</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J620"/>
+  <autoFilter ref="A1:J622"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 91, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$624</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$625</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J624"/>
+  <dimension ref="A1:J625"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25914,8 +25914,49 @@
         </is>
       </c>
     </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>1211214669</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>ritoselect</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>【No.1クレンジングティッシュ】 ザ・パーフェクト クレンジングティッシュ 100枚×2パック / メイク落とし クレンジングシート 毛穴の汚れ 時間を短縮 スキンケア 拭き取り メイク落とし</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>アリウル</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>2820</v>
+      </c>
+      <c r="G625" t="n">
+        <v>0</v>
+      </c>
+      <c r="H625" t="b">
+        <v>0</v>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211214669</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J624"/>
+  <autoFilter ref="A1:J625"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 95, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$627</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$630</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J627"/>
+  <dimension ref="A1:J630"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26037,8 +26037,131 @@
         </is>
       </c>
     </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>1212713731</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>boundless</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>シャンプー メンズ ドライ2点セット (シャンプー ＆ コンディショナー) 乾燥肌用350ml+350g</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>スカルプD</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G628" t="n">
+        <v>0</v>
+      </c>
+      <c r="H628" t="b">
+        <v>0</v>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212713731</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>1211207443</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>rusion</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>マトメージュオム ポイントデザインスティック</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>ウテナ</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>1480</v>
+      </c>
+      <c r="G629" t="n">
+        <v>0</v>
+      </c>
+      <c r="H629" t="b">
+        <v>0</v>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211207443</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>1207663027</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>rusion</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>白ワキ姫 わきの黒ずみに 塗ってぽろぽろワキ美人 リベルタ</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>ヒメコト</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>1370</v>
+      </c>
+      <c r="G630" t="n">
+        <v>1</v>
+      </c>
+      <c r="H630" t="b">
+        <v>0</v>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207663027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J627"/>
+  <autoFilter ref="A1:J630"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 97, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$631</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$632</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J631"/>
+  <dimension ref="A1:J632"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26201,8 +26201,49 @@
         </is>
       </c>
     </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>1208501534</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>zagzag</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>[ポスト投函][ロゼット]ロゼット洗顔サボン スムースウォッシュ 詰替え 170ml[2個セット]</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>ロゼット</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>1562</v>
+      </c>
+      <c r="G632" t="n">
+        <v>1</v>
+      </c>
+      <c r="H632" t="b">
+        <v>0</v>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208501534</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J631"/>
+  <autoFilter ref="A1:J632"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 103, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$635</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$637</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J635"/>
+  <dimension ref="A1:J637"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26365,8 +26365,90 @@
         </is>
       </c>
     </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>1099343162</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>noin_beauty</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>【夏のヘアケア福袋】by Yarden バイヤーデン ダメージケア シャンプー2個&amp;amp;トリートメント2個&amp;amp;スカルプリリーフセラムセット</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>by yarden</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G636" t="n">
+        <v>4</v>
+      </c>
+      <c r="H636" t="b">
+        <v>0</v>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1099343162</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>1201956239</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>noin_beauty</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>【ヘアセラム】by Yarden バイヤーデン スカルプ リリーフ セラム</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>by yarden</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G637" t="n">
+        <v>1</v>
+      </c>
+      <c r="H637" t="b">
+        <v>0</v>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201956239</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J635"/>
+  <autoFilter ref="A1:J637"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 104, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$637</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$638</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J637"/>
+  <dimension ref="A1:J638"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26447,8 +26447,49 @@
         </is>
       </c>
     </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>1209047946</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>offon</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>【公式】お試しセット / ミニサイズ セット (ボディウォッシュ 50g + ボディローション 50g) トラベルセット 敏感肌 鎮静 背中ニキビ 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>OFFON</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G638" t="n">
+        <v>0</v>
+      </c>
+      <c r="H638" t="b">
+        <v>0</v>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209047946</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J637"/>
+  <autoFilter ref="A1:J638"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 106, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$638</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$642</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J638"/>
+  <dimension ref="A1:J642"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26488,8 +26488,172 @@
         </is>
       </c>
     </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>1163878412</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>maisonlexia</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>マイバイオーム　ナリッシュ トリートメント　300g　ヘアトリートメント ［ 植物 × 乳酸菌 マイクロバイオームケア ］</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>MAISON LEXIA</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G639" t="n">
+        <v>3</v>
+      </c>
+      <c r="H639" t="b">
+        <v>0</v>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163878412</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>1163878364</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>maisonlexia</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>マイバイオーム スカルプケア シャンプー 300mL ［ 植物 × 乳酸菌 マイクロバイオームケア ］</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>MAISON LEXIA</t>
+        </is>
+      </c>
+      <c r="F640" t="n">
+        <v>3850</v>
+      </c>
+      <c r="G640" t="n">
+        <v>7</v>
+      </c>
+      <c r="H640" t="b">
+        <v>0</v>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163878364</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>1128829845</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>drscalp</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>【公式】Dr.Scalp スカルプトリートメント 頭皮ケア ダメージヘア 超乾燥毛 集中補修 韓国ヴィーガン認証 ノンシリコン サロン品質</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>DR.SCALP</t>
+        </is>
+      </c>
+      <c r="F641" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G641" t="n">
+        <v>4</v>
+      </c>
+      <c r="H641" t="b">
+        <v>0</v>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1128829845</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>1050605219</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>drscalp</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>【公式】スカルプシャンプー 女性用 抜け毛対策 頭皮ケア 頭皮シャンプー 韓国 人気 シャンプー ビーガン成分</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>DR.SCALP</t>
+        </is>
+      </c>
+      <c r="F642" t="n">
+        <v>1860</v>
+      </c>
+      <c r="G642" t="n">
+        <v>9</v>
+      </c>
+      <c r="H642" t="b">
+        <v>0</v>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1050605219</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J638"/>
+  <autoFilter ref="A1:J642"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 107, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$642</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$644</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J642"/>
+  <dimension ref="A1:J644"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26652,8 +26652,90 @@
         </is>
       </c>
     </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>1083807374</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>vitalism</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>【公式】スカルプシャンプー＆コンディショナー トライアルパウチ4個セット WOMEN</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>バイタリズム</t>
+        </is>
+      </c>
+      <c r="F643" t="n">
+        <v>980</v>
+      </c>
+      <c r="G643" t="n">
+        <v>2</v>
+      </c>
+      <c r="H643" t="b">
+        <v>0</v>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083807374</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>915021168</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>vitalism</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>【公式】スカルプケア シャンプー＆コンディショナー セット for MEN 各350ml</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>バイタリズム</t>
+        </is>
+      </c>
+      <c r="F644" t="n">
+        <v>5277</v>
+      </c>
+      <c r="G644" t="n">
+        <v>4</v>
+      </c>
+      <c r="H644" t="b">
+        <v>0</v>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=915021168</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J642"/>
+  <autoFilter ref="A1:J644"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 109, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$644</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$645</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J644"/>
+  <dimension ref="A1:J645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26734,8 +26734,49 @@
         </is>
       </c>
     </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>1169651049</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>dermafume_official</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>【公式】ワイン＆ビール酵母2X スカルプケア トリートメント 520ml [高い洗浄力/泡立ち/すすぎやすい/保湿ケア/髪がサラサラ/香りが良い]</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Derma:fume</t>
+        </is>
+      </c>
+      <c r="F645" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G645" t="n">
+        <v>0</v>
+      </c>
+      <c r="H645" t="b">
+        <v>0</v>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169651049</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J644"/>
+  <autoFilter ref="A1:J645"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 110, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$645</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$646</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J645"/>
+  <dimension ref="A1:J646"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26775,8 +26775,49 @@
         </is>
       </c>
     </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>987579304</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>wowmedical</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>スカルプシャンプー メンズ 大容量 500ml 薬用 男性 男性用 オーガニック アミノ酸系 フケ かゆみ 頭皮ケア 無添加 医薬部外品</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>SUPER SAIYA</t>
+        </is>
+      </c>
+      <c r="F646" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G646" t="n">
+        <v>0</v>
+      </c>
+      <c r="H646" t="b">
+        <v>0</v>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=987579304</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J645"/>
+  <autoFilter ref="A1:J646"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 111, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$646</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$650</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J646"/>
+  <dimension ref="A1:J650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26816,8 +26816,172 @@
         </is>
       </c>
     </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>1061832722</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>modest</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>フケ かゆみ 頭皮臭 頭皮湿疹 脂漏性対策 リバラン 頭皮ケアシャンプー アミノ酸 医薬部外品 ノンシリコン シトラスの香り ReBALAN（スカルプシャンプー1本）250mL</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>modest pharmaceutical</t>
+        </is>
+      </c>
+      <c r="F647" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G647" t="n">
+        <v>9</v>
+      </c>
+      <c r="H647" t="b">
+        <v>0</v>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1061832722</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>1061662934</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>modest</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>医薬部外品 フケ かゆみ 脂漏性の対策に リバラン シャンプートリートメントセット ノンシリコン アミノ酸 弱酸性 低刺激 250ml/250g</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>modest pharmaceutical</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>6780</v>
+      </c>
+      <c r="G648" t="n">
+        <v>7</v>
+      </c>
+      <c r="H648" t="b">
+        <v>0</v>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1061662934</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>1061466807</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>modest</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>お風呂で使える BathVio デリケートゾーン お尻 脇 お腹など 全身OK 黒ずみケア クリーム 保湿効果 乾燥対策 男女兼用 レディース メンズ バスビオ 医薬部外品 2本セット 1本25g</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>modest pharmaceutical</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>3740</v>
+      </c>
+      <c r="G649" t="n">
+        <v>6</v>
+      </c>
+      <c r="H649" t="b">
+        <v>0</v>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1061466807</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>1061344640</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>modest</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>お風呂で使える BathVio デリケートゾーン お尻 脇 お腹など 全身OK 黒ずみケア クリーム 保湿効果 乾燥対策 男女兼用［レディース メンズ］ バスビオ 医薬部外品 1本 25g</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>modest pharmaceutical</t>
+        </is>
+      </c>
+      <c r="F650" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G650" t="n">
+        <v>8</v>
+      </c>
+      <c r="H650" t="b">
+        <v>0</v>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1061344640</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J646"/>
+  <autoFilter ref="A1:J650"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 115, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$650</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$656</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J650"/>
+  <dimension ref="A1:J656"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26980,8 +26980,254 @@
         </is>
       </c>
     </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>1162198725</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>hairplus_official</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>【公式】オフレッシーディープハーバルスカルプシャンプー700ml /フケ・かゆみ 対策 /ハーブ 配合/クール感/メントール</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>ヘアプラス</t>
+        </is>
+      </c>
+      <c r="F651" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G651" t="n">
+        <v>2</v>
+      </c>
+      <c r="H651" t="b">
+        <v>0</v>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162198725</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>1157285015</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>hairplus_official</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>【公式】オフレッシュディープハーバルスカルプ頭皮ウォータースケーラー200ml /フケ・かゆみ 対策 /ハーブ 配合/クール感/メントール</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>ヘアプラス</t>
+        </is>
+      </c>
+      <c r="F652" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G652" t="n">
+        <v>3</v>
+      </c>
+      <c r="H652" t="b">
+        <v>0</v>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157285015</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>1204563857</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>ratedgreenjp</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>【クーポン使って8/10～8/15はお得！シャンプーサンプル付き・選べる2種セット】スカルプパック50ml×2パック 1+1 頭皮ケア ヘッドスパ トリートメント 韓国ヘアパック 美髪改善</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>RATED GREEN</t>
+        </is>
+      </c>
+      <c r="F653" t="n">
+        <v>999</v>
+      </c>
+      <c r="G653" t="n">
+        <v>2</v>
+      </c>
+      <c r="H653" t="b">
+        <v>0</v>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204563857</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>1185930477</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>ratedgreenjp</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>デタングリングパフュームヘアミスト80ml　1本（3種類の香りの中からお選びください）　ヘアコロン　香水　保湿</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>RATED GREEN</t>
+        </is>
+      </c>
+      <c r="F654" t="n">
+        <v>3564</v>
+      </c>
+      <c r="G654" t="n">
+        <v>0</v>
+      </c>
+      <c r="H654" t="b">
+        <v>0</v>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185930477</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>1170189170</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>ratedgreenjp</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>【8月のおすすめ】リアルマリーピュリファイングスカルプスケーラー200ml　夏にぴったり　すっきり爽快　ハーブの香り　やさしく洗浄　潤い　保湿　鎮静</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>RATED GREEN</t>
+        </is>
+      </c>
+      <c r="F655" t="n">
+        <v>2534</v>
+      </c>
+      <c r="G655" t="n">
+        <v>5</v>
+      </c>
+      <c r="H655" t="b">
+        <v>0</v>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170189170</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>1085996682</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>ratedgreenjp</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>【洗い流さないトリートメント 貴方の髪に潤いを与える】 リアルシア シアバター プロテインリチャージ トリートメント（アウトバス用） 50ml お試し 潤い ヘアケア</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>RATED GREEN</t>
+        </is>
+      </c>
+      <c r="F656" t="n">
+        <v>1452</v>
+      </c>
+      <c r="G656" t="n">
+        <v>3</v>
+      </c>
+      <c r="H656" t="b">
+        <v>0</v>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1085996682</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J650"/>
+  <autoFilter ref="A1:J656"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 116, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$656</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$659</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J656"/>
+  <dimension ref="A1:J659"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27226,8 +27226,131 @@
         </is>
       </c>
     </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>1172490062</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>mintree</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>【公式】ディープダメージ ヘアパック 430ml</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>mintree</t>
+        </is>
+      </c>
+      <c r="F657" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G657" t="n">
+        <v>2</v>
+      </c>
+      <c r="H657" t="b">
+        <v>0</v>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172490062</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>1172488759</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>mintree</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>【公式】スカルプシャンプー 500ml</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>mintree</t>
+        </is>
+      </c>
+      <c r="F658" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G658" t="n">
+        <v>5</v>
+      </c>
+      <c r="H658" t="b">
+        <v>0</v>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172488759</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>1169644916</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>mintree</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>【公式】炭酸バブル 頭皮クレンジング 30g 大容量 スカルプスケーラー</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>mintree</t>
+        </is>
+      </c>
+      <c r="F659" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G659" t="n">
+        <v>7</v>
+      </c>
+      <c r="H659" t="b">
+        <v>0</v>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169644916</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J656"/>
+  <autoFilter ref="A1:J659"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 118, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$659</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$663</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J659"/>
+  <dimension ref="A1:J663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27349,8 +27349,172 @@
         </is>
       </c>
     </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>1213124167</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>韓国正規品 ローズマリー PDRN スカルプセラム 100ml 頭皮ケア ブラシ美容液</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>アロマティカ</t>
+        </is>
+      </c>
+      <c r="F660" t="n">
+        <v>3811</v>
+      </c>
+      <c r="G660" t="n">
+        <v>0</v>
+      </c>
+      <c r="H660" t="b">
+        <v>0</v>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213124167</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>1213317338</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>【選べる4種】敏感肌スキンケア 保湿乳液・洗顔料・化粧水・高保湿バーム 60ml～180ml 韓国正規品 韓国直送</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>2366</v>
+      </c>
+      <c r="G661" t="n">
+        <v>0</v>
+      </c>
+      <c r="H661" t="b">
+        <v>0</v>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213317338</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>1213260537</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>韓国正規品 リニューアル MLE保湿ローション 120ml／200ml 敏感肌 乾燥肌 ベビー 全身 肌バリア 韓国直送</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F662" t="n">
+        <v>2465</v>
+      </c>
+      <c r="G662" t="n">
+        <v>1</v>
+      </c>
+      <c r="H662" t="b">
+        <v>0</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213260537</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>1179712953</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>kabushikigaishairis</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>ヴァセリン オリジナルピュアスキンジェリー 40g　保湿　ボディクリーム　ハンドクリーム</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F663" t="n">
+        <v>660</v>
+      </c>
+      <c r="G663" t="n">
+        <v>5</v>
+      </c>
+      <c r="H663" t="b">
+        <v>0</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179712953</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J659"/>
+  <autoFilter ref="A1:J663"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 119, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$663</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$664</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J663"/>
+  <dimension ref="A1:J664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27513,8 +27513,49 @@
         </is>
       </c>
     </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>1197142140</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>cread_inc</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>プロ業務用 UVスプレー氷冷 日焼け止め 冷感 冷却 スプレー 日焼け止め クール 紫外線対策 敏感肌 UVスプレー 全身 顔 髪 頭皮 体 保湿</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>ヤーマン</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>1760</v>
+      </c>
+      <c r="G664" t="n">
+        <v>0</v>
+      </c>
+      <c r="H664" t="b">
+        <v>0</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197142140</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J663"/>
+  <autoFilter ref="A1:J664"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 120, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$664</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$666</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J664"/>
+  <dimension ref="A1:J666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27554,8 +27554,90 @@
         </is>
       </c>
     </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>1117071489</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>shearts</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>【公式】 スカルプブラシ ワールドプレミアムロング ギフトセット シャンプーブラシ ヘアケアブラシ 頭皮マッサージブラシ ヘアブラシ スカルプケア 頭皮ケア 女性 男性 誕生日</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>エス・ハート・エス</t>
+        </is>
+      </c>
+      <c r="F665" t="n">
+        <v>8800</v>
+      </c>
+      <c r="G665" t="n">
+        <v>8</v>
+      </c>
+      <c r="H665" t="b">
+        <v>0</v>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117071489</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>1175522511</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>skym-store</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>スカルプブラシ ワールドプレミアム ロング ゴールド 頭皮ケア</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>エス・ハート・エス</t>
+        </is>
+      </c>
+      <c r="F666" t="n">
+        <v>5200</v>
+      </c>
+      <c r="G666" t="n">
+        <v>2</v>
+      </c>
+      <c r="H666" t="b">
+        <v>0</v>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175522511</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J664"/>
+  <autoFilter ref="A1:J666"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 124, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$666</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$667</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J666"/>
+  <dimension ref="A1:J667"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27636,8 +27636,49 @@
         </is>
       </c>
     </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>1205678472</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>violus</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>スカルプブラシ 頭皮ブラシ シャンプーブラシ 頭皮マッサージ 頭皮ケア シリコンブラシ 血行促進 お風呂</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>VIOLUS</t>
+        </is>
+      </c>
+      <c r="F667" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G667" t="n">
+        <v>1</v>
+      </c>
+      <c r="H667" t="b">
+        <v>0</v>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205678472</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J666"/>
+  <autoFilter ref="A1:J667"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 127, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$667</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$668</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J667"/>
+  <dimension ref="A1:J668"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27677,8 +27677,49 @@
         </is>
       </c>
     </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>1063333400</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>shinbee</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>ココスター KOCOSTAR ピーチリップデュオデュオ 43g 桃 リップ リップスクラブ オイル クリーム リップバーム しっとりした唇 唇の角質取り 韓国コスメ「 乾燥 保湿 」 美容 唇</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>ココスター</t>
+        </is>
+      </c>
+      <c r="F668" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G668" t="n">
+        <v>1</v>
+      </c>
+      <c r="H668" t="b">
+        <v>0</v>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1063333400</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J667"/>
+  <autoFilter ref="A1:J668"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 128, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$668</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$670</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J668"/>
+  <dimension ref="A1:J670"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27718,8 +27718,90 @@
         </is>
       </c>
     </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>1158602279</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>ma-t-ma-to</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>VENUS(ヴィーナス) カミソリ 剃刀 女性用 レディース つるすべ肌へ 本体 替刃 2個 エンブレイス</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Embrace</t>
+        </is>
+      </c>
+      <c r="F669" t="n">
+        <v>1188</v>
+      </c>
+      <c r="G669" t="n">
+        <v>1</v>
+      </c>
+      <c r="H669" t="b">
+        <v>0</v>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158602279</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>1011438226</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>infinitycc</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>【 正規品 】 サブリミック アデノバイタル スカルプパワーショット 480ml リフィル （詰替用） 【２個】 ボリュームやハリやコシのない髪用</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>資生堂プロフェッショナル</t>
+        </is>
+      </c>
+      <c r="F670" t="n">
+        <v>27679</v>
+      </c>
+      <c r="G670" t="n">
+        <v>0</v>
+      </c>
+      <c r="H670" t="b">
+        <v>0</v>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1011438226</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J668"/>
+  <autoFilter ref="A1:J670"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 129)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$670</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$671</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J670"/>
+  <dimension ref="A1:J671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27800,8 +27800,49 @@
         </is>
       </c>
     </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>1159489284</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>essencher</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>【韓国人気】蜜蝋樹脂かっさマッサージャー 3点セット/頭皮/ヘアケア/全身/リンパ/肩こり/小顔/むくみ解消/リフトアップ/セルフケア</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>ESSENCHER</t>
+        </is>
+      </c>
+      <c r="F671" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G671" t="n">
+        <v>1</v>
+      </c>
+      <c r="H671" t="b">
+        <v>0</v>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159489284</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J670"/>
+  <autoFilter ref="A1:J671"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 130, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$671</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$674</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J671"/>
+  <dimension ref="A1:J674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27841,8 +27841,131 @@
         </is>
       </c>
     </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>1209229612</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>NATSUKISHOP</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>スキン コンダクター 60g</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>カネボウ</t>
+        </is>
+      </c>
+      <c r="F672" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G672" t="n">
+        <v>1</v>
+      </c>
+      <c r="H672" t="b">
+        <v>0</v>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209229612</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>1215334317</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>NATSUKISHOP</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>インシスト ラメラ UVダーマテクトエッセンス</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>FAITH</t>
+        </is>
+      </c>
+      <c r="F673" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G673" t="n">
+        <v>0</v>
+      </c>
+      <c r="H673" t="b">
+        <v>0</v>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215334317</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>1210143577</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>NATSUKISHOP</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>DRX AZAクリアクリーム</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>ロート製薬</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G674" t="n">
+        <v>1</v>
+      </c>
+      <c r="H674" t="b">
+        <v>0</v>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210143577</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J671"/>
+  <autoFilter ref="A1:J674"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 132, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$674</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$679</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J674"/>
+  <dimension ref="A1:J679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27964,8 +27964,213 @@
         </is>
       </c>
     </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>1179833428</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>loveForGreen</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>カカジェントポアリアクター 40mL毛穴ケア美容液・皮脂バランス・引き締め・韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>BRAVITY</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>3210</v>
+      </c>
+      <c r="G675" t="n">
+        <v>4</v>
+      </c>
+      <c r="H675" t="b">
+        <v>0</v>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179833428</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>1179831868</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>loveForGreen</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>モイスチャライジングアンプル 40mL高保湿美容液・乾燥肌・ツヤ肌サポート・韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>BRAVITY</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>3210</v>
+      </c>
+      <c r="G676" t="n">
+        <v>0</v>
+      </c>
+      <c r="H676" t="b">
+        <v>0</v>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179831868</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>1179833401</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>loveForGreen</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>ステムセルデイリーオールインワン 120g高保湿×ハリケア・時短スキンケア・敏感肌にも・韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>BRAVITY</t>
+        </is>
+      </c>
+      <c r="F677" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G677" t="n">
+        <v>0</v>
+      </c>
+      <c r="H677" t="b">
+        <v>0</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179833401</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>1200407108</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>loveForGreen</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>アイアイスマスク 50mL 目元ケア 保湿ケア ひんやり使用感 うるおい補給 敏感肌対応 アイケアクリーム</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>MBK</t>
+        </is>
+      </c>
+      <c r="F678" t="n">
+        <v>19320</v>
+      </c>
+      <c r="G678" t="n">
+        <v>0</v>
+      </c>
+      <c r="H678" t="b">
+        <v>0</v>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200407108</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>1179666444</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>loveForGreen</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>テラ シルキーベルベットクリーム 50g 韓国 保湿クリーム 乾燥肌 敏感肌向け</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>PAMSIBC</t>
+        </is>
+      </c>
+      <c r="F679" t="n">
+        <v>5180</v>
+      </c>
+      <c r="G679" t="n">
+        <v>9</v>
+      </c>
+      <c r="H679" t="b">
+        <v>0</v>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179666444</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J674"/>
+  <autoFilter ref="A1:J679"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 133, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$679</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$683</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J679"/>
+  <dimension ref="A1:J683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28169,8 +28169,172 @@
         </is>
       </c>
     </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>1195754504</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>hnhcorp</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>【国内発送】【100枚セット】ワンデーマスク 40ml 人気の全5種を20枚ずつ楽しめる / 保湿 / 栄養 / 乾燥 / フェイスパック / ダーマル / Dermal / Let’s Skin</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>DERMAL</t>
+        </is>
+      </c>
+      <c r="F680" t="n">
+        <v>5720</v>
+      </c>
+      <c r="G680" t="n">
+        <v>0</v>
+      </c>
+      <c r="H680" t="b">
+        <v>0</v>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195754504</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>1182953283</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>hnhcorp</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>【国内発送】【20枚セット】ブースターマスク 25ml 人気の全5種類 / 保湿 / 栄養 / 乾燥 / シートマスク / フェイスパック / ダーマル / Dermal / Let’s Skin</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Dermal+</t>
+        </is>
+      </c>
+      <c r="F681" t="n">
+        <v>3520</v>
+      </c>
+      <c r="G681" t="n">
+        <v>1</v>
+      </c>
+      <c r="H681" t="b">
+        <v>0</v>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182953283</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>1183653339</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>hnhcorp</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>【国内発送】【4個セット】ホワイトミルククリーム 50ml / 保湿 / 栄養 / 下地 / トーンアップ / 香り / 全身使える / Let’s Skin / Dermal / ダーマル</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>Let's Skin</t>
+        </is>
+      </c>
+      <c r="F682" t="n">
+        <v>4250</v>
+      </c>
+      <c r="G682" t="n">
+        <v>5</v>
+      </c>
+      <c r="H682" t="b">
+        <v>0</v>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183653339</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>1183014299</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>hnhcorp</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>【国内発送】【1個】ホワイトミルククリーム 50ml / 保湿 / 栄養 / 下地 / トーンアップ / 香り / 全身使える / Let’s Skin / Dermal / ダーマル</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Let's Skin</t>
+        </is>
+      </c>
+      <c r="F683" t="n">
+        <v>1518</v>
+      </c>
+      <c r="G683" t="n">
+        <v>1</v>
+      </c>
+      <c r="H683" t="b">
+        <v>0</v>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183014299</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J679"/>
+  <autoFilter ref="A1:J683"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 134, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$683</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$687</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J683"/>
+  <dimension ref="A1:J687"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28333,8 +28333,172 @@
         </is>
       </c>
     </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>1203559783</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>【公式】【選べるナノショットハイドロゲルマスク特集】ビタコラーゲン・ポアコラーゲン・カーミングコラーゲン・リアルスキンフィットコラーゲン 10枚入り 密着保湿 フェイスパック 韓国</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F684" t="n">
+        <v>6520</v>
+      </c>
+      <c r="G684" t="n">
+        <v>3</v>
+      </c>
+      <c r="H684" t="b">
+        <v>0</v>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203559783</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>1202277840</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>【公式】ビタコラーゲン ナノショット ハイドロゲルマスク, 5枚 3種コラーゲン 10種ビタミン 超低分子100Da 浸透ケア ツヤ 透明感 ハリ 毛穴ケア 保湿 密着 フェイスパック 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F685" t="n">
+        <v>3260</v>
+      </c>
+      <c r="G685" t="n">
+        <v>1</v>
+      </c>
+      <c r="H685" t="b">
+        <v>0</v>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202277840</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>1203576241</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>【公式】カーミング コラーゲン ナノショット ハイドロゲルマスク 5枚 /超低分子100Da / CICA / カーミングコンプレックス / 肌荒れ対策 / フェイスパック / 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F686" t="n">
+        <v>3260</v>
+      </c>
+      <c r="G686" t="n">
+        <v>0</v>
+      </c>
+      <c r="H686" t="b">
+        <v>0</v>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203576241</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>1202308494</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>【公式】ポアコラーゲン ナノショット ハイドロゲルマスク 5枚 /超低分子100Da / ポアコンプレックス /毛穴ケア / キメ / ハリ/ 保湿 / 密着 / フェイスパック / 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F687" t="n">
+        <v>3260</v>
+      </c>
+      <c r="G687" t="n">
+        <v>0</v>
+      </c>
+      <c r="H687" t="b">
+        <v>0</v>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202308494</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J683"/>
+  <autoFilter ref="A1:J687"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 136, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$687</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$688</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J687"/>
+  <dimension ref="A1:J688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28497,8 +28497,49 @@
         </is>
       </c>
     </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>1211968720</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>sumuadi</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>【公式】マリンTECA B5 セラム 30ml 美容液 高濃度パンテノール・TECA配合 海ぶどうエキス配合 ダメージケア 肌バリアケア 敏感肌 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>スムアディ</t>
+        </is>
+      </c>
+      <c r="F688" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G688" t="n">
+        <v>0</v>
+      </c>
+      <c r="H688" t="b">
+        <v>0</v>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211968720</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J687"/>
+  <autoFilter ref="A1:J688"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 137, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$688</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$689</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J688"/>
+  <dimension ref="A1:J689"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28538,8 +28538,49 @@
         </is>
       </c>
     </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>1138107008</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>sudii</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>【国内発送】【選べる1個】ボディウォッシュ 488ml [ヒノキ / ベルガモット] 【正規品】 BODYWASH 保湿 全身ケア 韓国 人気 香り しっとり なめらか</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>MARMAR;D</t>
+        </is>
+      </c>
+      <c r="F689" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G689" t="n">
+        <v>1</v>
+      </c>
+      <c r="H689" t="b">
+        <v>0</v>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138107008</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J688"/>
+  <autoFilter ref="A1:J689"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 138, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$689</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$690</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J689"/>
+  <dimension ref="A1:J690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28579,8 +28579,49 @@
         </is>
       </c>
     </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>1204620083</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>ELIBYTH</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>【ベタつきにくく・うるおい満たすコア保湿セラム】 デイリーハーモニー コアバランスセラム 30mL 韓国コスメ 保湿美容液 敏感肌 低刺激 乾燥肌 バリアケア</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>ELIBYTH</t>
+        </is>
+      </c>
+      <c r="F690" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G690" t="n">
+        <v>2</v>
+      </c>
+      <c r="H690" t="b">
+        <v>0</v>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204620083</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J689"/>
+  <autoFilter ref="A1:J690"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 139, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$690</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$691</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J690"/>
+  <dimension ref="A1:J691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28620,8 +28620,49 @@
         </is>
       </c>
     </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>1167411378</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>mediinlab</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>メディインラボ A5 クリーム 50g /6種ペプチド /NMN /EGF</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>MEDI IN LAB</t>
+        </is>
+      </c>
+      <c r="F691" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G691" t="n">
+        <v>0</v>
+      </c>
+      <c r="H691" t="b">
+        <v>0</v>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167411378</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J690"/>
+  <autoFilter ref="A1:J691"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 140, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$691</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$694</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J691"/>
+  <dimension ref="A1:J694"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28661,8 +28661,131 @@
         </is>
       </c>
     </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>1214025378</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>mitomojp</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>MITOMO カタツムリ フェイシャルエッセンスマスク 60枚[MTSS00516-E-6x006]</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>MITOMO</t>
+        </is>
+      </c>
+      <c r="F692" t="n">
+        <v>4212</v>
+      </c>
+      <c r="G692" t="n">
+        <v>0</v>
+      </c>
+      <c r="H692" t="b">
+        <v>0</v>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214025378</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>1214025265</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>mitomojp</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>MITOMO アロエ フェイシャルエッセンスマスク 30枚[MTSS0512-C-4Jx003]</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>MITOMO</t>
+        </is>
+      </c>
+      <c r="F693" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G693" t="n">
+        <v>0</v>
+      </c>
+      <c r="H693" t="b">
+        <v>0</v>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214025265</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>1198204681</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>credion</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>シミ・そばかすケア 5点セット</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F694" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G694" t="n">
+        <v>0</v>
+      </c>
+      <c r="H694" t="b">
+        <v>0</v>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198204681</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J691"/>
+  <autoFilter ref="A1:J694"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 142, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$694</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$697</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J694"/>
+  <dimension ref="A1:J697"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28784,8 +28784,131 @@
         </is>
       </c>
     </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>1202064382</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>thome</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>【残りわずか！】トーム コラーゲンブーストアンプル50g／PDRNサーモン／超音波伝道ジェル状／美顔器との相性抜群／保湿 肌バリアケア</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>THOME</t>
+        </is>
+      </c>
+      <c r="F695" t="n">
+        <v>5935</v>
+      </c>
+      <c r="G695" t="n">
+        <v>4</v>
+      </c>
+      <c r="H695" t="b">
+        <v>0</v>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202064382</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>1202031681</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>thome</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>【THOME公式】トーム ペプチドブーストアンプル50g／超音波伝道ジェル状／美顔器との相性抜群／ハリ・キメケア・シワ</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>THOME</t>
+        </is>
+      </c>
+      <c r="F696" t="n">
+        <v>6300</v>
+      </c>
+      <c r="G696" t="n">
+        <v>6</v>
+      </c>
+      <c r="H696" t="b">
+        <v>0</v>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202031681</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>1202025883</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>thome</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>【THOME公式】トーム ヒアルロン ブーストアンプル50g／スピキュール入り／超音波伝道ジェル状／美顔器との相性抜群／ツヤ・潤いケア</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>THOME</t>
+        </is>
+      </c>
+      <c r="F697" t="n">
+        <v>6300</v>
+      </c>
+      <c r="G697" t="n">
+        <v>1</v>
+      </c>
+      <c r="H697" t="b">
+        <v>0</v>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202025883</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J694"/>
+  <autoFilter ref="A1:J697"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 143, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$697</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$699</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J697"/>
+  <dimension ref="A1:J699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28907,8 +28907,90 @@
         </is>
       </c>
     </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>1195863212</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>beautywitch</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>コホンジン スキンベース 130ml</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>KOHONJIN</t>
+        </is>
+      </c>
+      <c r="F698" t="n">
+        <v>15939</v>
+      </c>
+      <c r="G698" t="n">
+        <v>0</v>
+      </c>
+      <c r="H698" t="b">
+        <v>0</v>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195863212</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>1129524636</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>theraum</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>シークレット エッセンス EX 1ml x 120枚 サンプル/韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F699" t="n">
+        <v>2459</v>
+      </c>
+      <c r="G699" t="n">
+        <v>3</v>
+      </c>
+      <c r="H699" t="b">
+        <v>0</v>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1129524636</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J697"/>
+  <autoFilter ref="A1:J699"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 145, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$699</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$700</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J699"/>
+  <dimension ref="A1:J700"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28989,8 +28989,49 @@
         </is>
       </c>
     </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>952985957</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>yakyu21</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>白玉生明鏡止水（ミョンキョンジス） HMFリンクル＆ホワイトケア（単品） 60ml</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>白玉生</t>
+        </is>
+      </c>
+      <c r="F700" t="n">
+        <v>14800</v>
+      </c>
+      <c r="G700" t="n">
+        <v>2</v>
+      </c>
+      <c r="H700" t="b">
+        <v>0</v>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J700" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=952985957</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J699"/>
+  <autoFilter ref="A1:J700"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 146, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$700</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$703</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J700"/>
+  <dimension ref="A1:J703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29030,8 +29030,131 @@
         </is>
       </c>
     </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>1036526420</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>pegasus</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>【送料無料】男女美 エフィーテシャンプー トリートメント Efire リンス 700ml オーガニック DANJOBI ダンジョビ 高麗人参</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Danjobi</t>
+        </is>
+      </c>
+      <c r="F701" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G701" t="n">
+        <v>4</v>
+      </c>
+      <c r="H701" t="b">
+        <v>0</v>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J701" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1036526420</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>1203337478</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>gyeolhaus</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>【6枚】 オリーブ&amp;amp;レモン ツヤ肌ハイドロゲルマスク 3枚入り（2箱）</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>GYEOL HAUS</t>
+        </is>
+      </c>
+      <c r="F702" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G702" t="n">
+        <v>0</v>
+      </c>
+      <c r="H702" t="b">
+        <v>0</v>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J702" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203337478</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>1185473716</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>gyeolhaus</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>【1個】 エクストリームアイスティーツリーパッド70枚入り</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>GYEOL HAUS</t>
+        </is>
+      </c>
+      <c r="F703" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G703" t="n">
+        <v>1</v>
+      </c>
+      <c r="H703" t="b">
+        <v>0</v>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J703" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185473716</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J700"/>
+  <autoFilter ref="A1:J703"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 41, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$725</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$726</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J725"/>
+  <dimension ref="A1:J726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30055,8 +30055,49 @@
         </is>
       </c>
     </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>1208838957</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>halomy</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>ローぜリティクス グロウレイヤーアンプル 30mL 美容液</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>halomy</t>
+        </is>
+      </c>
+      <c r="F726" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G726" t="n">
+        <v>4</v>
+      </c>
+      <c r="H726" t="b">
+        <v>0</v>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J726" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208838957</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J725"/>
+  <autoFilter ref="A1:J726"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 46, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$733</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$735</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J733"/>
+  <dimension ref="A1:J735"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30383,8 +30383,90 @@
         </is>
       </c>
     </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>1192893922</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>babaco</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>【公式】マルチサニー バーム 10g SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>ババコ</t>
+        </is>
+      </c>
+      <c r="F734" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G734" t="n">
+        <v>2</v>
+      </c>
+      <c r="H734" t="b">
+        <v>0</v>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J734" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192893922</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>1188332484</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>babaco</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>【公式】オールインワン水光サンクリーム 50ml SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>ババコ</t>
+        </is>
+      </c>
+      <c r="F735" t="n">
+        <v>4070</v>
+      </c>
+      <c r="G735" t="n">
+        <v>7</v>
+      </c>
+      <c r="H735" t="b">
+        <v>0</v>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J735" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188332484</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J733"/>
+  <autoFilter ref="A1:J735"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 65, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$746</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$750</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J746"/>
+  <dimension ref="A1:J750"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30916,8 +30916,172 @@
         </is>
       </c>
     </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>1213124574</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>shade02</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>【満足度No.1】【pffeel 公式】お試しサイズ登場！ コラーゲン ラッピング マスク 7g×3個 剥がすフェイスマスク 垂れない シートマスク フェイスパック パック シート 保湿 コラーゲン</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>p'ffeel</t>
+        </is>
+      </c>
+      <c r="F747" t="n">
+        <v>1320</v>
+      </c>
+      <c r="G747" t="n">
+        <v>0</v>
+      </c>
+      <c r="H747" t="b">
+        <v>0</v>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J747" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213124574</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>1215704916</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Myh</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>on:myskin オンマイスキン ハーブピーリングソリューション フェイス用 4ml × 8個 ヨミテ メール便送料無料NYH / オンマイピーリング顔S02-02 / OMSHPF-01P</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>on:myskin</t>
+        </is>
+      </c>
+      <c r="F748" t="n">
+        <v>5380</v>
+      </c>
+      <c r="G748" t="n">
+        <v>0</v>
+      </c>
+      <c r="H748" t="b">
+        <v>0</v>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J748" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215704916</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>1215185623</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Myh</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>ユリイロ YURiiRO インティメイト＆ボディオイル チェリーブロッサム 100ml E-seeds メール便送料無料NYH / ユリイロオイルCBS01-02 / YRIOCB-01P</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>YURiiRO</t>
+        </is>
+      </c>
+      <c r="F749" t="n">
+        <v>6380</v>
+      </c>
+      <c r="G749" t="n">
+        <v>0</v>
+      </c>
+      <c r="H749" t="b">
+        <v>0</v>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215185623</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>1215633377</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Myh</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>ヴィオテラスC+ クリアセラム VIOTERAS Cプラス [ リニューアル最新版 ] 20ml 美容液 メール便送料無料NYH / ヴィオテラスC20mlS06-01 / VOTRSC-01P</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>VIOTERAS</t>
+        </is>
+      </c>
+      <c r="F750" t="n">
+        <v>8680</v>
+      </c>
+      <c r="G750" t="n">
+        <v>0</v>
+      </c>
+      <c r="H750" t="b">
+        <v>0</v>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215633377</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J746"/>
+  <autoFilter ref="A1:J750"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 17, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$753</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$757</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J753"/>
+  <dimension ref="A1:J757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31203,8 +31203,172 @@
         </is>
       </c>
     </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>1010366811</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>cosmedefrance</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>デトランスピラン　ノーマル肌用　6個セット　制汗剤</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>エティアキシル</t>
+        </is>
+      </c>
+      <c r="F754" t="n">
+        <v>11500</v>
+      </c>
+      <c r="G754" t="n">
+        <v>2</v>
+      </c>
+      <c r="H754" t="b">
+        <v>0</v>
+      </c>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J754" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1010366811</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>1155301814</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>cosmedefrance</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>デトランスピラン　普通肌用　15ml　1個</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>エティアキシル</t>
+        </is>
+      </c>
+      <c r="F755" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G755" t="n">
+        <v>0</v>
+      </c>
+      <c r="H755" t="b">
+        <v>0</v>
+      </c>
+      <c r="I755" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J755" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155301814</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>1010397752</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>cosmedefrance</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>トリートメント　デトランスピラン　ローション　足用　敏感肌用 100ml 足の汗対策　制汗剤</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>エティアキシル</t>
+        </is>
+      </c>
+      <c r="F756" t="n">
+        <v>4480</v>
+      </c>
+      <c r="G756" t="n">
+        <v>3</v>
+      </c>
+      <c r="H756" t="b">
+        <v>0</v>
+      </c>
+      <c r="I756" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J756" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1010397752</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>1010367357</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>cosmedefrance</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>デトランスピラン　コンフォート　3個セット　大量発汗を調整　超乾燥肌向け　制汗剤</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>エティアキシル</t>
+        </is>
+      </c>
+      <c r="F757" t="n">
+        <v>6380</v>
+      </c>
+      <c r="G757" t="n">
+        <v>7</v>
+      </c>
+      <c r="H757" t="b">
+        <v>0</v>
+      </c>
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J757" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1010367357</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J753"/>
+  <autoFilter ref="A1:J757"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 6)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$792</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$795</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J792"/>
+  <dimension ref="A1:J795"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32802,8 +32802,131 @@
         </is>
       </c>
     </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>1191791021</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>earhcare</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>【乾燥肌・敏感肌の方に】アクシリオ 薬用メディフェクトゲル 1.5g×7包 敏感肌 乾燥肌 高保湿 ニキビ予防 肌荒れ対策 赤ちゃんOK オールインワン 保湿ゲル 医薬部外品　日本製　お試しセット</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>earthcare</t>
+        </is>
+      </c>
+      <c r="F793" t="n">
+        <v>1430</v>
+      </c>
+      <c r="G793" t="n">
+        <v>1</v>
+      </c>
+      <c r="H793" t="b">
+        <v>0</v>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J793" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191791021</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>1177887352</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>earhcare</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>【乾燥肌・敏感肌の方に】アクアテクトゲル250g オールインワン保湿ジェル/肌荒れ・乾燥でお困りの方に/小じわ改善/低刺激/化粧水・美容液・クリームいらず/アースケア公式/日本製</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>earthcare</t>
+        </is>
+      </c>
+      <c r="F794" t="n">
+        <v>8450</v>
+      </c>
+      <c r="G794" t="n">
+        <v>0</v>
+      </c>
+      <c r="H794" t="b">
+        <v>0</v>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177887352</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>1159590790</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>earhcare</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>【乾燥肌・敏感肌の方に】アクアテクトゲル100g オールインワン保湿ジェル/肌荒れ・乾燥でお困りの方に/小じわ改善/低刺激/化粧水・美容液・クリームいらず/earthcare公式/日本製</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>earthcare</t>
+        </is>
+      </c>
+      <c r="F795" t="n">
+        <v>4160</v>
+      </c>
+      <c r="G795" t="n">
+        <v>2</v>
+      </c>
+      <c r="H795" t="b">
+        <v>0</v>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J795" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159590790</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J792"/>
+  <autoFilter ref="A1:J795"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 7)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$809</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$810</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J809"/>
+  <dimension ref="A1:J810"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33499,8 +33499,49 @@
         </is>
       </c>
     </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>1015476194</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>TOUCHBeauty</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>電動洗顔ブラシ シリコン洗顔ブラシ 三色選べる ソニックフェイシャルクレンザー IPX6防水 振動バイブレーション 充電式TB-1788食品級シリコン製</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>タッチビューティ</t>
+        </is>
+      </c>
+      <c r="F810" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G810" t="n">
+        <v>0</v>
+      </c>
+      <c r="H810" t="b">
+        <v>0</v>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J810" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1015476194</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J809"/>
+  <autoFilter ref="A1:J810"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 13, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$810</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$811</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J810"/>
+  <dimension ref="A1:J811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33540,8 +33540,49 @@
         </is>
       </c>
     </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>1209681232</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>healgrids</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>ヒルグリーズ ナイアシンアミド 4% トーニング デオドラント</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>HEALGRIDS</t>
+        </is>
+      </c>
+      <c r="F811" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G811" t="n">
+        <v>0</v>
+      </c>
+      <c r="H811" t="b">
+        <v>0</v>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J811" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209681232</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J810"/>
+  <autoFilter ref="A1:J811"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 56, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$821</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$822</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J821"/>
+  <dimension ref="A1:J822"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33991,8 +33991,49 @@
         </is>
       </c>
     </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>1000094101</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Hachi88</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>plus alpha 3 bee さらさらUVスティック 14g 日本製 SPF50+/PA++++ スティックタイプ 日焼け止め 無香料 ノンパラペン</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>plus alpha 3</t>
+        </is>
+      </c>
+      <c r="F822" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G822" t="n">
+        <v>5</v>
+      </c>
+      <c r="H822" t="b">
+        <v>0</v>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J822" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1000094101</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J821"/>
+  <autoFilter ref="A1:J822"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 3 own-file progress (반복 23)
</commit_message>
<xml_diff>
--- a/output/discovery_result_3.xlsx
+++ b/output/discovery_result_3.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$827</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$828</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J827"/>
+  <dimension ref="A1:J828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34237,8 +34237,49 @@
         </is>
       </c>
     </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>1143096239</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>quadthera</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>3Dブースターマスクジェル230g</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>FORHERTZ</t>
+        </is>
+      </c>
+      <c r="F828" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G828" t="n">
+        <v>9</v>
+      </c>
+      <c r="H828" t="b">
+        <v>0</v>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J828" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143096239</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J827"/>
+  <autoFilter ref="A1:J828"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>